<commit_message>
Standardize all QA documentation and test cases
docs(qa): synchronize master test cases, daily checklists, templates, and bug reports with standard QA metadata
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\SIAP_UPLOAD_GITHUB\qa-testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\docs\qa-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE677915-9568-4233-94A1-B002FDCFF909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27161A07-7B65-45CC-8040-B9FD6F881852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="220" windowWidth="14400" windowHeight="7810" firstSheet="1" activeTab="1" xr2:uid="{D20540B9-5A4B-4C0F-A1AA-6997D01BA992}"/>
+    <workbookView xWindow="0" yWindow="220" windowWidth="14400" windowHeight="7810" firstSheet="2" activeTab="4" xr2:uid="{D20540B9-5A4B-4C0F-A1AA-6997D01BA992}"/>
   </bookViews>
   <sheets>
     <sheet name="MASTER_TC" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="830">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="830">
   <si>
     <t>TC ID</t>
   </si>
@@ -1644,9 +1644,6 @@
     <t>Domain email DEFAULT_AUTH salah (@taims.local bukan @taims_db.local) 401 fallback</t>
   </si>
   <si>
-    <t>Dika / Reza</t>
-  </si>
-  <si>
     <t>BUG-007</t>
   </si>
   <si>
@@ -2658,9 +2655,6 @@
     <t>Audit selesai, defect logged to BUG-018</t>
   </si>
   <si>
-    <t>Dika Yoga Pratama</t>
-  </si>
-  <si>
     <t>Fixed &amp; Verified (SLA 30 hari sinkron 99.1% Target Achieved, kartu AI real-time health 0.0% standby)</t>
   </si>
   <si>
@@ -2695,6 +2689,12 @@
   </si>
   <si>
     <t>screenshots/Hari-10/2026-10-21_Hari-10_final-dashboard_users-rbac.png</t>
+  </si>
+  <si>
+    <t>Status 200 OK. message: Heartbeat received, status: online, next_heartbeat_in: 30, Response Time 33 ms</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png</t>
   </si>
 </sst>
 </file>
@@ -2918,7 +2918,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3003,20 +3003,11 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -3034,13 +3025,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -3064,27 +3049,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -3948,7 +3934,7 @@
         <v>55</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>75</v>
@@ -3957,8 +3943,8 @@
         <v>93</v>
       </c>
       <c r="M12" s="7"/>
-      <c r="N12" s="53" t="s">
-        <v>755</v>
+      <c r="N12" s="48" t="s">
+        <v>754</v>
       </c>
       <c r="O12" s="14" t="s">
         <v>24</v>
@@ -4077,7 +4063,7 @@
         <v>228</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -4277,7 +4263,7 @@
         <v>417</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
@@ -4317,7 +4303,7 @@
         <v>231</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
@@ -4397,7 +4383,7 @@
         <v>233</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
@@ -4517,7 +4503,7 @@
         <v>236</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
@@ -4677,7 +4663,7 @@
         <v>240</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
@@ -4757,7 +4743,7 @@
         <v>242</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
@@ -4997,7 +4983,7 @@
         <v>223</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -5037,7 +5023,7 @@
         <v>247</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -5215,8 +5201,8 @@
       <c r="M43" s="4" t="s">
         <v>440</v>
       </c>
-      <c r="N43" s="50" t="s">
-        <v>595</v>
+      <c r="N43" s="45" t="s">
+        <v>594</v>
       </c>
       <c r="O43" s="4" t="s">
         <v>24</v>
@@ -5305,8 +5291,8 @@
       <c r="M45" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="N45" s="50" t="s">
-        <v>593</v>
+      <c r="N45" s="45" t="s">
+        <v>592</v>
       </c>
       <c r="O45" s="4" t="s">
         <v>24</v>
@@ -5353,8 +5339,8 @@
       <c r="M46" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="N46" s="50" t="s">
-        <v>596</v>
+      <c r="N46" s="45" t="s">
+        <v>595</v>
       </c>
       <c r="O46" s="4" t="s">
         <v>24</v>
@@ -5563,8 +5549,8 @@
       <c r="M51" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="N51" s="50" t="s">
-        <v>594</v>
+      <c r="N51" s="45" t="s">
+        <v>593</v>
       </c>
       <c r="O51" s="4" t="s">
         <v>24</v>
@@ -5885,11 +5871,17 @@
       <c r="I59" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4"/>
+      <c r="J59" s="4" t="s">
+        <v>828</v>
+      </c>
+      <c r="K59" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L59" s="4"/>
       <c r="M59" s="4"/>
-      <c r="N59" s="7"/>
+      <c r="N59" s="57" t="s">
+        <v>829</v>
+      </c>
       <c r="O59" s="4" t="s">
         <v>24</v>
       </c>
@@ -6391,16 +6383,16 @@
     </row>
     <row r="72" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B72" s="10">
         <v>8</v>
       </c>
       <c r="C72" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>534</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>535</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>20</v>
@@ -6409,24 +6401,24 @@
         <v>21</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>536</v>
       </c>
-      <c r="H72" s="6" t="s">
+      <c r="I72" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="I72" s="6" t="s">
+      <c r="J72" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="J72" s="6" t="s">
-        <v>539</v>
-      </c>
-      <c r="K72" s="39" t="s">
+      <c r="K72" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L72" s="10"/>
       <c r="M72" s="10"/>
-      <c r="N72" s="50" t="s">
-        <v>603</v>
+      <c r="N72" s="45" t="s">
+        <v>602</v>
       </c>
       <c r="O72" s="4" t="s">
         <v>24</v>
@@ -6436,21 +6428,21 @@
       </c>
       <c r="Q72" s="4"/>
       <c r="R72" s="6" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="73" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B73" s="10">
         <v>8</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>20</v>
@@ -6459,24 +6451,24 @@
         <v>47</v>
       </c>
       <c r="G73" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="H73" s="6" t="s">
         <v>543</v>
       </c>
-      <c r="H73" s="6" t="s">
+      <c r="I73" s="6" t="s">
         <v>544</v>
       </c>
-      <c r="I73" s="6" t="s">
+      <c r="J73" s="6" t="s">
         <v>545</v>
       </c>
-      <c r="J73" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="K73" s="39" t="s">
+      <c r="K73" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L73" s="10"/>
       <c r="M73" s="10"/>
-      <c r="N73" s="50" t="s">
-        <v>604</v>
+      <c r="N73" s="45" t="s">
+        <v>603</v>
       </c>
       <c r="O73" s="4" t="s">
         <v>24</v>
@@ -6486,21 +6478,21 @@
       </c>
       <c r="Q73" s="4"/>
       <c r="R73" s="6" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="74" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B74" s="10">
         <v>8</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>20</v>
@@ -6509,24 +6501,24 @@
         <v>47</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>550</v>
       </c>
-      <c r="H74" s="6" t="s">
+      <c r="I74" s="6" t="s">
         <v>551</v>
       </c>
-      <c r="I74" s="6" t="s">
+      <c r="J74" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="J74" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="K74" s="39" t="s">
+      <c r="K74" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L74" s="10"/>
       <c r="M74" s="10"/>
-      <c r="N74" s="50" t="s">
-        <v>605</v>
+      <c r="N74" s="45" t="s">
+        <v>604</v>
       </c>
       <c r="O74" s="4" t="s">
         <v>24</v>
@@ -6536,21 +6528,21 @@
       </c>
       <c r="Q74" s="4"/>
       <c r="R74" s="6" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="75" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B75" s="10">
         <v>8</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>46</v>
@@ -6559,24 +6551,24 @@
         <v>21</v>
       </c>
       <c r="G75" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="H75" s="6" t="s">
         <v>557</v>
       </c>
-      <c r="H75" s="6" t="s">
+      <c r="I75" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="I75" s="6" t="s">
+      <c r="J75" s="6" t="s">
         <v>559</v>
       </c>
-      <c r="J75" s="6" t="s">
-        <v>560</v>
-      </c>
-      <c r="K75" s="39" t="s">
+      <c r="K75" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L75" s="10"/>
       <c r="M75" s="10"/>
-      <c r="N75" s="50" t="s">
-        <v>606</v>
+      <c r="N75" s="45" t="s">
+        <v>605</v>
       </c>
       <c r="O75" s="4" t="s">
         <v>24</v>
@@ -6586,21 +6578,21 @@
       </c>
       <c r="Q75" s="4"/>
       <c r="R75" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="76" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B76" s="10">
         <v>8</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>20</v>
@@ -6609,28 +6601,28 @@
         <v>47</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>564</v>
       </c>
-      <c r="H76" s="6" t="s">
+      <c r="I76" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="I76" s="6" t="s">
+      <c r="J76" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="J76" s="6" t="s">
-        <v>567</v>
-      </c>
-      <c r="K76" s="39" t="s">
+      <c r="K76" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L76" s="10" t="s">
         <v>420</v>
       </c>
       <c r="M76" s="10" t="s">
-        <v>491</v>
-      </c>
-      <c r="N76" s="50" t="s">
-        <v>601</v>
+        <v>490</v>
+      </c>
+      <c r="N76" s="45" t="s">
+        <v>600</v>
       </c>
       <c r="O76" s="4" t="s">
         <v>24</v>
@@ -6640,21 +6632,21 @@
       </c>
       <c r="Q76" s="4"/>
       <c r="R76" s="6" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="77" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B77" s="10">
         <v>8</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E77" s="4" t="s">
         <v>20</v>
@@ -6663,28 +6655,28 @@
         <v>21</v>
       </c>
       <c r="G77" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="H77" s="6" t="s">
         <v>571</v>
       </c>
-      <c r="H77" s="6" t="s">
+      <c r="I77" s="6" t="s">
         <v>572</v>
       </c>
-      <c r="I77" s="6" t="s">
+      <c r="J77" s="6" t="s">
         <v>573</v>
       </c>
-      <c r="J77" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="K77" s="39" t="s">
+      <c r="K77" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L77" s="10" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="M77" s="10" t="s">
-        <v>493</v>
-      </c>
-      <c r="N77" s="50" t="s">
-        <v>602</v>
+        <v>492</v>
+      </c>
+      <c r="N77" s="45" t="s">
+        <v>601</v>
       </c>
       <c r="O77" s="4" t="s">
         <v>24</v>
@@ -6694,21 +6686,21 @@
       </c>
       <c r="Q77" s="4"/>
       <c r="R77" s="6" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="78" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B78" s="10">
         <v>8</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>20</v>
@@ -6717,24 +6709,24 @@
         <v>47</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>578</v>
       </c>
-      <c r="H78" s="6" t="s">
+      <c r="I78" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="I78" s="6" t="s">
+      <c r="J78" s="6" t="s">
         <v>580</v>
       </c>
-      <c r="J78" s="6" t="s">
-        <v>581</v>
-      </c>
-      <c r="K78" s="39" t="s">
+      <c r="K78" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L78" s="10"/>
       <c r="M78" s="10"/>
-      <c r="N78" s="50" t="s">
-        <v>607</v>
+      <c r="N78" s="45" t="s">
+        <v>606</v>
       </c>
       <c r="O78" s="4" t="s">
         <v>24</v>
@@ -6744,47 +6736,47 @@
       </c>
       <c r="Q78" s="4"/>
       <c r="R78" s="6" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="79" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B79" s="6">
         <v>9</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D79" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="E79" s="6" t="s">
         <v>628</v>
-      </c>
-      <c r="E79" s="6" t="s">
-        <v>629</v>
       </c>
       <c r="F79" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G79" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="H79" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="H79" s="6" t="s">
+      <c r="I79" s="6" t="s">
         <v>631</v>
       </c>
-      <c r="I79" s="6" t="s">
+      <c r="J79" s="6" t="s">
         <v>632</v>
       </c>
-      <c r="J79" s="6" t="s">
-        <v>633</v>
-      </c>
-      <c r="K79" s="51" t="s">
+      <c r="K79" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L79" s="8"/>
       <c r="M79" s="8"/>
-      <c r="N79" s="52" t="s">
-        <v>634</v>
+      <c r="N79" s="47" t="s">
+        <v>633</v>
       </c>
       <c r="O79" s="6" t="s">
         <v>24</v>
@@ -6793,50 +6785,50 @@
         <v>104</v>
       </c>
       <c r="Q79" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="R79" s="6" t="s">
         <v>635</v>
-      </c>
-      <c r="R79" s="6" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="80" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B80" s="6">
         <v>9</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D80" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="E80" s="6" t="s">
         <v>638</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>639</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>640</v>
       </c>
-      <c r="H80" s="6" t="s">
+      <c r="I80" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="I80" s="6" t="s">
+      <c r="J80" s="6" t="s">
         <v>642</v>
       </c>
-      <c r="J80" s="6" t="s">
-        <v>643</v>
-      </c>
-      <c r="K80" s="51" t="s">
+      <c r="K80" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L80" s="8"/>
       <c r="M80" s="8"/>
-      <c r="N80" s="52" t="s">
-        <v>644</v>
+      <c r="N80" s="47" t="s">
+        <v>643</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>24</v>
@@ -6845,50 +6837,50 @@
         <v>104</v>
       </c>
       <c r="Q80" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R80" s="6" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="81" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B81" s="6">
         <v>9</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F81" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G81" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="H81" s="6" t="s">
         <v>648</v>
       </c>
-      <c r="H81" s="6" t="s">
+      <c r="I81" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="I81" s="6" t="s">
+      <c r="J81" s="6" t="s">
         <v>650</v>
       </c>
-      <c r="J81" s="6" t="s">
-        <v>651</v>
-      </c>
-      <c r="K81" s="51" t="s">
+      <c r="K81" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L81" s="8"/>
       <c r="M81" s="8"/>
-      <c r="N81" s="52" t="s">
-        <v>652</v>
+      <c r="N81" s="47" t="s">
+        <v>651</v>
       </c>
       <c r="O81" s="6" t="s">
         <v>24</v>
@@ -6897,50 +6889,50 @@
         <v>104</v>
       </c>
       <c r="Q81" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R81" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="82" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A82" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B82" s="6">
         <v>9</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D82" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="E82" s="6" t="s">
         <v>655</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>656</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="H82" s="6" t="s">
+      <c r="I82" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="I82" s="6" t="s">
+      <c r="J82" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="J82" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="K82" s="51" t="s">
+      <c r="K82" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L82" s="8"/>
       <c r="M82" s="8"/>
-      <c r="N82" s="52" t="s">
-        <v>661</v>
+      <c r="N82" s="47" t="s">
+        <v>660</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>24</v>
@@ -6949,50 +6941,50 @@
         <v>104</v>
       </c>
       <c r="Q82" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R82" s="6" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="6" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B83" s="6">
         <v>9</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F83" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G83" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="H83" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="H83" s="6" t="s">
+      <c r="I83" s="6" t="s">
         <v>666</v>
       </c>
-      <c r="I83" s="6" t="s">
+      <c r="J83" s="6" t="s">
         <v>667</v>
       </c>
-      <c r="J83" s="6" t="s">
-        <v>668</v>
-      </c>
-      <c r="K83" s="51" t="s">
+      <c r="K83" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L83" s="8"/>
       <c r="M83" s="8"/>
-      <c r="N83" s="52" t="s">
-        <v>669</v>
+      <c r="N83" s="47" t="s">
+        <v>668</v>
       </c>
       <c r="O83" s="6" t="s">
         <v>24</v>
@@ -7001,50 +6993,50 @@
         <v>104</v>
       </c>
       <c r="Q83" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R83" s="6" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A84" s="6" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B84" s="6">
         <v>9</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D84" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="E84" s="6" t="s">
         <v>672</v>
-      </c>
-      <c r="E84" s="6" t="s">
-        <v>673</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G84" s="6" t="s">
+        <v>673</v>
+      </c>
+      <c r="H84" s="6" t="s">
         <v>674</v>
       </c>
-      <c r="H84" s="6" t="s">
+      <c r="I84" s="6" t="s">
         <v>675</v>
       </c>
-      <c r="I84" s="6" t="s">
+      <c r="J84" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="J84" s="6" t="s">
-        <v>677</v>
-      </c>
-      <c r="K84" s="51" t="s">
+      <c r="K84" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L84" s="8"/>
       <c r="M84" s="8"/>
-      <c r="N84" s="52" t="s">
-        <v>678</v>
+      <c r="N84" s="47" t="s">
+        <v>677</v>
       </c>
       <c r="O84" s="6" t="s">
         <v>24</v>
@@ -7053,50 +7045,50 @@
         <v>104</v>
       </c>
       <c r="Q84" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R84" s="6" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="85" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" s="6" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B85" s="6">
         <v>9</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D85" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="E85" s="6" t="s">
         <v>681</v>
-      </c>
-      <c r="E85" s="6" t="s">
-        <v>682</v>
       </c>
       <c r="F85" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G85" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="H85" s="6" t="s">
         <v>683</v>
       </c>
-      <c r="H85" s="6" t="s">
+      <c r="I85" s="6" t="s">
         <v>684</v>
       </c>
-      <c r="I85" s="6" t="s">
+      <c r="J85" s="6" t="s">
         <v>685</v>
       </c>
-      <c r="J85" s="6" t="s">
-        <v>686</v>
-      </c>
-      <c r="K85" s="51" t="s">
+      <c r="K85" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L85" s="8"/>
       <c r="M85" s="8"/>
-      <c r="N85" s="52" t="s">
-        <v>687</v>
+      <c r="N85" s="47" t="s">
+        <v>686</v>
       </c>
       <c r="O85" s="6" t="s">
         <v>24</v>
@@ -7105,50 +7097,50 @@
         <v>104</v>
       </c>
       <c r="Q85" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R85" s="6" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="86" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" s="6" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B86" s="6">
         <v>9</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G86" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="H86" s="6" t="s">
+      <c r="I86" s="6" t="s">
         <v>692</v>
       </c>
-      <c r="I86" s="6" t="s">
+      <c r="J86" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="J86" s="6" t="s">
-        <v>694</v>
-      </c>
-      <c r="K86" s="51" t="s">
+      <c r="K86" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L86" s="8"/>
       <c r="M86" s="8"/>
-      <c r="N86" s="52" t="s">
-        <v>695</v>
+      <c r="N86" s="47" t="s">
+        <v>694</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>24</v>
@@ -7157,15 +7149,15 @@
         <v>104</v>
       </c>
       <c r="Q86" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="R86" s="6" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="87" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B87" s="6">
         <v>10</v>
@@ -7174,7 +7166,7 @@
         <v>35</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>20</v>
@@ -7183,24 +7175,24 @@
         <v>21</v>
       </c>
       <c r="G87" s="6" t="s">
+        <v>757</v>
+      </c>
+      <c r="H87" s="6" t="s">
         <v>758</v>
       </c>
-      <c r="H87" s="6" t="s">
+      <c r="I87" s="6" t="s">
         <v>759</v>
       </c>
-      <c r="I87" s="6" t="s">
+      <c r="J87" s="6" t="s">
         <v>760</v>
       </c>
-      <c r="J87" s="6" t="s">
-        <v>761</v>
-      </c>
-      <c r="K87" s="51" t="s">
+      <c r="K87" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L87" s="8"/>
       <c r="M87" s="8"/>
-      <c r="N87" s="52" t="s">
-        <v>755</v>
+      <c r="N87" s="47" t="s">
+        <v>754</v>
       </c>
       <c r="O87" s="6" t="s">
         <v>24</v>
@@ -7209,15 +7201,15 @@
         <v>107</v>
       </c>
       <c r="Q87" s="6" t="s">
+        <v>761</v>
+      </c>
+      <c r="R87" s="6" t="s">
         <v>762</v>
-      </c>
-      <c r="R87" s="6" t="s">
-        <v>763</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A88" s="6" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B88" s="6">
         <v>10</v>
@@ -7226,7 +7218,7 @@
         <v>35</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>20</v>
@@ -7235,24 +7227,24 @@
         <v>21</v>
       </c>
       <c r="G88" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="H88" s="6" t="s">
         <v>766</v>
       </c>
-      <c r="H88" s="6" t="s">
+      <c r="I88" s="6" t="s">
         <v>767</v>
       </c>
-      <c r="I88" s="6" t="s">
+      <c r="J88" s="6" t="s">
         <v>768</v>
       </c>
-      <c r="J88" s="6" t="s">
-        <v>769</v>
-      </c>
-      <c r="K88" s="51" t="s">
+      <c r="K88" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L88" s="8"/>
       <c r="M88" s="8"/>
-      <c r="N88" s="52" t="s">
-        <v>770</v>
+      <c r="N88" s="47" t="s">
+        <v>769</v>
       </c>
       <c r="O88" s="6" t="s">
         <v>24</v>
@@ -7261,15 +7253,15 @@
         <v>107</v>
       </c>
       <c r="Q88" s="6" t="s">
+        <v>761</v>
+      </c>
+      <c r="R88" s="6" t="s">
         <v>762</v>
-      </c>
-      <c r="R88" s="6" t="s">
-        <v>763</v>
       </c>
     </row>
     <row r="89" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B89" s="6">
         <v>10</v>
@@ -7278,7 +7270,7 @@
         <v>35</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>20</v>
@@ -7287,24 +7279,24 @@
         <v>21</v>
       </c>
       <c r="G89" s="6" t="s">
+        <v>772</v>
+      </c>
+      <c r="H89" s="6" t="s">
         <v>773</v>
       </c>
-      <c r="H89" s="6" t="s">
+      <c r="I89" s="6" t="s">
         <v>774</v>
       </c>
-      <c r="I89" s="6" t="s">
+      <c r="J89" s="6" t="s">
         <v>775</v>
       </c>
-      <c r="J89" s="6" t="s">
-        <v>776</v>
-      </c>
-      <c r="K89" s="51" t="s">
+      <c r="K89" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L89" s="8"/>
       <c r="M89" s="8"/>
-      <c r="N89" s="52" t="s">
-        <v>713</v>
+      <c r="N89" s="47" t="s">
+        <v>712</v>
       </c>
       <c r="O89" s="6" t="s">
         <v>24</v>
@@ -7313,50 +7305,50 @@
         <v>107</v>
       </c>
       <c r="Q89" s="6" t="s">
+        <v>761</v>
+      </c>
+      <c r="R89" s="6" t="s">
         <v>762</v>
-      </c>
-      <c r="R89" s="6" t="s">
-        <v>763</v>
       </c>
     </row>
     <row r="90" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A90" s="6" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B90" s="6">
         <v>10</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D90" s="6" t="s">
+        <v>777</v>
+      </c>
+      <c r="E90" s="6" t="s">
         <v>778</v>
-      </c>
-      <c r="E90" s="6" t="s">
-        <v>779</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G90" s="6" t="s">
+        <v>779</v>
+      </c>
+      <c r="H90" s="6" t="s">
         <v>780</v>
       </c>
-      <c r="H90" s="6" t="s">
+      <c r="I90" s="6" t="s">
         <v>781</v>
       </c>
-      <c r="I90" s="6" t="s">
+      <c r="J90" s="6" t="s">
         <v>782</v>
       </c>
-      <c r="J90" s="6" t="s">
-        <v>783</v>
-      </c>
-      <c r="K90" s="51" t="s">
+      <c r="K90" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L90" s="8"/>
       <c r="M90" s="8"/>
-      <c r="N90" s="52" t="s">
-        <v>705</v>
+      <c r="N90" s="47" t="s">
+        <v>704</v>
       </c>
       <c r="O90" s="6" t="s">
         <v>24</v>
@@ -7365,50 +7357,50 @@
         <v>107</v>
       </c>
       <c r="Q90" s="6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R90" s="6" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="91" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A91" s="6" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B91" s="6">
         <v>10</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D91" s="6" t="s">
+        <v>785</v>
+      </c>
+      <c r="E91" s="6" t="s">
         <v>786</v>
-      </c>
-      <c r="E91" s="6" t="s">
-        <v>787</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G91" s="6" t="s">
+        <v>787</v>
+      </c>
+      <c r="H91" s="6" t="s">
         <v>788</v>
       </c>
-      <c r="H91" s="6" t="s">
+      <c r="I91" s="6" t="s">
         <v>789</v>
       </c>
-      <c r="I91" s="6" t="s">
+      <c r="J91" s="6" t="s">
         <v>790</v>
       </c>
-      <c r="J91" s="6" t="s">
-        <v>791</v>
-      </c>
-      <c r="K91" s="51" t="s">
+      <c r="K91" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L91" s="8"/>
       <c r="M91" s="8"/>
-      <c r="N91" s="52" t="s">
-        <v>713</v>
+      <c r="N91" s="47" t="s">
+        <v>712</v>
       </c>
       <c r="O91" s="6" t="s">
         <v>24</v>
@@ -7417,50 +7409,50 @@
         <v>107</v>
       </c>
       <c r="Q91" s="6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R91" s="6" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="92" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A92" s="6" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B92" s="6">
         <v>10</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D92" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="E92" s="6" t="s">
         <v>794</v>
-      </c>
-      <c r="E92" s="6" t="s">
-        <v>795</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G92" s="6" t="s">
+        <v>795</v>
+      </c>
+      <c r="H92" s="6" t="s">
         <v>796</v>
       </c>
-      <c r="H92" s="6" t="s">
+      <c r="I92" s="6" t="s">
         <v>797</v>
       </c>
-      <c r="I92" s="6" t="s">
+      <c r="J92" s="6" t="s">
         <v>798</v>
       </c>
-      <c r="J92" s="6" t="s">
-        <v>799</v>
-      </c>
-      <c r="K92" s="51" t="s">
+      <c r="K92" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L92" s="8"/>
       <c r="M92" s="8"/>
-      <c r="N92" s="52" t="s">
-        <v>720</v>
+      <c r="N92" s="47" t="s">
+        <v>719</v>
       </c>
       <c r="O92" s="6" t="s">
         <v>24</v>
@@ -7469,50 +7461,50 @@
         <v>107</v>
       </c>
       <c r="Q92" s="6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R92" s="6" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="93" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="6" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B93" s="6">
         <v>10</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D93" s="6" t="s">
+        <v>801</v>
+      </c>
+      <c r="E93" s="6" t="s">
         <v>802</v>
       </c>
-      <c r="E93" s="6" t="s">
+      <c r="F93" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="G93" s="6" t="s">
         <v>803</v>
       </c>
-      <c r="F93" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="G93" s="6" t="s">
+      <c r="H93" s="6" t="s">
         <v>804</v>
       </c>
-      <c r="H93" s="6" t="s">
+      <c r="I93" s="6" t="s">
         <v>805</v>
       </c>
-      <c r="I93" s="6" t="s">
+      <c r="J93" s="6" t="s">
         <v>806</v>
       </c>
-      <c r="J93" s="6" t="s">
-        <v>807</v>
-      </c>
-      <c r="K93" s="51" t="s">
+      <c r="K93" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L93" s="8"/>
       <c r="M93" s="8"/>
-      <c r="N93" s="52" t="s">
-        <v>705</v>
+      <c r="N93" s="47" t="s">
+        <v>704</v>
       </c>
       <c r="O93" s="6" t="s">
         <v>24</v>
@@ -7521,50 +7513,50 @@
         <v>107</v>
       </c>
       <c r="Q93" s="6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R93" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="94" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A94" s="6" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B94" s="6">
         <v>10</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D94" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="E94" s="6" t="s">
         <v>810</v>
       </c>
-      <c r="E94" s="6" t="s">
+      <c r="F94" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="G94" s="6" t="s">
         <v>811</v>
       </c>
-      <c r="F94" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="G94" s="6" t="s">
+      <c r="H94" s="6" t="s">
         <v>812</v>
       </c>
-      <c r="H94" s="6" t="s">
+      <c r="I94" s="6" t="s">
         <v>813</v>
       </c>
-      <c r="I94" s="6" t="s">
+      <c r="J94" s="6" t="s">
         <v>814</v>
       </c>
-      <c r="J94" s="6" t="s">
-        <v>815</v>
-      </c>
-      <c r="K94" s="51" t="s">
+      <c r="K94" s="46" t="s">
         <v>75</v>
       </c>
       <c r="L94" s="8"/>
       <c r="M94" s="8"/>
-      <c r="N94" s="52" t="s">
-        <v>752</v>
+      <c r="N94" s="47" t="s">
+        <v>751</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>24</v>
@@ -7573,10 +7565,10 @@
         <v>107</v>
       </c>
       <c r="Q94" s="6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R94" s="6" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
   </sheetData>
@@ -7610,9 +7602,10 @@
     <hyperlink ref="N92" r:id="rId26" tooltip="2026-10-21_Hari-10_final-dashboard_desktop-1080p.png" xr:uid="{DF0874B5-F3A5-4940-B56E-5C8C97D816B7}"/>
     <hyperlink ref="N93" r:id="rId27" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{B17C34F4-F7BE-42EA-851C-9107F4B20CCB}"/>
     <hyperlink ref="N94" r:id="rId28" tooltip="2026-10-21_Hari-10_final-dashboard_users-rbac.png" xr:uid="{2241DBCB-8785-46FF-94D5-F6C6DED84A05}"/>
+    <hyperlink ref="N59" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png" xr:uid="{014D7D64-B7C6-4162-9E46-25E1D648DA6D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId29"/>
+  <pageSetup orientation="portrait" r:id="rId30"/>
 </worksheet>
 </file>
 
@@ -7660,7 +7653,7 @@
         <v>427</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -7685,14 +7678,14 @@
       <c r="F2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="38" t="s">
+      <c r="G2" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H2" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="I2" s="33" t="s">
-        <v>593</v>
+      <c r="I2" s="32" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
@@ -7714,14 +7707,14 @@
       <c r="F3" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="38" t="s">
+      <c r="G3" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H3" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="I3" s="33" t="s">
-        <v>594</v>
+      <c r="I3" s="32" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
@@ -7732,7 +7725,7 @@
         <v>93</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>260</v>
@@ -7743,14 +7736,14 @@
       <c r="F4" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="38" t="s">
+      <c r="G4" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="I4" s="33" t="s">
-        <v>595</v>
+      <c r="I4" s="32" t="s">
+        <v>594</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
@@ -7761,7 +7754,7 @@
         <v>96</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>282</v>
@@ -7772,14 +7765,14 @@
       <c r="F5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="38" t="s">
+      <c r="G5" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="I5" s="33" t="s">
-        <v>596</v>
+      <c r="I5" s="32" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -7801,14 +7794,14 @@
       <c r="F6" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="G6" s="38" t="s">
+      <c r="G6" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="I6" s="33" t="s">
-        <v>608</v>
+      <c r="I6" s="32" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="29" x14ac:dyDescent="0.35">
@@ -7828,27 +7821,27 @@
         <v>70</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="G7" s="38" t="s">
+        <v>614</v>
+      </c>
+      <c r="G7" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="I7" s="33" t="s">
-        <v>597</v>
+      <c r="I7" s="32" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>491</v>
-      </c>
-      <c r="B8" s="37" t="s">
+        <v>490</v>
+      </c>
+      <c r="B8" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>483</v>
@@ -7857,27 +7850,27 @@
         <v>420</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="G8" s="38" t="s">
+        <v>614</v>
+      </c>
+      <c r="G8" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="I8" s="33" t="s">
-        <v>598</v>
+      <c r="I8" s="32" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="B9" s="37" t="s">
+        <v>491</v>
+      </c>
+      <c r="B9" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>483</v>
@@ -7886,158 +7879,158 @@
         <v>420</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="G9" s="38" t="s">
+        <v>614</v>
+      </c>
+      <c r="G9" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="I9" s="33" t="s">
-        <v>598</v>
+      <c r="I9" s="32" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>483</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="G10" s="38" t="s">
+        <v>614</v>
+      </c>
+      <c r="G10" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="I10" s="33" t="s">
-        <v>599</v>
+      <c r="I10" s="32" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>483</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="G11" s="38" t="s">
+        <v>614</v>
+      </c>
+      <c r="G11" s="35" t="s">
         <v>438</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="I11" s="33" t="s">
-        <v>598</v>
+      <c r="I11" s="32" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="M12" s="54"/>
-      <c r="N12" s="54"/>
+      <c r="M12" s="49"/>
+      <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="58" t="s">
+      <c r="A13" s="56" t="s">
+        <v>588</v>
+      </c>
+      <c r="B13" s="56"/>
+      <c r="C13" s="56"/>
+      <c r="M13" s="49"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" s="56" t="s">
         <v>589</v>
       </c>
-      <c r="B13" s="58"/>
-      <c r="C13" s="58"/>
-      <c r="M13" s="54"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="58" t="s">
-        <v>590</v>
-      </c>
-      <c r="B14" s="58"/>
-      <c r="C14" s="58"/>
-      <c r="M14" s="54"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="M15" s="54"/>
+      <c r="M15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="M16" s="54"/>
+      <c r="M16" s="49"/>
     </row>
     <row r="17" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M17" s="54"/>
+      <c r="M17" s="49"/>
     </row>
     <row r="18" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M18" s="54"/>
+      <c r="M18" s="49"/>
     </row>
     <row r="19" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M19" s="54"/>
+      <c r="M19" s="49"/>
     </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N79" s="40"/>
+      <c r="N79" s="37"/>
     </row>
     <row r="80" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N80" s="40"/>
+      <c r="N80" s="37"/>
     </row>
     <row r="81" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N81" s="40"/>
+      <c r="N81" s="37"/>
     </row>
     <row r="82" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N82" s="40"/>
+      <c r="N82" s="37"/>
     </row>
     <row r="83" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N83" s="40"/>
+      <c r="N83" s="37"/>
     </row>
     <row r="84" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N84" s="40"/>
+      <c r="N84" s="37"/>
     </row>
     <row r="85" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N85" s="40"/>
+      <c r="N85" s="37"/>
     </row>
     <row r="86" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N86" s="40"/>
+      <c r="N86" s="37"/>
     </row>
     <row r="87" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N87" s="40"/>
+      <c r="N87" s="37"/>
     </row>
     <row r="88" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N88" s="40"/>
+      <c r="N88" s="37"/>
     </row>
     <row r="89" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N89" s="40"/>
+      <c r="N89" s="37"/>
     </row>
     <row r="90" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N90" s="40"/>
+      <c r="N90" s="37"/>
     </row>
     <row r="91" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N91" s="40"/>
+      <c r="N91" s="37"/>
     </row>
     <row r="92" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N92" s="40"/>
+      <c r="N92" s="37"/>
     </row>
     <row r="93" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N93" s="40"/>
+      <c r="N93" s="37"/>
     </row>
     <row r="94" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N94" s="40"/>
+      <c r="N94" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -8124,7 +8117,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="N1" s="22" t="s">
         <v>62</v>
@@ -8149,28 +8142,28 @@
       </c>
     </row>
     <row r="2" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="13" t="s">
         <v>67</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="32" t="s">
+      <c r="C2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I2" s="10"/>
@@ -8183,10 +8176,10 @@
       <c r="L2" s="6">
         <v>404</v>
       </c>
-      <c r="M2" s="35" t="s">
-        <v>593</v>
-      </c>
-      <c r="N2" s="34" t="s">
+      <c r="M2" s="51" t="s">
+        <v>592</v>
+      </c>
+      <c r="N2" s="33" t="s">
         <v>469</v>
       </c>
       <c r="O2" s="4" t="s">
@@ -8210,28 +8203,28 @@
       <c r="W2" s="2"/>
     </row>
     <row r="3" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="13" t="s">
         <v>69</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="32" t="s">
+      <c r="C3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I3" s="10"/>
@@ -8244,10 +8237,10 @@
       <c r="L3" s="6">
         <v>500</v>
       </c>
-      <c r="M3" s="35" t="s">
-        <v>594</v>
-      </c>
-      <c r="N3" s="34" t="s">
+      <c r="M3" s="51" t="s">
+        <v>593</v>
+      </c>
+      <c r="N3" s="33" t="s">
         <v>470</v>
       </c>
       <c r="O3" s="4" t="s">
@@ -8271,28 +8264,28 @@
       <c r="W3" s="2"/>
     </row>
     <row r="4" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="13" t="s">
         <v>440</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="10" t="s">
+      <c r="C4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I4" s="10"/>
@@ -8305,8 +8298,8 @@
       <c r="L4" s="6">
         <v>500</v>
       </c>
-      <c r="M4" s="35" t="s">
-        <v>595</v>
+      <c r="M4" s="51" t="s">
+        <v>594</v>
       </c>
       <c r="N4" s="23" t="s">
         <v>455</v>
@@ -8331,28 +8324,28 @@
       </c>
     </row>
     <row r="5" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="13" t="s">
         <v>459</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="10" t="s">
+      <c r="C5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I5" s="10"/>
@@ -8365,8 +8358,8 @@
       <c r="L5" s="6">
         <v>500</v>
       </c>
-      <c r="M5" s="35" t="s">
-        <v>596</v>
+      <c r="M5" s="51" t="s">
+        <v>595</v>
       </c>
       <c r="N5" s="23" t="s">
         <v>465</v>
@@ -8386,913 +8379,913 @@
       <c r="S5" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="T5" s="8" t="s">
+      <c r="T5" s="6" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="13" t="s">
         <v>481</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="10" t="s">
+      <c r="C6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>498</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="L6" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="M6" s="52" t="s">
+        <v>607</v>
+      </c>
+      <c r="N6" s="4" t="s">
         <v>500</v>
       </c>
-      <c r="M6" s="36" t="s">
+      <c r="O6" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S6" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T6" s="6" t="s">
         <v>608</v>
       </c>
-      <c r="N6" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="O6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="P6" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="S6" s="7" t="s">
+      <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="T6" s="8" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
-        <v>488</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>503</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>504</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>505</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="M7" s="35" t="s">
-        <v>597</v>
-      </c>
-      <c r="N7" s="7" t="s">
+      <c r="M7" s="51" t="s">
+        <v>596</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="O7" s="4" t="s">
         <v>506</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="P7" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S7" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>490</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>507</v>
       </c>
-      <c r="P7" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q7" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="S7" s="7" t="s">
+      <c r="C8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="T7" s="8" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
-        <v>491</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>508</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>509</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="L8" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="M8" s="51" t="s">
+        <v>597</v>
+      </c>
+      <c r="N8" s="4" t="s">
         <v>511</v>
       </c>
-      <c r="M8" s="35" t="s">
-        <v>598</v>
-      </c>
-      <c r="N8" s="7" t="s">
+      <c r="O8" s="4" t="s">
         <v>512</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="P8" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S8" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>491</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="P8" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q8" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="R8" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="S8" s="7" t="s">
+      <c r="C9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="T8" s="8" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
-        <v>492</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="L9" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="M9" s="51" t="s">
+        <v>597</v>
+      </c>
+      <c r="N9" s="4" t="s">
         <v>517</v>
       </c>
-      <c r="M9" s="35" t="s">
-        <v>598</v>
-      </c>
-      <c r="N9" s="7" t="s">
+      <c r="O9" s="4" t="s">
         <v>518</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="P9" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S9" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>492</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>519</v>
       </c>
-      <c r="P9" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q9" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="R9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="S9" s="7" t="s">
+      <c r="C10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="T9" s="8" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
-        <v>493</v>
-      </c>
-      <c r="B10" s="6" t="s">
+      <c r="E10" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>520</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>483</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>521</v>
-      </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="4" t="s">
         <v>431</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="K10" s="6" t="s">
         <v>522</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="L10" s="6" t="s">
         <v>523</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="M10" s="51" t="s">
+        <v>598</v>
+      </c>
+      <c r="N10" s="4" t="s">
         <v>524</v>
       </c>
-      <c r="M10" s="35" t="s">
-        <v>599</v>
-      </c>
-      <c r="N10" s="7" t="s">
+      <c r="O10" s="4" t="s">
         <v>525</v>
       </c>
-      <c r="O10" s="7" t="s">
+      <c r="P10" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S10" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T10" s="6" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="42" t="s">
+        <v>495</v>
+      </c>
+      <c r="B11" s="39" t="s">
         <v>526</v>
       </c>
-      <c r="P10" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q10" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="R10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="S10" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="T10" s="8" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="41" t="s">
-        <v>496</v>
-      </c>
-      <c r="B11" s="42" t="s">
-        <v>527</v>
-      </c>
-      <c r="C11" s="41" t="s">
+      <c r="C11" s="43" t="s">
         <v>24</v>
       </c>
       <c r="D11" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="E11" s="41" t="s">
+      <c r="E11" s="43" t="s">
         <v>483</v>
       </c>
-      <c r="F11" s="41" t="s">
-        <v>495</v>
-      </c>
-      <c r="G11" s="41" t="s">
-        <v>521</v>
-      </c>
-      <c r="H11" s="41" t="s">
+      <c r="F11" s="43" t="s">
+        <v>494</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>520</v>
+      </c>
+      <c r="H11" s="43" t="s">
         <v>431</v>
       </c>
-      <c r="I11" s="41"/>
-      <c r="J11" s="42" t="s">
+      <c r="I11" s="38"/>
+      <c r="J11" s="39" t="s">
+        <v>527</v>
+      </c>
+      <c r="K11" s="39" t="s">
         <v>528</v>
       </c>
-      <c r="K11" s="42" t="s">
+      <c r="L11" s="39" t="s">
         <v>529</v>
       </c>
-      <c r="L11" s="42" t="s">
+      <c r="M11" s="51" t="s">
+        <v>597</v>
+      </c>
+      <c r="N11" s="43" t="s">
         <v>530</v>
       </c>
-      <c r="M11" s="43" t="s">
-        <v>598</v>
-      </c>
-      <c r="N11" s="44" t="s">
+      <c r="O11" s="43" t="s">
         <v>531</v>
       </c>
-      <c r="O11" s="44" t="s">
-        <v>532</v>
-      </c>
-      <c r="P11" s="44" t="s">
+      <c r="P11" s="43" t="s">
         <v>438</v>
       </c>
-      <c r="Q11" s="44" t="s">
-        <v>490</v>
-      </c>
-      <c r="R11" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="S11" s="44" t="s">
+      <c r="Q11" s="43" t="s">
+        <v>614</v>
+      </c>
+      <c r="R11" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="S11" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="T11" s="45" t="s">
+      <c r="T11" s="39" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="50" t="s">
+        <v>696</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>697</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>701</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>702</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>703</v>
+      </c>
+      <c r="M12" s="48" t="s">
+        <v>704</v>
+      </c>
+      <c r="N12" s="53" t="s">
+        <v>705</v>
+      </c>
+      <c r="O12" s="55" t="s">
+        <v>824</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q12" s="4" t="s">
         <v>614</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="11" t="s">
-        <v>697</v>
-      </c>
-      <c r="B12" s="11" t="s">
+      <c r="R12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S12" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="T12" s="6" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="50" t="s">
+        <v>706</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>709</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>710</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>711</v>
+      </c>
+      <c r="M13" s="48" t="s">
+        <v>712</v>
+      </c>
+      <c r="N13" s="54" t="s">
+        <v>713</v>
+      </c>
+      <c r="O13" s="55" t="s">
+        <v>825</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S13" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="T13" s="6" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="50" t="s">
+        <v>714</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>716</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>717</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>718</v>
+      </c>
+      <c r="M14" s="48" t="s">
+        <v>719</v>
+      </c>
+      <c r="N14" s="54" t="s">
+        <v>720</v>
+      </c>
+      <c r="O14" s="55" t="s">
+        <v>826</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S14" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="T14" s="6" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="50" t="s">
+        <v>721</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>722</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>723</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>724</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>725</v>
+      </c>
+      <c r="M15" s="48" t="s">
+        <v>719</v>
+      </c>
+      <c r="N15" s="54" t="s">
+        <v>726</v>
+      </c>
+      <c r="O15" s="55" t="s">
+        <v>826</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S15" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="50" t="s">
+        <v>727</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>728</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>730</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>731</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="M16" s="48" t="s">
+        <v>719</v>
+      </c>
+      <c r="N16" s="54" t="s">
+        <v>733</v>
+      </c>
+      <c r="O16" s="55" t="s">
+        <v>826</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S16" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="T16" s="6" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="50" t="s">
+        <v>734</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>735</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>736</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>737</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="M17" s="48" t="s">
+        <v>719</v>
+      </c>
+      <c r="N17" s="54" t="s">
+        <v>739</v>
+      </c>
+      <c r="O17" s="55" t="s">
+        <v>826</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S17" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="T17" s="6" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="50" t="s">
+        <v>740</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>741</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>698</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="11" t="s">
+      <c r="F18" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>742</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>743</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>744</v>
+      </c>
+      <c r="M18" s="48" t="s">
+        <v>704</v>
+      </c>
+      <c r="N18" s="54" t="s">
+        <v>745</v>
+      </c>
+      <c r="O18" s="55" t="s">
+        <v>824</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S18" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="T18" s="6" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="50" t="s">
+        <v>746</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>747</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="H19" s="6" t="s">
         <v>699</v>
       </c>
-      <c r="F12" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="11" t="s">
+      <c r="I19" s="11" t="s">
         <v>700</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>702</v>
-      </c>
-      <c r="K12" s="11" t="s">
-        <v>703</v>
-      </c>
-      <c r="L12" s="11" t="s">
-        <v>704</v>
-      </c>
-      <c r="M12" s="61" t="s">
-        <v>705</v>
-      </c>
-      <c r="N12" s="55" t="s">
-        <v>706</v>
-      </c>
-      <c r="O12" s="56" t="s">
-        <v>826</v>
-      </c>
-      <c r="P12" s="59" t="s">
+      <c r="J19" s="11" t="s">
+        <v>748</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>749</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>750</v>
+      </c>
+      <c r="M19" s="48" t="s">
+        <v>751</v>
+      </c>
+      <c r="N19" s="54" t="s">
+        <v>752</v>
+      </c>
+      <c r="O19" s="55" t="s">
+        <v>827</v>
+      </c>
+      <c r="P19" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="Q12" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R12" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S12" s="59" t="s">
+      <c r="Q19" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="S19" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="T12" s="60" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
-        <v>707</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>708</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>709</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>710</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>711</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>712</v>
-      </c>
-      <c r="M13" s="61" t="s">
-        <v>713</v>
-      </c>
-      <c r="N13" s="57" t="s">
-        <v>714</v>
-      </c>
-      <c r="O13" s="56" t="s">
-        <v>827</v>
-      </c>
-      <c r="P13" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q13" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R13" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S13" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T13" s="60" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
-        <v>715</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>716</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>420</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>717</v>
-      </c>
-      <c r="K14" s="11" t="s">
-        <v>718</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>719</v>
-      </c>
-      <c r="M14" s="61" t="s">
-        <v>720</v>
-      </c>
-      <c r="N14" s="57" t="s">
-        <v>721</v>
-      </c>
-      <c r="O14" s="56" t="s">
-        <v>828</v>
-      </c>
-      <c r="P14" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q14" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R14" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S14" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T14" s="60" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="11" t="s">
-        <v>722</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>723</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>495</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>521</v>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>724</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>725</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>726</v>
-      </c>
-      <c r="M15" s="61" t="s">
-        <v>720</v>
-      </c>
-      <c r="N15" s="57" t="s">
-        <v>727</v>
-      </c>
-      <c r="O15" s="56" t="s">
-        <v>828</v>
-      </c>
-      <c r="P15" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q15" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R15" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S15" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T15" s="60" t="s">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="11" t="s">
-        <v>728</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>729</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>730</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>420</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>731</v>
-      </c>
-      <c r="K16" s="11" t="s">
-        <v>732</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>733</v>
-      </c>
-      <c r="M16" s="61" t="s">
-        <v>720</v>
-      </c>
-      <c r="N16" s="57" t="s">
-        <v>734</v>
-      </c>
-      <c r="O16" s="56" t="s">
-        <v>828</v>
-      </c>
-      <c r="P16" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q16" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R16" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S16" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T16" s="60" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="11" t="s">
-        <v>735</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>736</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>420</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>737</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>738</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>739</v>
-      </c>
-      <c r="M17" s="61" t="s">
-        <v>720</v>
-      </c>
-      <c r="N17" s="57" t="s">
-        <v>740</v>
-      </c>
-      <c r="O17" s="56" t="s">
-        <v>828</v>
-      </c>
-      <c r="P17" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q17" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R17" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S17" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T17" s="60" t="s">
+      <c r="T19" s="6" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
-        <v>741</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>742</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>699</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>495</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>521</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>743</v>
-      </c>
-      <c r="K18" s="11" t="s">
-        <v>744</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>745</v>
-      </c>
-      <c r="M18" s="61" t="s">
-        <v>705</v>
-      </c>
-      <c r="N18" s="57" t="s">
-        <v>746</v>
-      </c>
-      <c r="O18" s="56" t="s">
-        <v>826</v>
-      </c>
-      <c r="P18" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q18" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R18" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S18" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T18" s="60" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="11" t="s">
-        <v>747</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>748</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>282</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>495</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>521</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>700</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>701</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>749</v>
-      </c>
-      <c r="K19" s="11" t="s">
-        <v>750</v>
-      </c>
-      <c r="L19" s="11" t="s">
-        <v>751</v>
-      </c>
-      <c r="M19" s="61" t="s">
-        <v>752</v>
-      </c>
-      <c r="N19" s="57" t="s">
-        <v>753</v>
-      </c>
-      <c r="O19" s="56" t="s">
-        <v>829</v>
-      </c>
-      <c r="P19" s="59" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q19" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="R19" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="S19" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="T19" s="60" t="s">
-        <v>825</v>
-      </c>
-    </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N79" s="40"/>
+      <c r="N79" s="37"/>
     </row>
     <row r="80" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N80" s="40"/>
+      <c r="N80" s="37"/>
     </row>
     <row r="81" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N81" s="40"/>
+      <c r="N81" s="37"/>
     </row>
     <row r="82" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N82" s="40"/>
+      <c r="N82" s="37"/>
     </row>
     <row r="83" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N83" s="40"/>
+      <c r="N83" s="37"/>
     </row>
     <row r="84" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N84" s="40"/>
+      <c r="N84" s="37"/>
     </row>
     <row r="85" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N85" s="40"/>
+      <c r="N85" s="37"/>
     </row>
     <row r="86" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N86" s="40"/>
+      <c r="N86" s="37"/>
     </row>
     <row r="87" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N87" s="40"/>
+      <c r="N87" s="37"/>
     </row>
     <row r="88" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N88" s="40"/>
+      <c r="N88" s="37"/>
     </row>
     <row r="89" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N89" s="40"/>
+      <c r="N89" s="37"/>
     </row>
     <row r="90" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N90" s="40"/>
+      <c r="N90" s="37"/>
     </row>
     <row r="91" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N91" s="40"/>
+      <c r="N91" s="37"/>
     </row>
     <row r="92" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N92" s="40"/>
+      <c r="N92" s="37"/>
     </row>
     <row r="93" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N93" s="40"/>
+      <c r="N93" s="37"/>
     </row>
     <row r="94" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N94" s="40"/>
+      <c r="N94" s="37"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9306,14 +9299,14 @@
     <hyperlink ref="M10" r:id="rId8" tooltip="Bukti Bug BUG-009 (Modal detail offline badge forced)" xr:uid="{957AC965-CDAE-4E45-9715-3F261B118AA6}"/>
     <hyperlink ref="M11" r:id="rId9" tooltip="Bukti Bug BUG-010 (Kontras rendah &amp; font mikroskopis)" xr:uid="{2472314D-181C-4762-93DD-373BD42FF2A8}"/>
     <hyperlink ref="M6" r:id="rId10" tooltip="Bukti Error ZIP Corrupt (Windows cannot open folder - zip is invalid)" xr:uid="{66D2B4BE-3BA7-41E6-9543-27F46434CB16}"/>
-    <hyperlink ref="M12" r:id="rId11" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{D6814995-189E-4B20-A2B0-530BF1B89F49}"/>
-    <hyperlink ref="M13" r:id="rId12" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{8BC39E5B-41A9-4A5F-9E5F-CC7C53EEE103}"/>
-    <hyperlink ref="M14" r:id="rId13" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{25A97AC8-DE1A-459E-8420-2DA4BC4AD966}"/>
-    <hyperlink ref="M15" r:id="rId14" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{26A83C54-2000-447D-B722-0C4DA7A28417}"/>
-    <hyperlink ref="M16" r:id="rId15" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{27B578EC-B406-43A3-8376-10E14DA97076}"/>
-    <hyperlink ref="M17" r:id="rId16" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{FE2E578F-A747-40DF-B70A-F7EBAC061E92}"/>
-    <hyperlink ref="M18" r:id="rId17" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{DAF3B109-1DD3-4844-90EA-F48D5A4867FC}"/>
-    <hyperlink ref="M19" r:id="rId18" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{D31C288A-EE09-4F41-98E2-4C6A3E9BB863}"/>
+    <hyperlink ref="M12" r:id="rId11" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{554E9CD6-0E2D-46E9-99E9-86DF7BE25C93}"/>
+    <hyperlink ref="M13" r:id="rId12" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{101E7DF8-CC3C-4B60-8E0F-863683CBE6BD}"/>
+    <hyperlink ref="M14" r:id="rId13" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{4ED403FB-2A6E-49BE-9EC0-A9979F823AF8}"/>
+    <hyperlink ref="M15" r:id="rId14" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{1225B56A-2AFB-4FDD-AD9E-C737023B98E6}"/>
+    <hyperlink ref="M16" r:id="rId15" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{7C31B6E8-3F6C-4965-9B3F-FD830B430453}"/>
+    <hyperlink ref="M17" r:id="rId16" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{BAEBB03A-5DEE-4DC5-A7F6-01A8B56A7F03}"/>
+    <hyperlink ref="M18" r:id="rId17" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{FC09FA71-E15B-4E40-9FDE-FC2E06A5C390}"/>
+    <hyperlink ref="M19" r:id="rId18" tooltip="Buka Bukti Screenshot Hari-10" xr:uid="{BE4C4261-C49E-4C6D-BD5B-5CB08247E9E3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId19"/>
@@ -9633,10 +9626,10 @@
         <v>5</v>
       </c>
       <c r="K8" s="24" t="s">
+        <v>582</v>
+      </c>
+      <c r="L8" s="7" t="s">
         <v>583</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>584</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -9671,10 +9664,10 @@
         <v>5</v>
       </c>
       <c r="K9" s="24" t="s">
+        <v>584</v>
+      </c>
+      <c r="L9" s="7" t="s">
         <v>585</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -9716,40 +9709,40 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="47">
+      <c r="B11" s="42">
         <v>10</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="D11" s="47">
+      <c r="D11" s="42">
         <v>9</v>
       </c>
-      <c r="E11" s="47">
+      <c r="E11" s="42">
         <v>9</v>
       </c>
-      <c r="F11" s="47">
-        <v>0</v>
-      </c>
-      <c r="G11" s="47">
-        <v>0</v>
-      </c>
-      <c r="H11" s="47">
-        <v>0</v>
-      </c>
-      <c r="I11" s="47">
+      <c r="F11" s="42">
+        <v>0</v>
+      </c>
+      <c r="G11" s="42">
+        <v>0</v>
+      </c>
+      <c r="H11" s="42">
+        <v>0</v>
+      </c>
+      <c r="I11" s="42">
         <v>1</v>
       </c>
-      <c r="J11" s="47">
-        <v>0</v>
-      </c>
-      <c r="K11" s="49" t="s">
+      <c r="J11" s="42">
+        <v>0</v>
+      </c>
+      <c r="K11" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="L11" s="44" t="s">
+      <c r="L11" s="40" t="s">
         <v>106</v>
       </c>
     </row>
@@ -9767,10 +9760,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="13">
         <v>0</v>
@@ -9790,8 +9783,8 @@
       <c r="L12" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="M12" s="54"/>
-      <c r="N12" s="54"/>
+      <c r="M12" s="49"/>
+      <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="12" t="s">
@@ -9830,7 +9823,7 @@
       <c r="L13" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="M13" s="54"/>
+      <c r="M13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="12" t="s">
@@ -9869,7 +9862,7 @@
       <c r="L14" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="M14" s="54"/>
+      <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="12" t="s">
@@ -9908,7 +9901,7 @@
       <c r="L15" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="M15" s="54"/>
+      <c r="M15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="12" t="s">
@@ -9947,7 +9940,7 @@
       <c r="L16" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="M16" s="54"/>
+      <c r="M16" s="49"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="12" t="s">
@@ -9986,7 +9979,7 @@
       <c r="L17" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="M17" s="54"/>
+      <c r="M17" s="49"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="12" t="s">
@@ -10025,7 +10018,7 @@
       <c r="L18" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="M18" s="54"/>
+      <c r="M18" s="49"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="12" t="s">
@@ -10064,7 +10057,7 @@
       <c r="L19" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="M19" s="54"/>
+      <c r="M19" s="49"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="12" t="s">
@@ -10523,52 +10516,52 @@
       </c>
     </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N79" s="40"/>
+      <c r="N79" s="37"/>
     </row>
     <row r="80" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N80" s="40"/>
+      <c r="N80" s="37"/>
     </row>
     <row r="81" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N81" s="40"/>
+      <c r="N81" s="37"/>
     </row>
     <row r="82" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N82" s="40"/>
+      <c r="N82" s="37"/>
     </row>
     <row r="83" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N83" s="40"/>
+      <c r="N83" s="37"/>
     </row>
     <row r="84" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N84" s="40"/>
+      <c r="N84" s="37"/>
     </row>
     <row r="85" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N85" s="40"/>
+      <c r="N85" s="37"/>
     </row>
     <row r="86" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N86" s="40"/>
+      <c r="N86" s="37"/>
     </row>
     <row r="87" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N87" s="40"/>
+      <c r="N87" s="37"/>
     </row>
     <row r="88" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N88" s="40"/>
+      <c r="N88" s="37"/>
     </row>
     <row r="89" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N89" s="40"/>
+      <c r="N89" s="37"/>
     </row>
     <row r="90" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N90" s="40"/>
+      <c r="N90" s="37"/>
     </row>
     <row r="91" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N91" s="40"/>
+      <c r="N91" s="37"/>
     </row>
     <row r="92" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N92" s="40"/>
+      <c r="N92" s="37"/>
     </row>
     <row r="93" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N93" s="40"/>
+      <c r="N93" s="37"/>
     </row>
     <row r="94" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N94" s="40"/>
+      <c r="N94" s="37"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10907,7 +10900,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="27" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B14" s="13">
         <f>COUNTIF(MASTER_TC!C:C,A14)</f>
@@ -10932,7 +10925,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B15" s="30">
         <f>SUM(B2:B14)</f>

</xml_diff>

<commit_message>
feat(qa): release day-12 test reports, evidence screenshots, master test cases, and floorplan calibration
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\docs\qa-testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\PENGUMPULAN_DRIVE_HARI-12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27161A07-7B65-45CC-8040-B9FD6F881852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F4E92F-C8F5-4D3A-B612-2E2C1BAC2576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="220" windowWidth="14400" windowHeight="7810" firstSheet="2" activeTab="4" xr2:uid="{D20540B9-5A4B-4C0F-A1AA-6997D01BA992}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="830">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="858">
   <si>
     <t>TC ID</t>
   </si>
@@ -1441,9 +1441,6 @@
     <t>Test di Postman, backend jalan</t>
   </si>
   <si>
-    <t>200 OK, token didapat</t>
-  </si>
-  <si>
     <t>404 Endpoint belum 
 diimplementasi</t>
   </si>
@@ -1604,10 +1601,6 @@
     <t>Aset bertambah dari 16 menjadi 17, sistem normal</t>
   </si>
   <si>
-    <t>200 OK, data 17 aset tampil 
-di database</t>
-  </si>
-  <si>
     <t>Backend jalan, Postman 
 siap</t>
   </si>
@@ -2691,10 +2684,100 @@
     <t>screenshots/Hari-10/2026-10-21_Hari-10_final-dashboard_users-rbac.png</t>
   </si>
   <si>
-    <t>Status 200 OK. message: Heartbeat received, status: online, next_heartbeat_in: 30, Response Time 33 ms</t>
-  </si>
-  <si>
     <t>2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png</t>
+  </si>
+  <si>
+    <t>201 Created, log_id disimpan, ICMP ping latency 2ms, 0% packet loss, status online</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-MON-001_icmp-ping.png</t>
+  </si>
+  <si>
+    <t>201 Created, log_id disimpan, HTTP 200 OK, latency 27ms, status online</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-MON-002_http-health.png</t>
+  </si>
+  <si>
+    <t>201 Created, log_id disimpan, TCP port 80/443 OPEN, latency 33ms, status online</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-MON-003_tcp-port-scan.png</t>
+  </si>
+  <si>
+    <t>200 OK, 184 log telemetri &amp; latency berhasil ditarik dengan pagination limit 10, latency 19ms</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-MON-004_latency-logs.png</t>
+  </si>
+  <si>
+    <t>200 OK, summary data 17 unit online across 10 kategori tervalidasi presisi, latency 17ms</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-MON-005_monitoring-summary.png</t>
+  </si>
+  <si>
+    <t>200 OK, message: Heartbeat received, status online, RSSI -58 dBm, Response Time 33ms</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-INC-001_auto-incident-generated.png</t>
+  </si>
+  <si>
+    <t>Status kembali online saat paket ping baru masuk, tiket insiden otomatis berubah menjadi resolved (Auto-Recovery)</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-REC-001_auto-resolved-recovery.png</t>
+  </si>
+  <si>
+    <t>Status offline terekam, incident type Device Offline, severity high, tiket insiden #99 open tervalidasi via API</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-FAIL-001_offline-detection.png</t>
+  </si>
+  <si>
+    <t>Status offline terverifikasi, last_seen stop dihentikan saat sinyal telemetri terputus, notifikasi terkirim</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-NOTIF-001_alert-notification-trigger.png</t>
+  </si>
+  <si>
+    <t>Status sensor terputus tervalidasi, paket heartbeat timeout memicu alert, rekoneksi sukses menerima 200 OK (98ms)</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-HB-002_iot-heartbeat-recovery.png</t>
+  </si>
+  <si>
+    <t>Injeksi latensi tinggi &gt; 1000ms (1450ms) dan loss 15% memicu transisi status WARNING pada log dan dashboard</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-WARN-001_high-latency-warning.png</t>
+  </si>
+  <si>
+    <t>200 OK, message: Login berhasil!, token JWT aktif 24 jam diterima</t>
+  </si>
+  <si>
+    <t>Reza Tri Wardana</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_POST_1-Login_200-OK.png</t>
+  </si>
+  <si>
+    <t>200 OK, user_id: 5, full_name: Ahmad Reza Fahmi, role: admin</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_GET_2-Me_200-OK.png</t>
+  </si>
+  <si>
+    <t>200 OK, total 18 aset berhasil ditarik lengkap dengan pagination limit 20</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_GET_1-List-Assets_200-OK.png</t>
+  </si>
+  <si>
+    <t>200 OK, total 118 insiden terekam, auto-incident #120 tercatat untuk IOT-ESP-01</t>
+  </si>
+  <si>
+    <t>200 OK, total 79 notifikasi terekam, pagination limit 50, alert notif terverifikasi</t>
   </si>
 </sst>
 </file>
@@ -2918,7 +3001,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3067,10 +3150,17 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -3483,7 +3573,7 @@
         <v>21</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>22</v>
@@ -3492,16 +3582,20 @@
         <v>23</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>478</v>
+        <v>854</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
+      <c r="L2" s="57">
+        <v>46318</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>850</v>
+      </c>
+      <c r="N2" s="58" t="s">
+        <v>855</v>
+      </c>
       <c r="O2" s="4" t="s">
         <v>24</v>
       </c>
@@ -3510,7 +3604,7 @@
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3538,7 +3632,7 @@
         <v>48</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>75</v>
@@ -3579,14 +3673,14 @@
         <v>21</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>75</v>
@@ -3628,7 +3722,7 @@
         <v>50</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>75</v>
@@ -3670,7 +3764,7 @@
         <v>51</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>75</v>
@@ -3712,7 +3806,7 @@
         <v>52</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>75</v>
@@ -3726,7 +3820,7 @@
         <v>24</v>
       </c>
       <c r="P7" s="20" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
@@ -3756,7 +3850,7 @@
         <v>53</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>75</v>
@@ -3798,7 +3892,7 @@
         <v>50</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>75</v>
@@ -3840,7 +3934,7 @@
         <v>54</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>75</v>
@@ -3879,10 +3973,10 @@
         <v>47</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>55</v>
@@ -3906,7 +4000,7 @@
       </c>
       <c r="Q11" s="7"/>
       <c r="R11" s="6" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -3934,7 +4028,7 @@
         <v>55</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>75</v>
@@ -3944,7 +4038,7 @@
       </c>
       <c r="M12" s="7"/>
       <c r="N12" s="48" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="O12" s="14" t="s">
         <v>24</v>
@@ -3954,7 +4048,7 @@
       </c>
       <c r="Q12" s="7"/>
       <c r="R12" s="8" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -3977,7 +4071,7 @@
         <v>21</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>226</v>
@@ -4063,7 +4157,7 @@
         <v>228</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -4263,7 +4357,7 @@
         <v>417</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
@@ -4303,7 +4397,7 @@
         <v>231</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
@@ -4383,7 +4477,7 @@
         <v>233</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
@@ -4503,7 +4597,7 @@
         <v>236</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
@@ -4585,15 +4679,27 @@
       <c r="I28" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
+      <c r="J28" s="4" t="s">
+        <v>856</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="L28" s="59">
+        <v>46318</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>850</v>
+      </c>
+      <c r="N28" s="56" t="s">
+        <v>838</v>
+      </c>
       <c r="O28" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P28" s="5"/>
+      <c r="P28" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="Q28" s="7"/>
       <c r="R28" s="7"/>
     </row>
@@ -4625,15 +4731,23 @@
       <c r="I29" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
+      <c r="J29" s="4" t="s">
+        <v>839</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
-      <c r="N29" s="7"/>
+      <c r="N29" s="56" t="s">
+        <v>840</v>
+      </c>
       <c r="O29" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P29" s="5"/>
+      <c r="P29" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="Q29" s="7"/>
       <c r="R29" s="7"/>
     </row>
@@ -4663,17 +4777,25 @@
         <v>240</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>622</v>
-      </c>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
+        <v>620</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>841</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
-      <c r="N30" s="7"/>
+      <c r="N30" s="56" t="s">
+        <v>842</v>
+      </c>
       <c r="O30" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P30" s="5"/>
+      <c r="P30" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="Q30" s="7"/>
       <c r="R30" s="7"/>
     </row>
@@ -4705,15 +4827,23 @@
       <c r="I31" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
+      <c r="J31" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L31" s="7"/>
       <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
+      <c r="N31" s="56" t="s">
+        <v>844</v>
+      </c>
       <c r="O31" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P31" s="5"/>
+      <c r="P31" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="Q31" s="7"/>
       <c r="R31" s="7"/>
     </row>
@@ -4743,17 +4873,25 @@
         <v>242</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
+        <v>623</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>845</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L32" s="7"/>
       <c r="M32" s="7"/>
-      <c r="N32" s="7"/>
+      <c r="N32" s="56" t="s">
+        <v>846</v>
+      </c>
       <c r="O32" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P32" s="5"/>
+      <c r="P32" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="Q32" s="7"/>
       <c r="R32" s="7"/>
     </row>
@@ -4785,15 +4923,23 @@
       <c r="I33" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
+      <c r="J33" s="4" t="s">
+        <v>847</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L33" s="7"/>
       <c r="M33" s="7"/>
-      <c r="N33" s="7"/>
+      <c r="N33" s="56" t="s">
+        <v>848</v>
+      </c>
       <c r="O33" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P33" s="5"/>
+      <c r="P33" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="Q33" s="7"/>
       <c r="R33" s="7"/>
     </row>
@@ -4983,7 +5129,7 @@
         <v>223</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -5023,7 +5169,7 @@
         <v>247</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -5066,14 +5212,20 @@
         <v>263</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>429</v>
+        <v>849</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L40" s="4"/>
-      <c r="M40" s="4"/>
-      <c r="N40" s="7"/>
+      <c r="L40" s="57">
+        <v>46318</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>850</v>
+      </c>
+      <c r="N40" s="56" t="s">
+        <v>851</v>
+      </c>
       <c r="O40" s="4" t="s">
         <v>24</v>
       </c>
@@ -5193,16 +5345,20 @@
       <c r="I43" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="4" t="s">
-        <v>70</v>
+      <c r="J43" s="4" t="s">
+        <v>852</v>
+      </c>
+      <c r="K43" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="L43" s="57">
+        <v>46318</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="N43" s="45" t="s">
-        <v>594</v>
+        <v>850</v>
+      </c>
+      <c r="N43" s="47" t="s">
+        <v>853</v>
       </c>
       <c r="O43" s="4" t="s">
         <v>24</v>
@@ -5280,7 +5436,7 @@
         <v>280</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="K45" s="4" t="s">
         <v>76</v>
@@ -5292,7 +5448,7 @@
         <v>67</v>
       </c>
       <c r="N45" s="45" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="O45" s="4" t="s">
         <v>24</v>
@@ -5337,10 +5493,10 @@
         <v>70</v>
       </c>
       <c r="M46" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="N46" s="45" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="O46" s="4" t="s">
         <v>24</v>
@@ -5511,7 +5667,7 @@
     </row>
     <row r="51" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B51" s="13">
         <v>16</v>
@@ -5520,7 +5676,7 @@
         <v>282</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>20</v>
@@ -5529,16 +5685,16 @@
         <v>21</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="I51" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="J51" s="4" t="s">
         <v>473</v>
-      </c>
-      <c r="J51" s="4" t="s">
-        <v>474</v>
       </c>
       <c r="K51" s="4" t="s">
         <v>75</v>
@@ -5550,7 +5706,7 @@
         <v>69</v>
       </c>
       <c r="N51" s="45" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="O51" s="4" t="s">
         <v>24</v>
@@ -5560,7 +5716,7 @@
       </c>
       <c r="Q51" s="7"/>
       <c r="R51" s="4" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="52" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -5671,15 +5827,23 @@
       <c r="I54" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
+      <c r="J54" s="4" t="s">
+        <v>827</v>
+      </c>
+      <c r="K54" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L54" s="4"/>
       <c r="M54" s="4"/>
-      <c r="N54" s="7"/>
+      <c r="N54" s="56" t="s">
+        <v>828</v>
+      </c>
       <c r="O54" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P54" s="5"/>
+      <c r="P54" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="Q54" s="7"/>
       <c r="R54" s="7"/>
     </row>
@@ -5711,15 +5875,23 @@
       <c r="I55" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
+      <c r="J55" s="4" t="s">
+        <v>829</v>
+      </c>
+      <c r="K55" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L55" s="4"/>
       <c r="M55" s="4"/>
-      <c r="N55" s="7"/>
+      <c r="N55" s="56" t="s">
+        <v>830</v>
+      </c>
       <c r="O55" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P55" s="5"/>
+      <c r="P55" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="Q55" s="7"/>
       <c r="R55" s="7"/>
     </row>
@@ -5751,15 +5923,23 @@
       <c r="I56" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
+      <c r="J56" s="4" t="s">
+        <v>831</v>
+      </c>
+      <c r="K56" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L56" s="4"/>
       <c r="M56" s="4"/>
-      <c r="N56" s="7"/>
+      <c r="N56" s="56" t="s">
+        <v>832</v>
+      </c>
       <c r="O56" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P56" s="5"/>
+      <c r="P56" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="Q56" s="7"/>
       <c r="R56" s="7"/>
     </row>
@@ -5791,15 +5971,23 @@
       <c r="I57" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
+      <c r="J57" s="4" t="s">
+        <v>833</v>
+      </c>
+      <c r="K57" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L57" s="4"/>
       <c r="M57" s="4"/>
-      <c r="N57" s="7"/>
+      <c r="N57" s="56" t="s">
+        <v>834</v>
+      </c>
       <c r="O57" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P57" s="5"/>
+      <c r="P57" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="Q57" s="7"/>
       <c r="R57" s="7"/>
     </row>
@@ -5831,15 +6019,23 @@
       <c r="I58" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
+      <c r="J58" s="4" t="s">
+        <v>835</v>
+      </c>
+      <c r="K58" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
-      <c r="N58" s="7"/>
+      <c r="N58" s="56" t="s">
+        <v>836</v>
+      </c>
       <c r="O58" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P58" s="5"/>
+      <c r="P58" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="Q58" s="7"/>
       <c r="R58" s="7"/>
     </row>
@@ -5872,20 +6068,22 @@
         <v>323</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>828</v>
+        <v>837</v>
       </c>
       <c r="K59" s="4" t="s">
         <v>75</v>
       </c>
       <c r="L59" s="4"/>
       <c r="M59" s="4"/>
-      <c r="N59" s="57" t="s">
-        <v>829</v>
+      <c r="N59" s="37" t="s">
+        <v>826</v>
       </c>
       <c r="O59" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P59" s="5"/>
+      <c r="P59" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="Q59" s="7"/>
       <c r="R59" s="7"/>
     </row>
@@ -6077,11 +6275,21 @@
       <c r="I64" s="4" t="s">
         <v>340</v>
       </c>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="4"/>
-      <c r="M64" s="4"/>
-      <c r="N64" s="7"/>
+      <c r="J64" s="4" t="s">
+        <v>857</v>
+      </c>
+      <c r="K64" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="L64" s="57">
+        <v>46318</v>
+      </c>
+      <c r="M64" s="4" t="s">
+        <v>850</v>
+      </c>
+      <c r="N64" s="56" t="s">
+        <v>844</v>
+      </c>
       <c r="O64" s="4" t="s">
         <v>24</v>
       </c>
@@ -6198,7 +6406,7 @@
         <v>349</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="K67" s="4" t="s">
         <v>75</v>
@@ -6212,7 +6420,7 @@
       <c r="P67" s="5"/>
       <c r="Q67" s="7"/>
       <c r="R67" s="6" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="68" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -6324,7 +6532,7 @@
         <v>358</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="K70" s="4" t="s">
         <v>75</v>
@@ -6383,16 +6591,16 @@
     </row>
     <row r="72" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B72" s="10">
         <v>8</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>20</v>
@@ -6401,16 +6609,16 @@
         <v>21</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="I72" s="6" t="s">
         <v>535</v>
       </c>
-      <c r="H72" s="6" t="s">
+      <c r="J72" s="6" t="s">
         <v>536</v>
-      </c>
-      <c r="I72" s="6" t="s">
-        <v>537</v>
-      </c>
-      <c r="J72" s="6" t="s">
-        <v>538</v>
       </c>
       <c r="K72" s="36" t="s">
         <v>75</v>
@@ -6418,7 +6626,7 @@
       <c r="L72" s="10"/>
       <c r="M72" s="10"/>
       <c r="N72" s="45" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="O72" s="4" t="s">
         <v>24</v>
@@ -6428,21 +6636,21 @@
       </c>
       <c r="Q72" s="4"/>
       <c r="R72" s="6" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="73" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B73" s="10">
         <v>8</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>20</v>
@@ -6451,16 +6659,16 @@
         <v>47</v>
       </c>
       <c r="G73" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="I73" s="6" t="s">
         <v>542</v>
       </c>
-      <c r="H73" s="6" t="s">
+      <c r="J73" s="6" t="s">
         <v>543</v>
-      </c>
-      <c r="I73" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="J73" s="6" t="s">
-        <v>545</v>
       </c>
       <c r="K73" s="36" t="s">
         <v>75</v>
@@ -6468,7 +6676,7 @@
       <c r="L73" s="10"/>
       <c r="M73" s="10"/>
       <c r="N73" s="45" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="O73" s="4" t="s">
         <v>24</v>
@@ -6478,21 +6686,21 @@
       </c>
       <c r="Q73" s="4"/>
       <c r="R73" s="6" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="74" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B74" s="10">
         <v>8</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>20</v>
@@ -6501,16 +6709,16 @@
         <v>47</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="I74" s="6" t="s">
         <v>549</v>
       </c>
-      <c r="H74" s="6" t="s">
+      <c r="J74" s="6" t="s">
         <v>550</v>
-      </c>
-      <c r="I74" s="6" t="s">
-        <v>551</v>
-      </c>
-      <c r="J74" s="6" t="s">
-        <v>552</v>
       </c>
       <c r="K74" s="36" t="s">
         <v>75</v>
@@ -6518,7 +6726,7 @@
       <c r="L74" s="10"/>
       <c r="M74" s="10"/>
       <c r="N74" s="45" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="O74" s="4" t="s">
         <v>24</v>
@@ -6528,21 +6736,21 @@
       </c>
       <c r="Q74" s="4"/>
       <c r="R74" s="6" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="75" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B75" s="10">
         <v>8</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>46</v>
@@ -6551,16 +6759,16 @@
         <v>21</v>
       </c>
       <c r="G75" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="I75" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="H75" s="6" t="s">
+      <c r="J75" s="6" t="s">
         <v>557</v>
-      </c>
-      <c r="I75" s="6" t="s">
-        <v>558</v>
-      </c>
-      <c r="J75" s="6" t="s">
-        <v>559</v>
       </c>
       <c r="K75" s="36" t="s">
         <v>75</v>
@@ -6568,7 +6776,7 @@
       <c r="L75" s="10"/>
       <c r="M75" s="10"/>
       <c r="N75" s="45" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="O75" s="4" t="s">
         <v>24</v>
@@ -6578,21 +6786,21 @@
       </c>
       <c r="Q75" s="4"/>
       <c r="R75" s="6" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="76" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B76" s="10">
         <v>8</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>20</v>
@@ -6601,16 +6809,16 @@
         <v>47</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="I76" s="6" t="s">
         <v>563</v>
       </c>
-      <c r="H76" s="6" t="s">
+      <c r="J76" s="6" t="s">
         <v>564</v>
-      </c>
-      <c r="I76" s="6" t="s">
-        <v>565</v>
-      </c>
-      <c r="J76" s="6" t="s">
-        <v>566</v>
       </c>
       <c r="K76" s="36" t="s">
         <v>75</v>
@@ -6619,10 +6827,10 @@
         <v>420</v>
       </c>
       <c r="M76" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="N76" s="45" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="O76" s="4" t="s">
         <v>24</v>
@@ -6632,21 +6840,21 @@
       </c>
       <c r="Q76" s="4"/>
       <c r="R76" s="6" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="77" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="B77" s="10">
         <v>8</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E77" s="4" t="s">
         <v>20</v>
@@ -6655,28 +6863,28 @@
         <v>21</v>
       </c>
       <c r="G77" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="I77" s="6" t="s">
         <v>570</v>
       </c>
-      <c r="H77" s="6" t="s">
+      <c r="J77" s="6" t="s">
         <v>571</v>
-      </c>
-      <c r="I77" s="6" t="s">
-        <v>572</v>
-      </c>
-      <c r="J77" s="6" t="s">
-        <v>573</v>
       </c>
       <c r="K77" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L77" s="10" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="M77" s="10" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="N77" s="45" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="O77" s="4" t="s">
         <v>24</v>
@@ -6686,21 +6894,21 @@
       </c>
       <c r="Q77" s="4"/>
       <c r="R77" s="6" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="78" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B78" s="10">
         <v>8</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>20</v>
@@ -6709,16 +6917,16 @@
         <v>47</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="I78" s="6" t="s">
         <v>577</v>
       </c>
-      <c r="H78" s="6" t="s">
+      <c r="J78" s="6" t="s">
         <v>578</v>
-      </c>
-      <c r="I78" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="J78" s="6" t="s">
-        <v>580</v>
       </c>
       <c r="K78" s="36" t="s">
         <v>75</v>
@@ -6726,7 +6934,7 @@
       <c r="L78" s="10"/>
       <c r="M78" s="10"/>
       <c r="N78" s="45" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="O78" s="4" t="s">
         <v>24</v>
@@ -6736,39 +6944,39 @@
       </c>
       <c r="Q78" s="4"/>
       <c r="R78" s="6" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="79" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="B79" s="6">
         <v>9</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="F79" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G79" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="I79" s="6" t="s">
         <v>629</v>
       </c>
-      <c r="H79" s="6" t="s">
+      <c r="J79" s="6" t="s">
         <v>630</v>
-      </c>
-      <c r="I79" s="6" t="s">
-        <v>631</v>
-      </c>
-      <c r="J79" s="6" t="s">
-        <v>632</v>
       </c>
       <c r="K79" s="46" t="s">
         <v>75</v>
@@ -6776,7 +6984,7 @@
       <c r="L79" s="8"/>
       <c r="M79" s="8"/>
       <c r="N79" s="47" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="O79" s="6" t="s">
         <v>24</v>
@@ -6785,42 +6993,42 @@
         <v>104</v>
       </c>
       <c r="Q79" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R79" s="6" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
     <row r="80" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B80" s="6">
         <v>9</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="I80" s="6" t="s">
         <v>639</v>
       </c>
-      <c r="H80" s="6" t="s">
+      <c r="J80" s="6" t="s">
         <v>640</v>
-      </c>
-      <c r="I80" s="6" t="s">
-        <v>641</v>
-      </c>
-      <c r="J80" s="6" t="s">
-        <v>642</v>
       </c>
       <c r="K80" s="46" t="s">
         <v>75</v>
@@ -6828,7 +7036,7 @@
       <c r="L80" s="8"/>
       <c r="M80" s="8"/>
       <c r="N80" s="47" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>24</v>
@@ -6837,42 +7045,42 @@
         <v>104</v>
       </c>
       <c r="Q80" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R80" s="6" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
     </row>
     <row r="81" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B81" s="6">
         <v>9</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F81" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G81" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="I81" s="6" t="s">
         <v>647</v>
       </c>
-      <c r="H81" s="6" t="s">
+      <c r="J81" s="6" t="s">
         <v>648</v>
-      </c>
-      <c r="I81" s="6" t="s">
-        <v>649</v>
-      </c>
-      <c r="J81" s="6" t="s">
-        <v>650</v>
       </c>
       <c r="K81" s="46" t="s">
         <v>75</v>
@@ -6880,7 +7088,7 @@
       <c r="L81" s="8"/>
       <c r="M81" s="8"/>
       <c r="N81" s="47" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="O81" s="6" t="s">
         <v>24</v>
@@ -6889,42 +7097,42 @@
         <v>104</v>
       </c>
       <c r="Q81" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R81" s="6" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
     </row>
     <row r="82" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A82" s="6" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B82" s="6">
         <v>9</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="I82" s="6" t="s">
         <v>656</v>
       </c>
-      <c r="H82" s="6" t="s">
+      <c r="J82" s="6" t="s">
         <v>657</v>
-      </c>
-      <c r="I82" s="6" t="s">
-        <v>658</v>
-      </c>
-      <c r="J82" s="6" t="s">
-        <v>659</v>
       </c>
       <c r="K82" s="46" t="s">
         <v>75</v>
@@ -6932,7 +7140,7 @@
       <c r="L82" s="8"/>
       <c r="M82" s="8"/>
       <c r="N82" s="47" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>24</v>
@@ -6941,42 +7149,42 @@
         <v>104</v>
       </c>
       <c r="Q82" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R82" s="6" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="6" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B83" s="6">
         <v>9</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F83" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G83" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="I83" s="6" t="s">
         <v>664</v>
       </c>
-      <c r="H83" s="6" t="s">
+      <c r="J83" s="6" t="s">
         <v>665</v>
-      </c>
-      <c r="I83" s="6" t="s">
-        <v>666</v>
-      </c>
-      <c r="J83" s="6" t="s">
-        <v>667</v>
       </c>
       <c r="K83" s="46" t="s">
         <v>75</v>
@@ -6984,7 +7192,7 @@
       <c r="L83" s="8"/>
       <c r="M83" s="8"/>
       <c r="N83" s="47" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="O83" s="6" t="s">
         <v>24</v>
@@ -6993,42 +7201,42 @@
         <v>104</v>
       </c>
       <c r="Q83" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R83" s="6" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A84" s="6" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B84" s="6">
         <v>9</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G84" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="I84" s="6" t="s">
         <v>673</v>
       </c>
-      <c r="H84" s="6" t="s">
+      <c r="J84" s="6" t="s">
         <v>674</v>
-      </c>
-      <c r="I84" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="J84" s="6" t="s">
-        <v>676</v>
       </c>
       <c r="K84" s="46" t="s">
         <v>75</v>
@@ -7036,7 +7244,7 @@
       <c r="L84" s="8"/>
       <c r="M84" s="8"/>
       <c r="N84" s="47" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="O84" s="6" t="s">
         <v>24</v>
@@ -7045,42 +7253,42 @@
         <v>104</v>
       </c>
       <c r="Q84" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R84" s="6" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
     </row>
     <row r="85" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" s="6" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B85" s="6">
         <v>9</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="F85" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G85" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="I85" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="H85" s="6" t="s">
+      <c r="J85" s="6" t="s">
         <v>683</v>
-      </c>
-      <c r="I85" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="J85" s="6" t="s">
-        <v>685</v>
       </c>
       <c r="K85" s="46" t="s">
         <v>75</v>
@@ -7088,7 +7296,7 @@
       <c r="L85" s="8"/>
       <c r="M85" s="8"/>
       <c r="N85" s="47" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="O85" s="6" t="s">
         <v>24</v>
@@ -7097,42 +7305,42 @@
         <v>104</v>
       </c>
       <c r="Q85" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R85" s="6" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
     </row>
     <row r="86" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" s="6" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B86" s="6">
         <v>9</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G86" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="I86" s="6" t="s">
         <v>690</v>
       </c>
-      <c r="H86" s="6" t="s">
+      <c r="J86" s="6" t="s">
         <v>691</v>
-      </c>
-      <c r="I86" s="6" t="s">
-        <v>692</v>
-      </c>
-      <c r="J86" s="6" t="s">
-        <v>693</v>
       </c>
       <c r="K86" s="46" t="s">
         <v>75</v>
@@ -7140,7 +7348,7 @@
       <c r="L86" s="8"/>
       <c r="M86" s="8"/>
       <c r="N86" s="47" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>24</v>
@@ -7149,15 +7357,15 @@
         <v>104</v>
       </c>
       <c r="Q86" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="R86" s="6" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
     </row>
     <row r="87" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="B87" s="6">
         <v>10</v>
@@ -7166,7 +7374,7 @@
         <v>35</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>20</v>
@@ -7175,16 +7383,16 @@
         <v>21</v>
       </c>
       <c r="G87" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>756</v>
+      </c>
+      <c r="I87" s="6" t="s">
         <v>757</v>
       </c>
-      <c r="H87" s="6" t="s">
+      <c r="J87" s="6" t="s">
         <v>758</v>
-      </c>
-      <c r="I87" s="6" t="s">
-        <v>759</v>
-      </c>
-      <c r="J87" s="6" t="s">
-        <v>760</v>
       </c>
       <c r="K87" s="46" t="s">
         <v>75</v>
@@ -7192,7 +7400,7 @@
       <c r="L87" s="8"/>
       <c r="M87" s="8"/>
       <c r="N87" s="47" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="O87" s="6" t="s">
         <v>24</v>
@@ -7201,15 +7409,15 @@
         <v>107</v>
       </c>
       <c r="Q87" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R87" s="6" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A88" s="6" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B88" s="6">
         <v>10</v>
@@ -7218,7 +7426,7 @@
         <v>35</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>20</v>
@@ -7227,16 +7435,16 @@
         <v>21</v>
       </c>
       <c r="G88" s="6" t="s">
+        <v>763</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="I88" s="6" t="s">
         <v>765</v>
       </c>
-      <c r="H88" s="6" t="s">
+      <c r="J88" s="6" t="s">
         <v>766</v>
-      </c>
-      <c r="I88" s="6" t="s">
-        <v>767</v>
-      </c>
-      <c r="J88" s="6" t="s">
-        <v>768</v>
       </c>
       <c r="K88" s="46" t="s">
         <v>75</v>
@@ -7244,7 +7452,7 @@
       <c r="L88" s="8"/>
       <c r="M88" s="8"/>
       <c r="N88" s="47" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="O88" s="6" t="s">
         <v>24</v>
@@ -7253,15 +7461,15 @@
         <v>107</v>
       </c>
       <c r="Q88" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R88" s="6" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="89" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B89" s="6">
         <v>10</v>
@@ -7270,7 +7478,7 @@
         <v>35</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>20</v>
@@ -7279,16 +7487,16 @@
         <v>21</v>
       </c>
       <c r="G89" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="I89" s="6" t="s">
         <v>772</v>
       </c>
-      <c r="H89" s="6" t="s">
+      <c r="J89" s="6" t="s">
         <v>773</v>
-      </c>
-      <c r="I89" s="6" t="s">
-        <v>774</v>
-      </c>
-      <c r="J89" s="6" t="s">
-        <v>775</v>
       </c>
       <c r="K89" s="46" t="s">
         <v>75</v>
@@ -7296,7 +7504,7 @@
       <c r="L89" s="8"/>
       <c r="M89" s="8"/>
       <c r="N89" s="47" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="O89" s="6" t="s">
         <v>24</v>
@@ -7305,42 +7513,42 @@
         <v>107</v>
       </c>
       <c r="Q89" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R89" s="6" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="90" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A90" s="6" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B90" s="6">
         <v>10</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G90" s="6" t="s">
+        <v>777</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="I90" s="6" t="s">
         <v>779</v>
       </c>
-      <c r="H90" s="6" t="s">
+      <c r="J90" s="6" t="s">
         <v>780</v>
-      </c>
-      <c r="I90" s="6" t="s">
-        <v>781</v>
-      </c>
-      <c r="J90" s="6" t="s">
-        <v>782</v>
       </c>
       <c r="K90" s="46" t="s">
         <v>75</v>
@@ -7348,7 +7556,7 @@
       <c r="L90" s="8"/>
       <c r="M90" s="8"/>
       <c r="N90" s="47" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="O90" s="6" t="s">
         <v>24</v>
@@ -7357,42 +7565,42 @@
         <v>107</v>
       </c>
       <c r="Q90" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R90" s="6" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="91" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A91" s="6" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B91" s="6">
         <v>10</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G91" s="6" t="s">
+        <v>785</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="I91" s="6" t="s">
         <v>787</v>
       </c>
-      <c r="H91" s="6" t="s">
+      <c r="J91" s="6" t="s">
         <v>788</v>
-      </c>
-      <c r="I91" s="6" t="s">
-        <v>789</v>
-      </c>
-      <c r="J91" s="6" t="s">
-        <v>790</v>
       </c>
       <c r="K91" s="46" t="s">
         <v>75</v>
@@ -7400,7 +7608,7 @@
       <c r="L91" s="8"/>
       <c r="M91" s="8"/>
       <c r="N91" s="47" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="O91" s="6" t="s">
         <v>24</v>
@@ -7409,42 +7617,42 @@
         <v>107</v>
       </c>
       <c r="Q91" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R91" s="6" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
     </row>
     <row r="92" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A92" s="6" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B92" s="6">
         <v>10</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G92" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="I92" s="6" t="s">
         <v>795</v>
       </c>
-      <c r="H92" s="6" t="s">
+      <c r="J92" s="6" t="s">
         <v>796</v>
-      </c>
-      <c r="I92" s="6" t="s">
-        <v>797</v>
-      </c>
-      <c r="J92" s="6" t="s">
-        <v>798</v>
       </c>
       <c r="K92" s="46" t="s">
         <v>75</v>
@@ -7452,7 +7660,7 @@
       <c r="L92" s="8"/>
       <c r="M92" s="8"/>
       <c r="N92" s="47" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="O92" s="6" t="s">
         <v>24</v>
@@ -7461,42 +7669,42 @@
         <v>107</v>
       </c>
       <c r="Q92" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R92" s="6" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
     </row>
     <row r="93" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="6" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B93" s="6">
         <v>10</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D93" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="G93" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="E93" s="6" t="s">
+      <c r="H93" s="6" t="s">
         <v>802</v>
       </c>
-      <c r="F93" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="G93" s="6" t="s">
+      <c r="I93" s="6" t="s">
         <v>803</v>
       </c>
-      <c r="H93" s="6" t="s">
+      <c r="J93" s="6" t="s">
         <v>804</v>
-      </c>
-      <c r="I93" s="6" t="s">
-        <v>805</v>
-      </c>
-      <c r="J93" s="6" t="s">
-        <v>806</v>
       </c>
       <c r="K93" s="46" t="s">
         <v>75</v>
@@ -7504,7 +7712,7 @@
       <c r="L93" s="8"/>
       <c r="M93" s="8"/>
       <c r="N93" s="47" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="O93" s="6" t="s">
         <v>24</v>
@@ -7513,42 +7721,42 @@
         <v>107</v>
       </c>
       <c r="Q93" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R93" s="6" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="94" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A94" s="6" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="B94" s="6">
         <v>10</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D94" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>808</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="G94" s="6" t="s">
         <v>809</v>
       </c>
-      <c r="E94" s="6" t="s">
+      <c r="H94" s="6" t="s">
         <v>810</v>
       </c>
-      <c r="F94" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="G94" s="6" t="s">
+      <c r="I94" s="6" t="s">
         <v>811</v>
       </c>
-      <c r="H94" s="6" t="s">
+      <c r="J94" s="6" t="s">
         <v>812</v>
-      </c>
-      <c r="I94" s="6" t="s">
-        <v>813</v>
-      </c>
-      <c r="J94" s="6" t="s">
-        <v>814</v>
       </c>
       <c r="K94" s="46" t="s">
         <v>75</v>
@@ -7556,7 +7764,7 @@
       <c r="L94" s="8"/>
       <c r="M94" s="8"/>
       <c r="N94" s="47" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>24</v>
@@ -7565,16 +7773,16 @@
         <v>107</v>
       </c>
       <c r="Q94" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="R94" s="6" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="N43" r:id="rId1" tooltip="Bukti error 500 column created_at" xr:uid="{F1645194-E524-4B93-93C0-93775656DF38}"/>
+    <hyperlink ref="N43" r:id="rId1" xr:uid="{F1645194-E524-4B93-93C0-93775656DF38}"/>
     <hyperlink ref="N45" r:id="rId2" tooltip="Bukti retest pass change-password" xr:uid="{83495BB2-4F28-4636-8350-D973F94E0902}"/>
     <hyperlink ref="N46" r:id="rId3" tooltip="Bukti retest pass GET /users" xr:uid="{2A6474F4-7C4B-46EE-BFDD-FFE06AF40E86}"/>
     <hyperlink ref="N51" r:id="rId4" tooltip="Bukti retest pass GET /users/1" xr:uid="{1D4D0B11-6BC6-4996-9878-75C18A64CB5A}"/>
@@ -7602,10 +7810,24 @@
     <hyperlink ref="N92" r:id="rId26" tooltip="2026-10-21_Hari-10_final-dashboard_desktop-1080p.png" xr:uid="{DF0874B5-F3A5-4940-B56E-5C8C97D816B7}"/>
     <hyperlink ref="N93" r:id="rId27" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{B17C34F4-F7BE-42EA-851C-9107F4B20CCB}"/>
     <hyperlink ref="N94" r:id="rId28" tooltip="2026-10-21_Hari-10_final-dashboard_users-rbac.png" xr:uid="{2241DBCB-8785-46FF-94D5-F6C6DED84A05}"/>
-    <hyperlink ref="N59" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png" xr:uid="{014D7D64-B7C6-4162-9E46-25E1D648DA6D}"/>
+    <hyperlink ref="N54" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-MON-001_icmp-ping.png" xr:uid="{8C32334C-50E2-461D-89AF-8EB45F63C7C7}"/>
+    <hyperlink ref="N55" r:id="rId30" tooltip="2026-10-22_Hari-11_TC-MON-002_http-health.png" xr:uid="{5D47D286-D7AE-4B03-A0A4-866AE4CEBB25}"/>
+    <hyperlink ref="N56" r:id="rId31" tooltip="2026-10-22_Hari-11_TC-MON-003_tcp-port-scan.png" xr:uid="{54A22B2F-0B75-42D5-8371-1C9E401985B0}"/>
+    <hyperlink ref="N57" r:id="rId32" tooltip="2026-10-22_Hari-11_TC-MON-004_latency-logs.png" xr:uid="{3B45532E-6326-4EFF-907E-9865FA5CE054}"/>
+    <hyperlink ref="N58" r:id="rId33" tooltip="2026-10-22_Hari-11_TC-MON-005_monitoring-summary.png" xr:uid="{C3BDC459-DA6D-4F63-83EB-830608126897}"/>
+    <hyperlink ref="N59" r:id="rId34" tooltip="2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png" xr:uid="{756D28A9-DCDF-427F-B5A7-F01AB6696F3F}"/>
+    <hyperlink ref="N28" r:id="rId35" xr:uid="{007CCACA-3220-4F7C-912C-66F1A0DC4260}"/>
+    <hyperlink ref="N29" r:id="rId36" tooltip="2026-10-23_Hari-12_TC-REC-001_auto-resolved-recovery.png" xr:uid="{DB45E82C-A556-4308-B54C-1019F073E6BD}"/>
+    <hyperlink ref="N30" r:id="rId37" tooltip="2026-10-23_Hari-12_TC-FAIL-001_offline-detection.png" xr:uid="{028E6BEF-3D80-4EAC-B73A-A23554BC740F}"/>
+    <hyperlink ref="N31" r:id="rId38" tooltip="2026-10-23_Hari-12_TC-NOTIF-001_alert-notification-trigger.png" xr:uid="{3D282DAD-DBA6-48CA-AB3F-2D3422710268}"/>
+    <hyperlink ref="N32" r:id="rId39" tooltip="2026-10-23_Hari-12_TC-HB-002_iot-heartbeat-recovery.png" xr:uid="{D3C4FE45-45EE-4B9C-B10E-CB4590A69183}"/>
+    <hyperlink ref="N33" r:id="rId40" tooltip="2026-10-23_Hari-12_TC-WARN-001_high-latency-warning.png" xr:uid="{5C311F97-1645-4AF3-BE81-26737B5A7616}"/>
+    <hyperlink ref="N40" r:id="rId41" xr:uid="{84DCE3CA-9396-4774-BABE-BA65D327F058}"/>
+    <hyperlink ref="N2" r:id="rId42" xr:uid="{38DE97AC-647E-4FAA-91DF-3E239D926B21}"/>
+    <hyperlink ref="N64" r:id="rId43" xr:uid="{4E8FCC19-840B-4A93-9C43-C6BBA664F2BB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId30"/>
+  <pageSetup orientation="portrait" r:id="rId44"/>
 </worksheet>
 </file>
 
@@ -7653,7 +7875,7 @@
         <v>427</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -7667,7 +7889,7 @@
         <v>87</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>260</v>
@@ -7679,13 +7901,13 @@
         <v>71</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H2" s="12" t="s">
         <v>90</v>
       </c>
       <c r="I2" s="32" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
@@ -7696,7 +7918,7 @@
         <v>87</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>282</v>
@@ -7708,24 +7930,24 @@
         <v>71</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H3" s="12" t="s">
         <v>96</v>
       </c>
       <c r="I3" s="32" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>93</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>260</v>
@@ -7737,24 +7959,24 @@
         <v>71</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>96</v>
       </c>
       <c r="I4" s="32" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>96</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>282</v>
@@ -7766,187 +7988,187 @@
         <v>71</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>96</v>
       </c>
       <c r="I5" s="32" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>100</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I6" s="32" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I7" s="32" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>420</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I8" s="32" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B9" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>420</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I9" s="32" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I10" s="32" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I11" s="32" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
@@ -7954,19 +8176,19 @@
       <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="56" t="s">
-        <v>588</v>
-      </c>
-      <c r="B13" s="56"/>
-      <c r="C13" s="56"/>
+      <c r="A13" s="60" t="s">
+        <v>586</v>
+      </c>
+      <c r="B13" s="60"/>
+      <c r="C13" s="60"/>
       <c r="M13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="56" t="s">
-        <v>589</v>
-      </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
+      <c r="A14" s="60" t="s">
+        <v>587</v>
+      </c>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
       <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
@@ -8117,7 +8339,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="N1" s="22" t="s">
         <v>62</v>
@@ -8146,7 +8368,7 @@
         <v>67</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>24</v>
@@ -8164,29 +8386,29 @@
         <v>21</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>451</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>452</v>
       </c>
       <c r="L2" s="6">
         <v>404</v>
       </c>
       <c r="M2" s="51" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="N2" s="33" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q2" s="4" t="s">
         <v>71</v>
@@ -8198,7 +8420,7 @@
         <v>90</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="W2" s="2"/>
     </row>
@@ -8207,7 +8429,7 @@
         <v>69</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>24</v>
@@ -8225,29 +8447,29 @@
         <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L3" s="6">
         <v>500</v>
       </c>
       <c r="M3" s="51" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="N3" s="33" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q3" s="4" t="s">
         <v>71</v>
@@ -8259,16 +8481,16 @@
         <v>96</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="W3" s="2"/>
     </row>
     <row r="4" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>24</v>
@@ -8286,29 +8508,29 @@
         <v>21</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I4" s="10"/>
       <c r="J4" s="6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L4" s="6">
         <v>500</v>
       </c>
       <c r="M4" s="51" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="N4" s="23" t="s">
+        <v>454</v>
+      </c>
+      <c r="O4" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="O4" s="4" t="s">
-        <v>456</v>
-      </c>
       <c r="P4" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>71</v>
@@ -8320,15 +8542,15 @@
         <v>96</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>24</v>
@@ -8346,29 +8568,29 @@
         <v>21</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" s="6" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L5" s="6">
         <v>500</v>
       </c>
       <c r="M5" s="51" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="N5" s="23" t="s">
+        <v>464</v>
+      </c>
+      <c r="O5" s="4" t="s">
         <v>465</v>
       </c>
-      <c r="O5" s="4" t="s">
-        <v>466</v>
-      </c>
       <c r="P5" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q5" s="4" t="s">
         <v>71</v>
@@ -8380,15 +8602,15 @@
         <v>96</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>24</v>
@@ -8397,7 +8619,7 @@
         <v>100</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>70</v>
@@ -8406,32 +8628,32 @@
         <v>21</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="L6" s="6" t="s">
         <v>497</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="M6" s="52" t="s">
+        <v>605</v>
+      </c>
+      <c r="N6" s="4" t="s">
         <v>498</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="O6" s="4" t="s">
         <v>499</v>
       </c>
-      <c r="M6" s="52" t="s">
-        <v>607</v>
-      </c>
-      <c r="N6" s="4" t="s">
-        <v>500</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>501</v>
-      </c>
       <c r="P6" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>24</v>
@@ -8440,15 +8662,15 @@
         <v>101</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>24</v>
@@ -8457,7 +8679,7 @@
         <v>101</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>70</v>
@@ -8466,32 +8688,32 @@
         <v>21</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" s="6" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>277</v>
       </c>
       <c r="M7" s="51" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R7" s="4" t="s">
         <v>24</v>
@@ -8500,15 +8722,15 @@
         <v>101</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>24</v>
@@ -8517,7 +8739,7 @@
         <v>101</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>420</v>
@@ -8526,32 +8748,32 @@
         <v>47</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>508</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="M8" s="51" t="s">
+        <v>595</v>
+      </c>
+      <c r="N8" s="4" t="s">
         <v>509</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="O8" s="4" t="s">
         <v>510</v>
       </c>
-      <c r="M8" s="51" t="s">
-        <v>597</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>512</v>
-      </c>
       <c r="P8" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R8" s="4" t="s">
         <v>24</v>
@@ -8560,15 +8782,15 @@
         <v>101</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>24</v>
@@ -8577,7 +8799,7 @@
         <v>101</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>420</v>
@@ -8586,32 +8808,32 @@
         <v>47</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="L9" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="M9" s="51" t="s">
+        <v>595</v>
+      </c>
+      <c r="N9" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="O9" s="4" t="s">
         <v>516</v>
       </c>
-      <c r="M9" s="51" t="s">
-        <v>597</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>517</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>518</v>
-      </c>
       <c r="P9" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R9" s="4" t="s">
         <v>24</v>
@@ -8620,15 +8842,15 @@
         <v>101</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>24</v>
@@ -8637,41 +8859,41 @@
         <v>101</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="L10" s="6" t="s">
         <v>521</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="M10" s="51" t="s">
+        <v>596</v>
+      </c>
+      <c r="N10" s="4" t="s">
         <v>522</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="O10" s="4" t="s">
         <v>523</v>
       </c>
-      <c r="M10" s="51" t="s">
-        <v>598</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>524</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>525</v>
-      </c>
       <c r="P10" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R10" s="4" t="s">
         <v>24</v>
@@ -8680,15 +8902,15 @@
         <v>101</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="11" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="42" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C11" s="43" t="s">
         <v>24</v>
@@ -8697,41 +8919,41 @@
         <v>101</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F11" s="43" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G11" s="43" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="H11" s="43" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I11" s="38"/>
       <c r="J11" s="39" t="s">
+        <v>525</v>
+      </c>
+      <c r="K11" s="39" t="s">
+        <v>526</v>
+      </c>
+      <c r="L11" s="39" t="s">
         <v>527</v>
       </c>
-      <c r="K11" s="39" t="s">
+      <c r="M11" s="51" t="s">
+        <v>595</v>
+      </c>
+      <c r="N11" s="43" t="s">
         <v>528</v>
       </c>
-      <c r="L11" s="39" t="s">
+      <c r="O11" s="43" t="s">
         <v>529</v>
       </c>
-      <c r="M11" s="51" t="s">
-        <v>597</v>
-      </c>
-      <c r="N11" s="43" t="s">
-        <v>530</v>
-      </c>
-      <c r="O11" s="43" t="s">
-        <v>531</v>
-      </c>
       <c r="P11" s="43" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q11" s="43" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R11" s="43" t="s">
         <v>24</v>
@@ -8740,15 +8962,15 @@
         <v>101</v>
       </c>
       <c r="T11" s="39" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="12" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="50" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>24</v>
@@ -8757,7 +8979,7 @@
         <v>107</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>70</v>
@@ -8766,34 +8988,34 @@
         <v>21</v>
       </c>
       <c r="H12" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>698</v>
+      </c>
+      <c r="J12" s="11" t="s">
         <v>699</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="K12" s="11" t="s">
         <v>700</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="L12" s="11" t="s">
         <v>701</v>
       </c>
-      <c r="K12" s="11" t="s">
+      <c r="M12" s="48" t="s">
         <v>702</v>
       </c>
-      <c r="L12" s="11" t="s">
+      <c r="N12" s="53" t="s">
         <v>703</v>
       </c>
-      <c r="M12" s="48" t="s">
-        <v>704</v>
-      </c>
-      <c r="N12" s="53" t="s">
-        <v>705</v>
-      </c>
       <c r="O12" s="55" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R12" s="4" t="s">
         <v>24</v>
@@ -8802,15 +9024,15 @@
         <v>107</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="50" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>24</v>
@@ -8819,7 +9041,7 @@
         <v>107</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>70</v>
@@ -8828,34 +9050,34 @@
         <v>21</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J13" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>708</v>
+      </c>
+      <c r="L13" s="11" t="s">
         <v>709</v>
       </c>
-      <c r="K13" s="11" t="s">
+      <c r="M13" s="48" t="s">
         <v>710</v>
       </c>
-      <c r="L13" s="11" t="s">
+      <c r="N13" s="54" t="s">
         <v>711</v>
       </c>
-      <c r="M13" s="48" t="s">
-        <v>712</v>
-      </c>
-      <c r="N13" s="54" t="s">
-        <v>713</v>
-      </c>
       <c r="O13" s="55" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q13" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R13" s="4" t="s">
         <v>24</v>
@@ -8864,15 +9086,15 @@
         <v>107</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="50" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>24</v>
@@ -8890,34 +9112,34 @@
         <v>47</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J14" s="11" t="s">
+        <v>714</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="L14" s="11" t="s">
         <v>716</v>
       </c>
-      <c r="K14" s="11" t="s">
+      <c r="M14" s="48" t="s">
         <v>717</v>
       </c>
-      <c r="L14" s="11" t="s">
+      <c r="N14" s="54" t="s">
         <v>718</v>
       </c>
-      <c r="M14" s="48" t="s">
-        <v>719</v>
-      </c>
-      <c r="N14" s="54" t="s">
-        <v>720</v>
-      </c>
       <c r="O14" s="55" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R14" s="4" t="s">
         <v>24</v>
@@ -8926,15 +9148,15 @@
         <v>107</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="50" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>24</v>
@@ -8946,40 +9168,40 @@
         <v>164</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J15" s="11" t="s">
+        <v>721</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>722</v>
+      </c>
+      <c r="L15" s="11" t="s">
         <v>723</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="M15" s="48" t="s">
+        <v>717</v>
+      </c>
+      <c r="N15" s="54" t="s">
         <v>724</v>
       </c>
-      <c r="L15" s="11" t="s">
-        <v>725</v>
-      </c>
-      <c r="M15" s="48" t="s">
-        <v>719</v>
-      </c>
-      <c r="N15" s="54" t="s">
-        <v>726</v>
-      </c>
       <c r="O15" s="55" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R15" s="4" t="s">
         <v>24</v>
@@ -8988,15 +9210,15 @@
         <v>107</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
     </row>
     <row r="16" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="50" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>24</v>
@@ -9005,7 +9227,7 @@
         <v>107</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>420</v>
@@ -9014,34 +9236,34 @@
         <v>47</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J16" s="11" t="s">
+        <v>728</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>729</v>
+      </c>
+      <c r="L16" s="11" t="s">
         <v>730</v>
       </c>
-      <c r="K16" s="11" t="s">
+      <c r="M16" s="48" t="s">
+        <v>717</v>
+      </c>
+      <c r="N16" s="54" t="s">
         <v>731</v>
       </c>
-      <c r="L16" s="11" t="s">
-        <v>732</v>
-      </c>
-      <c r="M16" s="48" t="s">
-        <v>719</v>
-      </c>
-      <c r="N16" s="54" t="s">
-        <v>733</v>
-      </c>
       <c r="O16" s="55" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R16" s="4" t="s">
         <v>24</v>
@@ -9050,15 +9272,15 @@
         <v>107</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="50" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>24</v>
@@ -9076,34 +9298,34 @@
         <v>47</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J17" s="11" t="s">
+        <v>734</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>735</v>
+      </c>
+      <c r="L17" s="11" t="s">
         <v>736</v>
       </c>
-      <c r="K17" s="11" t="s">
+      <c r="M17" s="48" t="s">
+        <v>717</v>
+      </c>
+      <c r="N17" s="54" t="s">
         <v>737</v>
       </c>
-      <c r="L17" s="11" t="s">
-        <v>738</v>
-      </c>
-      <c r="M17" s="48" t="s">
-        <v>719</v>
-      </c>
-      <c r="N17" s="54" t="s">
-        <v>739</v>
-      </c>
       <c r="O17" s="55" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q17" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R17" s="4" t="s">
         <v>24</v>
@@ -9112,15 +9334,15 @@
         <v>107</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
     </row>
     <row r="18" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="50" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>24</v>
@@ -9129,43 +9351,43 @@
         <v>107</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="I18" s="11" t="s">
         <v>698</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>700</v>
-      </c>
       <c r="J18" s="11" t="s">
+        <v>740</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>741</v>
+      </c>
+      <c r="L18" s="11" t="s">
         <v>742</v>
       </c>
-      <c r="K18" s="11" t="s">
+      <c r="M18" s="48" t="s">
+        <v>702</v>
+      </c>
+      <c r="N18" s="54" t="s">
         <v>743</v>
       </c>
-      <c r="L18" s="11" t="s">
-        <v>744</v>
-      </c>
-      <c r="M18" s="48" t="s">
-        <v>704</v>
-      </c>
-      <c r="N18" s="54" t="s">
-        <v>745</v>
-      </c>
       <c r="O18" s="55" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R18" s="4" t="s">
         <v>24</v>
@@ -9174,15 +9396,15 @@
         <v>107</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="50" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>24</v>
@@ -9194,40 +9416,40 @@
         <v>282</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J19" s="11" t="s">
+        <v>746</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>747</v>
+      </c>
+      <c r="L19" s="11" t="s">
         <v>748</v>
       </c>
-      <c r="K19" s="11" t="s">
+      <c r="M19" s="48" t="s">
         <v>749</v>
       </c>
-      <c r="L19" s="11" t="s">
+      <c r="N19" s="54" t="s">
         <v>750</v>
       </c>
-      <c r="M19" s="48" t="s">
-        <v>751</v>
-      </c>
-      <c r="N19" s="54" t="s">
-        <v>752</v>
-      </c>
       <c r="O19" s="55" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="R19" s="4" t="s">
         <v>24</v>
@@ -9236,7 +9458,7 @@
         <v>107</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
     </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.35">
@@ -9626,10 +9848,10 @@
         <v>5</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -9664,10 +9886,10 @@
         <v>5</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -9797,10 +10019,10 @@
         <v>82</v>
       </c>
       <c r="D13" s="13">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E13" s="13">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F13" s="13">
         <v>0</v>
@@ -10900,7 +11122,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="27" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B14" s="13">
         <f>COUNTIF(MASTER_TC!C:C,A14)</f>
@@ -10925,7 +11147,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B15" s="30">
         <f>SUM(B2:B14)</f>

</xml_diff>

<commit_message>
refactor(qa): sanitize and standardize day-12 authentic screenshots to exact 6 test cases
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\PENGUMPULAN_DRIVE_HARI-12\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\TAIMS_REMOTE_CHECK\docs\qa-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F4E92F-C8F5-4D3A-B612-2E2C1BAC2576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11FEC61-2AF6-4AB4-B1DF-98A63920229A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="220" windowWidth="14400" windowHeight="7810" firstSheet="2" activeTab="4" xr2:uid="{D20540B9-5A4B-4C0F-A1AA-6997D01BA992}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="858">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1697" uniqueCount="849">
   <si>
     <t>TC ID</t>
   </si>
@@ -2711,73 +2711,46 @@
     <t>2026-10-22_Hari-11_TC-MON-004_latency-logs.png</t>
   </si>
   <si>
-    <t>200 OK, summary data 17 unit online across 10 kategori tervalidasi presisi, latency 17ms</t>
-  </si>
-  <si>
-    <t>2026-10-22_Hari-11_TC-MON-005_monitoring-summary.png</t>
-  </si>
-  <si>
     <t>200 OK, message: Heartbeat received, status online, RSSI -58 dBm, Response Time 33ms</t>
   </si>
   <si>
     <t>2026-10-23_Hari-12_TC-INC-001_auto-incident-generated.png</t>
   </si>
   <si>
-    <t>Status kembali online saat paket ping baru masuk, tiket insiden otomatis berubah menjadi resolved (Auto-Recovery)</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-REC-001_auto-resolved-recovery.png</t>
-  </si>
-  <si>
-    <t>Status offline terekam, incident type Device Offline, severity high, tiket insiden #99 open tervalidasi via API</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-FAIL-001_offline-detection.png</t>
-  </si>
-  <si>
-    <t>Status offline terverifikasi, last_seen stop dihentikan saat sinyal telemetri terputus, notifikasi terkirim</t>
-  </si>
-  <si>
     <t>2026-10-23_Hari-12_TC-NOTIF-001_alert-notification-trigger.png</t>
   </si>
   <si>
-    <t>Status sensor terputus tervalidasi, paket heartbeat timeout memicu alert, rekoneksi sukses menerima 200 OK (98ms)</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-HB-002_iot-heartbeat-recovery.png</t>
-  </si>
-  <si>
-    <t>Injeksi latensi tinggi &gt; 1000ms (1450ms) dan loss 15% memicu transisi status WARNING pada log dan dashboard</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-WARN-001_high-latency-warning.png</t>
-  </si>
-  <si>
     <t>200 OK, message: Login berhasil!, token JWT aktif 24 jam diterima</t>
   </si>
   <si>
     <t>Reza Tri Wardana</t>
   </si>
   <si>
-    <t>2026-10-23_Hari-12_POST_1-Login_200-OK.png</t>
-  </si>
-  <si>
     <t>200 OK, user_id: 5, full_name: Ahmad Reza Fahmi, role: admin</t>
   </si>
   <si>
-    <t>2026-10-23_Hari-12_GET_2-Me_200-OK.png</t>
-  </si>
-  <si>
     <t>200 OK, total 18 aset berhasil ditarik lengkap dengan pagination limit 20</t>
   </si>
   <si>
-    <t>2026-10-23_Hari-12_GET_1-List-Assets_200-OK.png</t>
-  </si>
-  <si>
     <t>200 OK, total 118 insiden terekam, auto-incident #120 tercatat untuk IOT-ESP-01</t>
   </si>
   <si>
     <t>200 OK, total 79 notifikasi terekam, pagination limit 50, alert notif terverifikasi</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-AUTH-001_login-admin.png</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-AUTH-004_user-profile-me.png</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-ASSET-001_list-infrastruktur-assets.png</t>
+  </si>
+  <si>
+    <t>200 OK, total_devices: 18, statistik pemantauan aktif tervalidasi presisi</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-MON-005_dashboard-stats.png</t>
   </si>
 </sst>
 </file>
@@ -3001,7 +2974,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3152,9 +3125,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -3582,7 +3552,7 @@
         <v>23</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>854</v>
+        <v>841</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>75</v>
@@ -3591,10 +3561,10 @@
         <v>46318</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>850</v>
-      </c>
-      <c r="N2" s="58" t="s">
-        <v>855</v>
+        <v>839</v>
+      </c>
+      <c r="N2" s="37" t="s">
+        <v>846</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>24</v>
@@ -4680,19 +4650,19 @@
         <v>252</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>856</v>
+        <v>842</v>
       </c>
       <c r="K28" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L28" s="59">
+      <c r="L28" s="58">
         <v>46318</v>
       </c>
       <c r="M28" s="7" t="s">
-        <v>850</v>
-      </c>
-      <c r="N28" s="56" t="s">
-        <v>838</v>
+        <v>839</v>
+      </c>
+      <c r="N28" s="37" t="s">
+        <v>836</v>
       </c>
       <c r="O28" s="4" t="s">
         <v>24</v>
@@ -4731,17 +4701,10 @@
       <c r="I29" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="J29" s="4" t="s">
-        <v>839</v>
-      </c>
-      <c r="K29" s="4" t="s">
-        <v>75</v>
-      </c>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
-      <c r="N29" s="56" t="s">
-        <v>840</v>
-      </c>
       <c r="O29" s="4" t="s">
         <v>24</v>
       </c>
@@ -4779,17 +4742,10 @@
       <c r="I30" s="6" t="s">
         <v>620</v>
       </c>
-      <c r="J30" s="4" t="s">
-        <v>841</v>
-      </c>
-      <c r="K30" s="4" t="s">
-        <v>75</v>
-      </c>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
-      <c r="N30" s="56" t="s">
-        <v>842</v>
-      </c>
       <c r="O30" s="4" t="s">
         <v>24</v>
       </c>
@@ -4827,17 +4783,10 @@
       <c r="I31" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="J31" s="4" t="s">
-        <v>843</v>
-      </c>
-      <c r="K31" s="4" t="s">
-        <v>75</v>
-      </c>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
       <c r="L31" s="7"/>
       <c r="M31" s="7"/>
-      <c r="N31" s="56" t="s">
-        <v>844</v>
-      </c>
       <c r="O31" s="4" t="s">
         <v>24</v>
       </c>
@@ -4875,17 +4824,10 @@
       <c r="I32" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="J32" s="4" t="s">
-        <v>845</v>
-      </c>
-      <c r="K32" s="4" t="s">
-        <v>75</v>
-      </c>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
       <c r="L32" s="7"/>
       <c r="M32" s="7"/>
-      <c r="N32" s="56" t="s">
-        <v>846</v>
-      </c>
       <c r="O32" s="4" t="s">
         <v>24</v>
       </c>
@@ -4923,17 +4865,10 @@
       <c r="I33" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="J33" s="4" t="s">
-        <v>847</v>
-      </c>
-      <c r="K33" s="4" t="s">
-        <v>75</v>
-      </c>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
       <c r="L33" s="7"/>
       <c r="M33" s="7"/>
-      <c r="N33" s="56" t="s">
-        <v>848</v>
-      </c>
       <c r="O33" s="4" t="s">
         <v>24</v>
       </c>
@@ -5212,7 +5147,7 @@
         <v>263</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>849</v>
+        <v>838</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>75</v>
@@ -5221,10 +5156,10 @@
         <v>46318</v>
       </c>
       <c r="M40" s="4" t="s">
-        <v>850</v>
-      </c>
-      <c r="N40" s="56" t="s">
-        <v>851</v>
+        <v>839</v>
+      </c>
+      <c r="N40" s="37" t="s">
+        <v>844</v>
       </c>
       <c r="O40" s="4" t="s">
         <v>24</v>
@@ -5346,7 +5281,7 @@
         <v>273</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>852</v>
+        <v>840</v>
       </c>
       <c r="K43" s="4" t="s">
         <v>75</v>
@@ -5355,10 +5290,10 @@
         <v>46318</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>850</v>
-      </c>
-      <c r="N43" s="47" t="s">
-        <v>853</v>
+        <v>839</v>
+      </c>
+      <c r="N43" s="37" t="s">
+        <v>845</v>
       </c>
       <c r="O43" s="4" t="s">
         <v>24</v>
@@ -6020,15 +5955,19 @@
         <v>318</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>835</v>
+        <v>847</v>
       </c>
       <c r="K58" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="56" t="s">
-        <v>836</v>
+      <c r="L58" s="57">
+        <v>46318</v>
+      </c>
+      <c r="M58" s="4" t="s">
+        <v>839</v>
+      </c>
+      <c r="N58" s="37" t="s">
+        <v>848</v>
       </c>
       <c r="O58" s="4" t="s">
         <v>24</v>
@@ -6068,7 +6007,7 @@
         <v>323</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="K59" s="4" t="s">
         <v>75</v>
@@ -6276,7 +6215,7 @@
         <v>340</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>857</v>
+        <v>843</v>
       </c>
       <c r="K64" s="4" t="s">
         <v>75</v>
@@ -6285,10 +6224,10 @@
         <v>46318</v>
       </c>
       <c r="M64" s="4" t="s">
-        <v>850</v>
-      </c>
-      <c r="N64" s="56" t="s">
-        <v>844</v>
+        <v>839</v>
+      </c>
+      <c r="N64" s="37" t="s">
+        <v>837</v>
       </c>
       <c r="O64" s="4" t="s">
         <v>24</v>
@@ -7782,52 +7721,47 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="N43" r:id="rId1" xr:uid="{F1645194-E524-4B93-93C0-93775656DF38}"/>
-    <hyperlink ref="N45" r:id="rId2" tooltip="Bukti retest pass change-password" xr:uid="{83495BB2-4F28-4636-8350-D973F94E0902}"/>
-    <hyperlink ref="N46" r:id="rId3" tooltip="Bukti retest pass GET /users" xr:uid="{2A6474F4-7C4B-46EE-BFDD-FFE06AF40E86}"/>
-    <hyperlink ref="N51" r:id="rId4" tooltip="Bukti retest pass GET /users/1" xr:uid="{1D4D0B11-6BC6-4996-9878-75C18A64CB5A}"/>
-    <hyperlink ref="N76" r:id="rId5" tooltip="Bukti verifikasi pemisahan angka &amp; persen Donut Chart" xr:uid="{352E79BE-EA5E-416B-9A46-0975FC5478D9}"/>
-    <hyperlink ref="N77" r:id="rId6" tooltip="Bukti modal detail badge unknown amber" xr:uid="{29EBF0BA-A607-4A63-BA02-BD4E08334471}"/>
-    <hyperlink ref="N72" r:id="rId7" tooltip="Wireframe Desktop 1080p" xr:uid="{C5D30B54-7FD1-4625-80AF-A671A87A34CF}"/>
-    <hyperlink ref="N73" r:id="rId8" tooltip="Wireframe Tablet 768p" xr:uid="{BCF9F7C0-2A4A-40E9-82B6-7F9837E16225}"/>
-    <hyperlink ref="N74" r:id="rId9" tooltip="Wireframe Mobile 375p" xr:uid="{940DC609-433C-41F2-9018-441CF70ED274}"/>
-    <hyperlink ref="N75" r:id="rId10" tooltip="Wireframe RBAC Super Admin" xr:uid="{97835F1A-F840-4B49-B544-65C134EE20E7}"/>
-    <hyperlink ref="N78" r:id="rId11" tooltip="Wireframe Persistensi Settings" xr:uid="{D49569CC-A7E8-4FD1-9EEA-11943C68624C}"/>
-    <hyperlink ref="N79" r:id="rId12" tooltip="2026-10-20_Hari-9_dashboard_desktop-1080p.png" xr:uid="{C44BD706-1024-496D-BC2C-FEC5F2FDDBC4}"/>
-    <hyperlink ref="N80" r:id="rId13" tooltip="2026-10-20_Hari-9_dashboard_devices-table.png" xr:uid="{C4E76EE7-1F92-4D21-BE02-3C227961FFA8}"/>
-    <hyperlink ref="N81" r:id="rId14" tooltip="2026-10-20_Hari-9_dashboard_monitoring-live.png" xr:uid="{008D6612-6DA8-41AF-95FA-34960211B1D3}"/>
-    <hyperlink ref="N82" r:id="rId15" tooltip="2026-10-20_Hari-9_dashboard_location-gis.png" xr:uid="{114DF096-9EB4-45C7-A09A-1AF0A57EECAC}"/>
-    <hyperlink ref="N83" r:id="rId16" tooltip="2026-10-20_Hari-9_dashboard_alerts-incidents.png" xr:uid="{8287D95D-5C56-42D7-AE0D-0B12830ABA1F}"/>
-    <hyperlink ref="N84" r:id="rId17" tooltip="2026-10-20_Hari-9_dashboard_users-management.png" xr:uid="{A1CD8320-354E-4D47-A2C0-889080A5FE2D}"/>
-    <hyperlink ref="N85" r:id="rId18" tooltip="2026-10-20_Hari-9_dashboard_tablet-768p.png" xr:uid="{688E4F75-BC2A-4D87-8928-B390BB230019}"/>
-    <hyperlink ref="N86" r:id="rId19" tooltip="2026-10-20_Hari-9_dashboard_mobile-375p.png" xr:uid="{E56ED74B-D5E4-4FB8-A1EC-6EE6A17542CE}"/>
-    <hyperlink ref="N12" r:id="rId20" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA5214D5-F1E0-4AB5-8F33-130BA9BECE39}"/>
-    <hyperlink ref="N87" r:id="rId21" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA69F703-3295-4E68-83AE-6D1BD44B5B8D}"/>
-    <hyperlink ref="N88" r:id="rId22" tooltip="2026-10-21_Hari-10_final-dashboard_alerts-tickets.png" xr:uid="{4605776D-F959-42A0-8F71-F8599BA27AB1}"/>
-    <hyperlink ref="N89" r:id="rId23" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{D4C20B14-4E67-4FE8-B1D7-74877549AED3}"/>
-    <hyperlink ref="N90" r:id="rId24" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{AE154EBE-7DA7-4240-A572-D2F2DBD07D3E}"/>
-    <hyperlink ref="N91" r:id="rId25" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{FABA0045-223F-4258-9055-43736084C725}"/>
-    <hyperlink ref="N92" r:id="rId26" tooltip="2026-10-21_Hari-10_final-dashboard_desktop-1080p.png" xr:uid="{DF0874B5-F3A5-4940-B56E-5C8C97D816B7}"/>
-    <hyperlink ref="N93" r:id="rId27" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{B17C34F4-F7BE-42EA-851C-9107F4B20CCB}"/>
-    <hyperlink ref="N94" r:id="rId28" tooltip="2026-10-21_Hari-10_final-dashboard_users-rbac.png" xr:uid="{2241DBCB-8785-46FF-94D5-F6C6DED84A05}"/>
-    <hyperlink ref="N54" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-MON-001_icmp-ping.png" xr:uid="{8C32334C-50E2-461D-89AF-8EB45F63C7C7}"/>
-    <hyperlink ref="N55" r:id="rId30" tooltip="2026-10-22_Hari-11_TC-MON-002_http-health.png" xr:uid="{5D47D286-D7AE-4B03-A0A4-866AE4CEBB25}"/>
-    <hyperlink ref="N56" r:id="rId31" tooltip="2026-10-22_Hari-11_TC-MON-003_tcp-port-scan.png" xr:uid="{54A22B2F-0B75-42D5-8371-1C9E401985B0}"/>
-    <hyperlink ref="N57" r:id="rId32" tooltip="2026-10-22_Hari-11_TC-MON-004_latency-logs.png" xr:uid="{3B45532E-6326-4EFF-907E-9865FA5CE054}"/>
-    <hyperlink ref="N58" r:id="rId33" tooltip="2026-10-22_Hari-11_TC-MON-005_monitoring-summary.png" xr:uid="{C3BDC459-DA6D-4F63-83EB-830608126897}"/>
-    <hyperlink ref="N59" r:id="rId34" tooltip="2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png" xr:uid="{756D28A9-DCDF-427F-B5A7-F01AB6696F3F}"/>
-    <hyperlink ref="N28" r:id="rId35" xr:uid="{007CCACA-3220-4F7C-912C-66F1A0DC4260}"/>
-    <hyperlink ref="N29" r:id="rId36" tooltip="2026-10-23_Hari-12_TC-REC-001_auto-resolved-recovery.png" xr:uid="{DB45E82C-A556-4308-B54C-1019F073E6BD}"/>
-    <hyperlink ref="N30" r:id="rId37" tooltip="2026-10-23_Hari-12_TC-FAIL-001_offline-detection.png" xr:uid="{028E6BEF-3D80-4EAC-B73A-A23554BC740F}"/>
-    <hyperlink ref="N31" r:id="rId38" tooltip="2026-10-23_Hari-12_TC-NOTIF-001_alert-notification-trigger.png" xr:uid="{3D282DAD-DBA6-48CA-AB3F-2D3422710268}"/>
-    <hyperlink ref="N32" r:id="rId39" tooltip="2026-10-23_Hari-12_TC-HB-002_iot-heartbeat-recovery.png" xr:uid="{D3C4FE45-45EE-4B9C-B10E-CB4590A69183}"/>
-    <hyperlink ref="N33" r:id="rId40" tooltip="2026-10-23_Hari-12_TC-WARN-001_high-latency-warning.png" xr:uid="{5C311F97-1645-4AF3-BE81-26737B5A7616}"/>
-    <hyperlink ref="N40" r:id="rId41" xr:uid="{84DCE3CA-9396-4774-BABE-BA65D327F058}"/>
-    <hyperlink ref="N2" r:id="rId42" xr:uid="{38DE97AC-647E-4FAA-91DF-3E239D926B21}"/>
-    <hyperlink ref="N64" r:id="rId43" xr:uid="{4E8FCC19-840B-4A93-9C43-C6BBA664F2BB}"/>
+    <hyperlink ref="N45" r:id="rId1" tooltip="Bukti retest pass change-password" xr:uid="{83495BB2-4F28-4636-8350-D973F94E0902}"/>
+    <hyperlink ref="N46" r:id="rId2" tooltip="Bukti retest pass GET /users" xr:uid="{2A6474F4-7C4B-46EE-BFDD-FFE06AF40E86}"/>
+    <hyperlink ref="N51" r:id="rId3" tooltip="Bukti retest pass GET /users/1" xr:uid="{1D4D0B11-6BC6-4996-9878-75C18A64CB5A}"/>
+    <hyperlink ref="N76" r:id="rId4" tooltip="Bukti verifikasi pemisahan angka &amp; persen Donut Chart" xr:uid="{352E79BE-EA5E-416B-9A46-0975FC5478D9}"/>
+    <hyperlink ref="N77" r:id="rId5" tooltip="Bukti modal detail badge unknown amber" xr:uid="{29EBF0BA-A607-4A63-BA02-BD4E08334471}"/>
+    <hyperlink ref="N72" r:id="rId6" tooltip="Wireframe Desktop 1080p" xr:uid="{C5D30B54-7FD1-4625-80AF-A671A87A34CF}"/>
+    <hyperlink ref="N73" r:id="rId7" tooltip="Wireframe Tablet 768p" xr:uid="{BCF9F7C0-2A4A-40E9-82B6-7F9837E16225}"/>
+    <hyperlink ref="N74" r:id="rId8" tooltip="Wireframe Mobile 375p" xr:uid="{940DC609-433C-41F2-9018-441CF70ED274}"/>
+    <hyperlink ref="N75" r:id="rId9" tooltip="Wireframe RBAC Super Admin" xr:uid="{97835F1A-F840-4B49-B544-65C134EE20E7}"/>
+    <hyperlink ref="N78" r:id="rId10" tooltip="Wireframe Persistensi Settings" xr:uid="{D49569CC-A7E8-4FD1-9EEA-11943C68624C}"/>
+    <hyperlink ref="N79" r:id="rId11" tooltip="2026-10-20_Hari-9_dashboard_desktop-1080p.png" xr:uid="{C44BD706-1024-496D-BC2C-FEC5F2FDDBC4}"/>
+    <hyperlink ref="N80" r:id="rId12" tooltip="2026-10-20_Hari-9_dashboard_devices-table.png" xr:uid="{C4E76EE7-1F92-4D21-BE02-3C227961FFA8}"/>
+    <hyperlink ref="N81" r:id="rId13" tooltip="2026-10-20_Hari-9_dashboard_monitoring-live.png" xr:uid="{008D6612-6DA8-41AF-95FA-34960211B1D3}"/>
+    <hyperlink ref="N82" r:id="rId14" tooltip="2026-10-20_Hari-9_dashboard_location-gis.png" xr:uid="{114DF096-9EB4-45C7-A09A-1AF0A57EECAC}"/>
+    <hyperlink ref="N83" r:id="rId15" tooltip="2026-10-20_Hari-9_dashboard_alerts-incidents.png" xr:uid="{8287D95D-5C56-42D7-AE0D-0B12830ABA1F}"/>
+    <hyperlink ref="N84" r:id="rId16" tooltip="2026-10-20_Hari-9_dashboard_users-management.png" xr:uid="{A1CD8320-354E-4D47-A2C0-889080A5FE2D}"/>
+    <hyperlink ref="N85" r:id="rId17" tooltip="2026-10-20_Hari-9_dashboard_tablet-768p.png" xr:uid="{688E4F75-BC2A-4D87-8928-B390BB230019}"/>
+    <hyperlink ref="N86" r:id="rId18" tooltip="2026-10-20_Hari-9_dashboard_mobile-375p.png" xr:uid="{E56ED74B-D5E4-4FB8-A1EC-6EE6A17542CE}"/>
+    <hyperlink ref="N12" r:id="rId19" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA5214D5-F1E0-4AB5-8F33-130BA9BECE39}"/>
+    <hyperlink ref="N87" r:id="rId20" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA69F703-3295-4E68-83AE-6D1BD44B5B8D}"/>
+    <hyperlink ref="N88" r:id="rId21" tooltip="2026-10-21_Hari-10_final-dashboard_alerts-tickets.png" xr:uid="{4605776D-F959-42A0-8F71-F8599BA27AB1}"/>
+    <hyperlink ref="N89" r:id="rId22" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{D4C20B14-4E67-4FE8-B1D7-74877549AED3}"/>
+    <hyperlink ref="N90" r:id="rId23" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{AE154EBE-7DA7-4240-A572-D2F2DBD07D3E}"/>
+    <hyperlink ref="N91" r:id="rId24" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{FABA0045-223F-4258-9055-43736084C725}"/>
+    <hyperlink ref="N92" r:id="rId25" tooltip="2026-10-21_Hari-10_final-dashboard_desktop-1080p.png" xr:uid="{DF0874B5-F3A5-4940-B56E-5C8C97D816B7}"/>
+    <hyperlink ref="N93" r:id="rId26" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{B17C34F4-F7BE-42EA-851C-9107F4B20CCB}"/>
+    <hyperlink ref="N94" r:id="rId27" tooltip="2026-10-21_Hari-10_final-dashboard_users-rbac.png" xr:uid="{2241DBCB-8785-46FF-94D5-F6C6DED84A05}"/>
+    <hyperlink ref="N54" r:id="rId28" tooltip="2026-10-22_Hari-11_TC-MON-001_icmp-ping.png" xr:uid="{8C32334C-50E2-461D-89AF-8EB45F63C7C7}"/>
+    <hyperlink ref="N55" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-MON-002_http-health.png" xr:uid="{5D47D286-D7AE-4B03-A0A4-866AE4CEBB25}"/>
+    <hyperlink ref="N56" r:id="rId30" tooltip="2026-10-22_Hari-11_TC-MON-003_tcp-port-scan.png" xr:uid="{54A22B2F-0B75-42D5-8371-1C9E401985B0}"/>
+    <hyperlink ref="N57" r:id="rId31" tooltip="2026-10-22_Hari-11_TC-MON-004_latency-logs.png" xr:uid="{3B45532E-6326-4EFF-907E-9865FA5CE054}"/>
+    <hyperlink ref="N59" r:id="rId32" tooltip="2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png" xr:uid="{756D28A9-DCDF-427F-B5A7-F01AB6696F3F}"/>
+    <hyperlink ref="N40" r:id="rId33" xr:uid="{A3C2BAA6-CBF3-4397-B41D-5A324045423D}"/>
+    <hyperlink ref="N43" r:id="rId34" xr:uid="{07F98721-DFA0-4CCD-906D-1564D3193455}"/>
+    <hyperlink ref="N2" r:id="rId35" xr:uid="{D09C9E3E-C97E-481F-A9D5-438C5725DB68}"/>
+    <hyperlink ref="N58" r:id="rId36" xr:uid="{E0B53A3F-B5C3-43B7-A2D4-E0601746F4FD}"/>
+    <hyperlink ref="N28" r:id="rId37" xr:uid="{2A9B3EBA-EB8F-4B77-9B6F-B5485EC42B5D}"/>
+    <hyperlink ref="N64" r:id="rId38" xr:uid="{55A145A2-869F-426A-A996-3D1E4599B081}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId44"/>
+  <pageSetup orientation="portrait" r:id="rId39"/>
 </worksheet>
 </file>
 
@@ -8176,19 +8110,19 @@
       <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="60" t="s">
+      <c r="A13" s="59" t="s">
         <v>586</v>
       </c>
-      <c r="B13" s="60"/>
-      <c r="C13" s="60"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="59"/>
       <c r="M13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="60" t="s">
+      <c r="A14" s="59" t="s">
         <v>587</v>
       </c>
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
+      <c r="B14" s="59"/>
+      <c r="C14" s="59"/>
       <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat(qa): release day-13 asset verification, iot heartbeat fallback, and pre-deploy audit deliverables
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\TAIMS_REMOTE_CHECK\docs\qa-testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\docs\qa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11FEC61-2AF6-4AB4-B1DF-98A63920229A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E068549-CA26-4798-A0F9-323449E3512F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="220" windowWidth="14400" windowHeight="7810" firstSheet="2" activeTab="4" xr2:uid="{D20540B9-5A4B-4C0F-A1AA-6997D01BA992}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1697" uniqueCount="849">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="886">
   <si>
     <t>TC ID</t>
   </si>
@@ -1441,6 +1441,9 @@
     <t>Test di Postman, backend jalan</t>
   </si>
   <si>
+    <t>200 OK, token didapat</t>
+  </si>
+  <si>
     <t>404 Endpoint belum 
 diimplementasi</t>
   </si>
@@ -1601,6 +1604,10 @@
     <t>Aset bertambah dari 16 menjadi 17, sistem normal</t>
   </si>
   <si>
+    <t>200 OK, data 17 aset tampil 
+di database</t>
+  </si>
+  <si>
     <t>Backend jalan, Postman 
 siap</t>
   </si>
@@ -2684,9 +2691,6 @@
     <t>screenshots/Hari-10/2026-10-21_Hari-10_final-dashboard_users-rbac.png</t>
   </si>
   <si>
-    <t>2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png</t>
-  </si>
-  <si>
     <t>201 Created, log_id disimpan, ICMP ping latency 2ms, 0% packet loss, status online</t>
   </si>
   <si>
@@ -2711,46 +2715,154 @@
     <t>2026-10-22_Hari-11_TC-MON-004_latency-logs.png</t>
   </si>
   <si>
+    <t>200 OK, summary data 17 unit online across 10 kategori tervalidasi presisi, latency 17ms</t>
+  </si>
+  <si>
+    <t>2026-10-22_Hari-11_TC-MON-005_monitoring-summary.png</t>
+  </si>
+  <si>
     <t>200 OK, message: Heartbeat received, status online, RSSI -58 dBm, Response Time 33ms</t>
   </si>
   <si>
+    <t>Status beralih ke offline, background checker mendeteksi timeout 45s, tiket insiden otomatis terbentuk, alert terkirim</t>
+  </si>
+  <si>
     <t>2026-10-23_Hari-12_TC-INC-001_auto-incident-generated.png</t>
   </si>
   <si>
+    <t>Status kembali online saat paket ping baru masuk, tiket insiden otomatis berubah menjadi resolved (Auto-Recovery)</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-REC-001_auto-resolved-recovery.png</t>
+  </si>
+  <si>
+    <t>Status offline terekam, incident type Device Offline, severity high, tiket insiden #99 open tervalidasi via API</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-FAIL-001_offline-detection.png</t>
+  </si>
+  <si>
+    <t>Status offline terverifikasi, last_seen stop dihentikan saat sinyal telemetri terputus, notifikasi terkirim</t>
+  </si>
+  <si>
     <t>2026-10-23_Hari-12_TC-NOTIF-001_alert-notification-trigger.png</t>
   </si>
   <si>
-    <t>200 OK, message: Login berhasil!, token JWT aktif 24 jam diterima</t>
-  </si>
-  <si>
-    <t>Reza Tri Wardana</t>
-  </si>
-  <si>
-    <t>200 OK, user_id: 5, full_name: Ahmad Reza Fahmi, role: admin</t>
-  </si>
-  <si>
-    <t>200 OK, total 18 aset berhasil ditarik lengkap dengan pagination limit 20</t>
-  </si>
-  <si>
-    <t>200 OK, total 118 insiden terekam, auto-incident #120 tercatat untuk IOT-ESP-01</t>
-  </si>
-  <si>
-    <t>200 OK, total 79 notifikasi terekam, pagination limit 50, alert notif terverifikasi</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-AUTH-001_login-admin.png</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-AUTH-004_user-profile-me.png</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-ASSET-001_list-infrastruktur-assets.png</t>
-  </si>
-  <si>
-    <t>200 OK, total_devices: 18, statistik pemantauan aktif tervalidasi presisi</t>
-  </si>
-  <si>
-    <t>2026-10-23_Hari-12_TC-MON-005_dashboard-stats.png</t>
+    <t>Status sensor terputus tervalidasi, paket heartbeat timeout memicu alert, rekoneksi sukses menerima 200 OK (98ms)</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-HB-002_iot-heartbeat-recovery.png</t>
+  </si>
+  <si>
+    <t>Injeksi latensi tinggi &gt; 1000ms (1450ms) dan loss 15% memicu transisi status WARNING pada log dan dashboard</t>
+  </si>
+  <si>
+    <t>2026-10-23_Hari-12_TC-WARN-001_high-latency-warning.png</t>
+  </si>
+  <si>
+    <t>200 OK, Router MikroTik MKRT-01 (192.168.1.2) terdaftar di database, status online</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-001_mikrotik-router-inventory.png</t>
+  </si>
+  <si>
+    <t>200 OK, Switch Manageable SWM-01 (192.168.3.1) terdaftar, port 80/443 aktif</t>
+  </si>
+  <si>
+    <t>200 OK, Access Point UniFi &amp; CCTV-01 (192.168.1.39) terdaftar, status offline</t>
+  </si>
+  <si>
+    <t>200 OK, Server Utama SRV-01 (192.168.3.15) terdaftar, service backend aktif</t>
+  </si>
+  <si>
+    <t>200 OK, Raspberry Pi RPI-01 &amp; RPI-02 (192.168.1.12 &amp; 3.16) terdaftar sebagai IoT Gateway</t>
+  </si>
+  <si>
+    <t>200 OK, Web Service &amp; Website T-AIMS terdaftar, HTTP health check 200 OK</t>
+  </si>
+  <si>
+    <t>200 OK, IoT Node ESP-01 (192.168.0.105) terdaftar, firmware v1.4.2 tervalidasi</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-014_esp32-mqtt-telemetry-config.png</t>
+  </si>
+  <si>
+    <t>200 OK, MQTT Broker Service terdaftar, channel telemetri aktif di port 1883</t>
+  </si>
+  <si>
+    <t>200 OK, PC Head Office 01 (PC-01, 192.168.1.2) terdaftar dan online</t>
+  </si>
+  <si>
+    <t>200 OK, Filter kategori Router berhasil menyaring 8 unit perangkat presisi</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-010_filter-category-router.png</t>
+  </si>
+  <si>
+    <t>200 OK, Filter kategori IoT Node berhasil menyaring node sensor ESP32 presisi</t>
+  </si>
+  <si>
+    <t>200 OK, Filter lokasi Head Office menyaring seluruh aset lab &amp; kantor presisi</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-012_filter-location-headoffice.png</t>
+  </si>
+  <si>
+    <t>200 OK, Alamat IP MikroTik 192.168.1.1 &amp; 1.2 tervalidasi aktif pada subnet LAN</t>
+  </si>
+  <si>
+    <t>200 OK, Topic MQTT taims/heartbeat/ESP-01 dan timeout 90s terkonfigurasi di DB</t>
+  </si>
+  <si>
+    <t>200 OK, Aset prioritas kritis = 1 (Router Core &amp; Switch) terverifikasi di level high</t>
+  </si>
+  <si>
+    <t>401 Unauthorized / Bad Request: Penolakan aman terhadap device_id tidak terdaftar</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-HB-002_unregistered-device-rejection.png</t>
+  </si>
+  <si>
+    <t>200 OK, Payload telemetri heartbeat terakhir ESP-01 berhasil ditarik dengan Bearer token</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-002_cisco-switch-inventory.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-003_unifi-cctv-inventory.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-004_ubuntu-server-inventory.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-005_raspberry-pi-gateway.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-006_website-service-online.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-007_esp32-node-detail.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-008_mqtt-broker-telemetry.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-009_pc-headoffice-inventory.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-011_filter-category-iotnode.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-013_mikrotik-ip-verification.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-ASSET-015_priority-1-critical-assets.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-HB-001_iot-heartbeat-telemetry.png</t>
+  </si>
+  <si>
+    <t>2026-10-24_Hari-13_TC-HB-003_latest-iot-heartbeat-denah.png</t>
   </si>
 </sst>
 </file>
@@ -2974,7 +3086,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3124,10 +3236,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -3543,7 +3651,7 @@
         <v>21</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>22</v>
@@ -3552,20 +3660,16 @@
         <v>23</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>841</v>
+        <v>478</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L2" s="57">
-        <v>46318</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>839</v>
-      </c>
-      <c r="N2" s="37" t="s">
-        <v>846</v>
-      </c>
+      <c r="L2" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
       <c r="O2" s="4" t="s">
         <v>24</v>
       </c>
@@ -3574,7 +3678,7 @@
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3602,7 +3706,7 @@
         <v>48</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>75</v>
@@ -3643,14 +3747,14 @@
         <v>21</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>75</v>
@@ -3692,7 +3796,7 @@
         <v>50</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>75</v>
@@ -3734,7 +3838,7 @@
         <v>51</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>75</v>
@@ -3776,7 +3880,7 @@
         <v>52</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>75</v>
@@ -3790,7 +3894,7 @@
         <v>24</v>
       </c>
       <c r="P7" s="20" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
@@ -3820,7 +3924,7 @@
         <v>53</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>75</v>
@@ -3862,7 +3966,7 @@
         <v>50</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>75</v>
@@ -3904,7 +4008,7 @@
         <v>54</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>75</v>
@@ -3943,10 +4047,10 @@
         <v>47</v>
       </c>
       <c r="G11" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>433</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>432</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>55</v>
@@ -3970,7 +4074,7 @@
       </c>
       <c r="Q11" s="7"/>
       <c r="R11" s="6" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -3998,7 +4102,7 @@
         <v>55</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>75</v>
@@ -4008,7 +4112,7 @@
       </c>
       <c r="M12" s="7"/>
       <c r="N12" s="48" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="O12" s="14" t="s">
         <v>24</v>
@@ -4018,7 +4122,7 @@
       </c>
       <c r="Q12" s="7"/>
       <c r="R12" s="8" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -4041,7 +4145,7 @@
         <v>21</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>226</v>
@@ -4049,15 +4153,23 @@
       <c r="I13" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
+      <c r="J13" s="4" t="s">
+        <v>851</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
+      <c r="N13" s="37" t="s">
+        <v>852</v>
+      </c>
       <c r="O13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P13" s="5"/>
+      <c r="P13" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
     </row>
@@ -4089,15 +4201,23 @@
       <c r="I14" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="J14" s="4" t="s">
+        <v>853</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
+      <c r="N14" s="37" t="s">
+        <v>873</v>
+      </c>
       <c r="O14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P14" s="5"/>
+      <c r="P14" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
     </row>
@@ -4127,17 +4247,25 @@
         <v>228</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>615</v>
-      </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+        <v>617</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>854</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
+      <c r="N15" s="37" t="s">
+        <v>874</v>
+      </c>
       <c r="O15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P15" s="5"/>
+      <c r="P15" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q15" s="7"/>
       <c r="R15" s="7"/>
     </row>
@@ -4169,19 +4297,27 @@
       <c r="I16" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="J16" s="4" t="s">
+        <v>855</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L16" s="7"/>
       <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
+      <c r="N16" s="37" t="s">
+        <v>875</v>
+      </c>
       <c r="O16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P16" s="5"/>
+      <c r="P16" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
     </row>
-    <row r="17" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>175</v>
       </c>
@@ -4209,15 +4345,23 @@
       <c r="I17" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
+      <c r="J17" s="4" t="s">
+        <v>856</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L17" s="7"/>
       <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
+      <c r="N17" s="37" t="s">
+        <v>876</v>
+      </c>
       <c r="O17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P17" s="5"/>
+      <c r="P17" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
     </row>
@@ -4249,15 +4393,23 @@
       <c r="I18" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="J18" s="4" t="s">
+        <v>857</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
+      <c r="N18" s="37" t="s">
+        <v>877</v>
+      </c>
       <c r="O18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P18" s="5"/>
+      <c r="P18" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
     </row>
@@ -4289,15 +4441,23 @@
       <c r="I19" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
+      <c r="J19" s="4" t="s">
+        <v>858</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L19" s="7"/>
       <c r="M19" s="7"/>
-      <c r="N19" s="7"/>
+      <c r="N19" s="37" t="s">
+        <v>878</v>
+      </c>
       <c r="O19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P19" s="5"/>
+      <c r="P19" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q19" s="7"/>
       <c r="R19" s="7"/>
     </row>
@@ -4327,17 +4487,25 @@
         <v>417</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>616</v>
-      </c>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
+        <v>618</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>860</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L20" s="7"/>
       <c r="M20" s="7"/>
-      <c r="N20" s="7"/>
+      <c r="N20" s="37" t="s">
+        <v>879</v>
+      </c>
       <c r="O20" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P20" s="5"/>
+      <c r="P20" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q20" s="7"/>
       <c r="R20" s="7"/>
     </row>
@@ -4367,17 +4535,25 @@
         <v>231</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>617</v>
-      </c>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
+        <v>619</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>861</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L21" s="7"/>
       <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
+      <c r="N21" s="37" t="s">
+        <v>880</v>
+      </c>
       <c r="O21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P21" s="5"/>
+      <c r="P21" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q21" s="7"/>
       <c r="R21" s="7"/>
     </row>
@@ -4409,15 +4585,23 @@
       <c r="I22" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+      <c r="J22" s="4" t="s">
+        <v>862</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L22" s="7"/>
       <c r="M22" s="7"/>
-      <c r="N22" s="7"/>
+      <c r="N22" s="37" t="s">
+        <v>863</v>
+      </c>
       <c r="O22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P22" s="5"/>
+      <c r="P22" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q22" s="7"/>
       <c r="R22" s="7"/>
     </row>
@@ -4447,17 +4631,25 @@
         <v>233</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>618</v>
-      </c>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
+        <v>620</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L23" s="7"/>
       <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
+      <c r="N23" s="37" t="s">
+        <v>881</v>
+      </c>
       <c r="O23" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P23" s="5"/>
+      <c r="P23" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
     </row>
@@ -4489,15 +4681,23 @@
       <c r="I24" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
+      <c r="J24" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L24" s="7"/>
       <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
+      <c r="N24" s="37" t="s">
+        <v>866</v>
+      </c>
       <c r="O24" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P24" s="5"/>
+      <c r="P24" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
     </row>
@@ -4529,15 +4729,23 @@
       <c r="I25" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
+      <c r="J25" s="4" t="s">
+        <v>867</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
-      <c r="N25" s="7"/>
+      <c r="N25" s="37" t="s">
+        <v>882</v>
+      </c>
       <c r="O25" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P25" s="5"/>
+      <c r="P25" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q25" s="7"/>
       <c r="R25" s="7"/>
     </row>
@@ -4567,17 +4775,25 @@
         <v>236</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>619</v>
-      </c>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
+        <v>621</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>868</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L26" s="7"/>
       <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
+      <c r="N26" s="37" t="s">
+        <v>859</v>
+      </c>
       <c r="O26" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P26" s="5"/>
+      <c r="P26" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q26" s="7"/>
       <c r="R26" s="7"/>
     </row>
@@ -4609,15 +4825,23 @@
       <c r="I27" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
+      <c r="J27" s="4" t="s">
+        <v>869</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L27" s="7"/>
       <c r="M27" s="7"/>
-      <c r="N27" s="7"/>
+      <c r="N27" s="37" t="s">
+        <v>883</v>
+      </c>
       <c r="O27" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P27" s="5"/>
+      <c r="P27" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q27" s="7"/>
       <c r="R27" s="7"/>
     </row>
@@ -4650,19 +4874,15 @@
         <v>252</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="K28" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L28" s="58">
-        <v>46318</v>
-      </c>
-      <c r="M28" s="7" t="s">
-        <v>839</v>
-      </c>
-      <c r="N28" s="37" t="s">
-        <v>836</v>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="56" t="s">
+        <v>840</v>
       </c>
       <c r="O28" s="4" t="s">
         <v>24</v>
@@ -4701,10 +4921,17 @@
       <c r="I29" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
+      <c r="J29" s="4" t="s">
+        <v>841</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
+      <c r="N29" s="56" t="s">
+        <v>842</v>
+      </c>
       <c r="O29" s="4" t="s">
         <v>24</v>
       </c>
@@ -4740,12 +4967,19 @@
         <v>240</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>620</v>
-      </c>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
+        <v>622</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
+      <c r="N30" s="56" t="s">
+        <v>844</v>
+      </c>
       <c r="O30" s="4" t="s">
         <v>24</v>
       </c>
@@ -4783,10 +5017,17 @@
       <c r="I31" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
+      <c r="J31" s="4" t="s">
+        <v>845</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L31" s="7"/>
       <c r="M31" s="7"/>
+      <c r="N31" s="56" t="s">
+        <v>846</v>
+      </c>
       <c r="O31" s="4" t="s">
         <v>24</v>
       </c>
@@ -4822,12 +5063,19 @@
         <v>242</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>623</v>
-      </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
+        <v>625</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>847</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L32" s="7"/>
       <c r="M32" s="7"/>
+      <c r="N32" s="56" t="s">
+        <v>848</v>
+      </c>
       <c r="O32" s="4" t="s">
         <v>24</v>
       </c>
@@ -4865,10 +5113,17 @@
       <c r="I33" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
+      <c r="J33" s="4" t="s">
+        <v>849</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L33" s="7"/>
       <c r="M33" s="7"/>
+      <c r="N33" s="56" t="s">
+        <v>850</v>
+      </c>
       <c r="O33" s="4" t="s">
         <v>24</v>
       </c>
@@ -5064,7 +5319,7 @@
         <v>223</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -5104,7 +5359,7 @@
         <v>247</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -5147,20 +5402,14 @@
         <v>263</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>838</v>
+        <v>429</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L40" s="57">
-        <v>46318</v>
-      </c>
-      <c r="M40" s="4" t="s">
-        <v>839</v>
-      </c>
-      <c r="N40" s="37" t="s">
-        <v>844</v>
-      </c>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="7"/>
       <c r="O40" s="4" t="s">
         <v>24</v>
       </c>
@@ -5280,20 +5529,16 @@
       <c r="I43" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="J43" s="4" t="s">
-        <v>840</v>
-      </c>
-      <c r="K43" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="L43" s="57">
-        <v>46318</v>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4" t="s">
+        <v>70</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>839</v>
-      </c>
-      <c r="N43" s="37" t="s">
-        <v>845</v>
+        <v>440</v>
+      </c>
+      <c r="N43" s="45" t="s">
+        <v>594</v>
       </c>
       <c r="O43" s="4" t="s">
         <v>24</v>
@@ -5371,7 +5616,7 @@
         <v>280</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K45" s="4" t="s">
         <v>76</v>
@@ -5383,7 +5628,7 @@
         <v>67</v>
       </c>
       <c r="N45" s="45" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="O45" s="4" t="s">
         <v>24</v>
@@ -5428,10 +5673,10 @@
         <v>70</v>
       </c>
       <c r="M46" s="4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="N46" s="45" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="O46" s="4" t="s">
         <v>24</v>
@@ -5602,7 +5847,7 @@
     </row>
     <row r="51" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B51" s="13">
         <v>16</v>
@@ -5611,7 +5856,7 @@
         <v>282</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>20</v>
@@ -5620,16 +5865,16 @@
         <v>21</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K51" s="4" t="s">
         <v>75</v>
@@ -5641,7 +5886,7 @@
         <v>69</v>
       </c>
       <c r="N51" s="45" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="O51" s="4" t="s">
         <v>24</v>
@@ -5651,7 +5896,7 @@
       </c>
       <c r="Q51" s="7"/>
       <c r="R51" s="4" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="52" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -5763,7 +6008,7 @@
         <v>308</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="K54" s="4" t="s">
         <v>75</v>
@@ -5771,7 +6016,7 @@
       <c r="L54" s="4"/>
       <c r="M54" s="4"/>
       <c r="N54" s="56" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="O54" s="4" t="s">
         <v>24</v>
@@ -5811,7 +6056,7 @@
         <v>308</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="K55" s="4" t="s">
         <v>75</v>
@@ -5819,7 +6064,7 @@
       <c r="L55" s="4"/>
       <c r="M55" s="4"/>
       <c r="N55" s="56" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="O55" s="4" t="s">
         <v>24</v>
@@ -5859,7 +6104,7 @@
         <v>308</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="K56" s="4" t="s">
         <v>75</v>
@@ -5867,7 +6112,7 @@
       <c r="L56" s="4"/>
       <c r="M56" s="4"/>
       <c r="N56" s="56" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="O56" s="4" t="s">
         <v>24</v>
@@ -5907,7 +6152,7 @@
         <v>315</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="K57" s="4" t="s">
         <v>75</v>
@@ -5915,7 +6160,7 @@
       <c r="L57" s="4"/>
       <c r="M57" s="4"/>
       <c r="N57" s="56" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="O57" s="4" t="s">
         <v>24</v>
@@ -5955,19 +6200,15 @@
         <v>318</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>847</v>
+        <v>836</v>
       </c>
       <c r="K58" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L58" s="57">
-        <v>46318</v>
-      </c>
-      <c r="M58" s="4" t="s">
-        <v>839</v>
-      </c>
-      <c r="N58" s="37" t="s">
-        <v>848</v>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="56" t="s">
+        <v>837</v>
       </c>
       <c r="O58" s="4" t="s">
         <v>24</v>
@@ -6007,7 +6248,7 @@
         <v>323</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="K59" s="4" t="s">
         <v>75</v>
@@ -6015,13 +6256,13 @@
       <c r="L59" s="4"/>
       <c r="M59" s="4"/>
       <c r="N59" s="37" t="s">
-        <v>826</v>
+        <v>884</v>
       </c>
       <c r="O59" s="4" t="s">
         <v>24</v>
       </c>
       <c r="P59" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="Q59" s="7"/>
       <c r="R59" s="7"/>
@@ -6054,15 +6295,23 @@
       <c r="I60" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
+      <c r="J60" s="4" t="s">
+        <v>870</v>
+      </c>
+      <c r="K60" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L60" s="4"/>
       <c r="M60" s="4"/>
-      <c r="N60" s="7"/>
+      <c r="N60" s="37" t="s">
+        <v>871</v>
+      </c>
       <c r="O60" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P60" s="5"/>
+      <c r="P60" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q60" s="7"/>
       <c r="R60" s="7"/>
     </row>
@@ -6094,15 +6343,23 @@
       <c r="I61" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
+      <c r="J61" s="4" t="s">
+        <v>872</v>
+      </c>
+      <c r="K61" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="L61" s="4"/>
       <c r="M61" s="4"/>
-      <c r="N61" s="7"/>
+      <c r="N61" s="37" t="s">
+        <v>885</v>
+      </c>
       <c r="O61" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="P61" s="5"/>
+      <c r="P61" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="Q61" s="7"/>
       <c r="R61" s="7"/>
     </row>
@@ -6214,21 +6471,11 @@
       <c r="I64" s="4" t="s">
         <v>340</v>
       </c>
-      <c r="J64" s="4" t="s">
-        <v>843</v>
-      </c>
-      <c r="K64" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="L64" s="57">
-        <v>46318</v>
-      </c>
-      <c r="M64" s="4" t="s">
-        <v>839</v>
-      </c>
-      <c r="N64" s="37" t="s">
-        <v>837</v>
-      </c>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="4"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="7"/>
       <c r="O64" s="4" t="s">
         <v>24</v>
       </c>
@@ -6345,7 +6592,7 @@
         <v>349</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="K67" s="4" t="s">
         <v>75</v>
@@ -6359,7 +6606,7 @@
       <c r="P67" s="5"/>
       <c r="Q67" s="7"/>
       <c r="R67" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="68" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -6471,7 +6718,7 @@
         <v>358</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="K70" s="4" t="s">
         <v>75</v>
@@ -6530,16 +6777,16 @@
     </row>
     <row r="72" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B72" s="10">
         <v>8</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>20</v>
@@ -6548,16 +6795,16 @@
         <v>21</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="K72" s="36" t="s">
         <v>75</v>
@@ -6565,7 +6812,7 @@
       <c r="L72" s="10"/>
       <c r="M72" s="10"/>
       <c r="N72" s="45" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="O72" s="4" t="s">
         <v>24</v>
@@ -6575,21 +6822,21 @@
       </c>
       <c r="Q72" s="4"/>
       <c r="R72" s="6" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="73" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B73" s="10">
         <v>8</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>20</v>
@@ -6598,16 +6845,16 @@
         <v>47</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="K73" s="36" t="s">
         <v>75</v>
@@ -6615,7 +6862,7 @@
       <c r="L73" s="10"/>
       <c r="M73" s="10"/>
       <c r="N73" s="45" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="O73" s="4" t="s">
         <v>24</v>
@@ -6625,21 +6872,21 @@
       </c>
       <c r="Q73" s="4"/>
       <c r="R73" s="6" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="74" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B74" s="10">
         <v>8</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>20</v>
@@ -6648,16 +6895,16 @@
         <v>47</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="K74" s="36" t="s">
         <v>75</v>
@@ -6665,7 +6912,7 @@
       <c r="L74" s="10"/>
       <c r="M74" s="10"/>
       <c r="N74" s="45" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="O74" s="4" t="s">
         <v>24</v>
@@ -6675,21 +6922,21 @@
       </c>
       <c r="Q74" s="4"/>
       <c r="R74" s="6" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="75" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B75" s="10">
         <v>8</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>46</v>
@@ -6698,16 +6945,16 @@
         <v>21</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="K75" s="36" t="s">
         <v>75</v>
@@ -6715,7 +6962,7 @@
       <c r="L75" s="10"/>
       <c r="M75" s="10"/>
       <c r="N75" s="45" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="O75" s="4" t="s">
         <v>24</v>
@@ -6725,21 +6972,21 @@
       </c>
       <c r="Q75" s="4"/>
       <c r="R75" s="6" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="76" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B76" s="10">
         <v>8</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>20</v>
@@ -6748,16 +6995,16 @@
         <v>47</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="K76" s="36" t="s">
         <v>75</v>
@@ -6766,10 +7013,10 @@
         <v>420</v>
       </c>
       <c r="M76" s="10" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="N76" s="45" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="O76" s="4" t="s">
         <v>24</v>
@@ -6779,21 +7026,21 @@
       </c>
       <c r="Q76" s="4"/>
       <c r="R76" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="77" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B77" s="10">
         <v>8</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="E77" s="4" t="s">
         <v>20</v>
@@ -6802,28 +7049,28 @@
         <v>21</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="J77" s="6" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="K77" s="36" t="s">
         <v>75</v>
       </c>
       <c r="L77" s="10" t="s">
+        <v>494</v>
+      </c>
+      <c r="M77" s="10" t="s">
         <v>492</v>
       </c>
-      <c r="M77" s="10" t="s">
-        <v>490</v>
-      </c>
       <c r="N77" s="45" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="O77" s="4" t="s">
         <v>24</v>
@@ -6833,21 +7080,21 @@
       </c>
       <c r="Q77" s="4"/>
       <c r="R77" s="6" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="78" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="B78" s="10">
         <v>8</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>20</v>
@@ -6856,16 +7103,16 @@
         <v>47</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="I78" s="6" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="J78" s="6" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="K78" s="36" t="s">
         <v>75</v>
@@ -6873,7 +7120,7 @@
       <c r="L78" s="10"/>
       <c r="M78" s="10"/>
       <c r="N78" s="45" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="O78" s="4" t="s">
         <v>24</v>
@@ -6883,39 +7130,39 @@
       </c>
       <c r="Q78" s="4"/>
       <c r="R78" s="6" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="79" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B79" s="6">
         <v>9</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="F79" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G79" s="6" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="J79" s="6" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="K79" s="46" t="s">
         <v>75</v>
@@ -6923,7 +7170,7 @@
       <c r="L79" s="8"/>
       <c r="M79" s="8"/>
       <c r="N79" s="47" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="O79" s="6" t="s">
         <v>24</v>
@@ -6932,42 +7179,42 @@
         <v>104</v>
       </c>
       <c r="Q79" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R79" s="6" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="80" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="B80" s="6">
         <v>9</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="J80" s="6" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="K80" s="46" t="s">
         <v>75</v>
@@ -6975,7 +7222,7 @@
       <c r="L80" s="8"/>
       <c r="M80" s="8"/>
       <c r="N80" s="47" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>24</v>
@@ -6984,42 +7231,42 @@
         <v>104</v>
       </c>
       <c r="Q80" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R80" s="6" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="81" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B81" s="6">
         <v>9</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F81" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G81" s="6" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="J81" s="6" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="K81" s="46" t="s">
         <v>75</v>
@@ -7027,7 +7274,7 @@
       <c r="L81" s="8"/>
       <c r="M81" s="8"/>
       <c r="N81" s="47" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="O81" s="6" t="s">
         <v>24</v>
@@ -7036,42 +7283,42 @@
         <v>104</v>
       </c>
       <c r="Q81" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R81" s="6" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="82" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A82" s="6" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B82" s="6">
         <v>9</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="I82" s="6" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="J82" s="6" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="K82" s="46" t="s">
         <v>75</v>
@@ -7079,7 +7326,7 @@
       <c r="L82" s="8"/>
       <c r="M82" s="8"/>
       <c r="N82" s="47" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>24</v>
@@ -7088,42 +7335,42 @@
         <v>104</v>
       </c>
       <c r="Q82" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R82" s="6" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="6" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="B83" s="6">
         <v>9</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F83" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G83" s="6" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="I83" s="6" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="J83" s="6" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="K83" s="46" t="s">
         <v>75</v>
@@ -7131,7 +7378,7 @@
       <c r="L83" s="8"/>
       <c r="M83" s="8"/>
       <c r="N83" s="47" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="O83" s="6" t="s">
         <v>24</v>
@@ -7140,42 +7387,42 @@
         <v>104</v>
       </c>
       <c r="Q83" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R83" s="6" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A84" s="6" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B84" s="6">
         <v>9</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="I84" s="6" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="J84" s="6" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="K84" s="46" t="s">
         <v>75</v>
@@ -7183,7 +7430,7 @@
       <c r="L84" s="8"/>
       <c r="M84" s="8"/>
       <c r="N84" s="47" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="O84" s="6" t="s">
         <v>24</v>
@@ -7192,42 +7439,42 @@
         <v>104</v>
       </c>
       <c r="Q84" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R84" s="6" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="85" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" s="6" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="B85" s="6">
         <v>9</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="F85" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G85" s="6" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="I85" s="6" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="J85" s="6" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="K85" s="46" t="s">
         <v>75</v>
@@ -7235,7 +7482,7 @@
       <c r="L85" s="8"/>
       <c r="M85" s="8"/>
       <c r="N85" s="47" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="O85" s="6" t="s">
         <v>24</v>
@@ -7244,42 +7491,42 @@
         <v>104</v>
       </c>
       <c r="Q85" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R85" s="6" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="86" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" s="6" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B86" s="6">
         <v>9</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="I86" s="6" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="J86" s="6" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="K86" s="46" t="s">
         <v>75</v>
@@ -7287,7 +7534,7 @@
       <c r="L86" s="8"/>
       <c r="M86" s="8"/>
       <c r="N86" s="47" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>24</v>
@@ -7296,15 +7543,15 @@
         <v>104</v>
       </c>
       <c r="Q86" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R86" s="6" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="87" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="B87" s="6">
         <v>10</v>
@@ -7313,7 +7560,7 @@
         <v>35</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>20</v>
@@ -7322,16 +7569,16 @@
         <v>21</v>
       </c>
       <c r="G87" s="6" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="I87" s="6" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="J87" s="6" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="K87" s="46" t="s">
         <v>75</v>
@@ -7339,7 +7586,7 @@
       <c r="L87" s="8"/>
       <c r="M87" s="8"/>
       <c r="N87" s="47" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="O87" s="6" t="s">
         <v>24</v>
@@ -7348,15 +7595,15 @@
         <v>107</v>
       </c>
       <c r="Q87" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R87" s="6" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A88" s="6" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="B88" s="6">
         <v>10</v>
@@ -7365,7 +7612,7 @@
         <v>35</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>20</v>
@@ -7374,16 +7621,16 @@
         <v>21</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="I88" s="6" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="J88" s="6" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="K88" s="46" t="s">
         <v>75</v>
@@ -7391,7 +7638,7 @@
       <c r="L88" s="8"/>
       <c r="M88" s="8"/>
       <c r="N88" s="47" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="O88" s="6" t="s">
         <v>24</v>
@@ -7400,15 +7647,15 @@
         <v>107</v>
       </c>
       <c r="Q88" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R88" s="6" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="89" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="B89" s="6">
         <v>10</v>
@@ -7417,7 +7664,7 @@
         <v>35</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>20</v>
@@ -7426,16 +7673,16 @@
         <v>21</v>
       </c>
       <c r="G89" s="6" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="I89" s="6" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="J89" s="6" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="K89" s="46" t="s">
         <v>75</v>
@@ -7443,7 +7690,7 @@
       <c r="L89" s="8"/>
       <c r="M89" s="8"/>
       <c r="N89" s="47" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="O89" s="6" t="s">
         <v>24</v>
@@ -7452,42 +7699,42 @@
         <v>107</v>
       </c>
       <c r="Q89" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R89" s="6" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="90" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A90" s="6" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="B90" s="6">
         <v>10</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="I90" s="6" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="J90" s="6" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="K90" s="46" t="s">
         <v>75</v>
@@ -7495,7 +7742,7 @@
       <c r="L90" s="8"/>
       <c r="M90" s="8"/>
       <c r="N90" s="47" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="O90" s="6" t="s">
         <v>24</v>
@@ -7504,42 +7751,42 @@
         <v>107</v>
       </c>
       <c r="Q90" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R90" s="6" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
     </row>
     <row r="91" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A91" s="6" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B91" s="6">
         <v>10</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G91" s="6" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="I91" s="6" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="J91" s="6" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="K91" s="46" t="s">
         <v>75</v>
@@ -7547,7 +7794,7 @@
       <c r="L91" s="8"/>
       <c r="M91" s="8"/>
       <c r="N91" s="47" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="O91" s="6" t="s">
         <v>24</v>
@@ -7556,42 +7803,42 @@
         <v>107</v>
       </c>
       <c r="Q91" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R91" s="6" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
     </row>
     <row r="92" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A92" s="6" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="B92" s="6">
         <v>10</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="I92" s="6" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="J92" s="6" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="K92" s="46" t="s">
         <v>75</v>
@@ -7599,7 +7846,7 @@
       <c r="L92" s="8"/>
       <c r="M92" s="8"/>
       <c r="N92" s="47" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="O92" s="6" t="s">
         <v>24</v>
@@ -7608,42 +7855,42 @@
         <v>107</v>
       </c>
       <c r="Q92" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R92" s="6" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
     </row>
     <row r="93" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="6" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="B93" s="6">
         <v>10</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="G93" s="6" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="I93" s="6" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="J93" s="6" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="K93" s="46" t="s">
         <v>75</v>
@@ -7651,7 +7898,7 @@
       <c r="L93" s="8"/>
       <c r="M93" s="8"/>
       <c r="N93" s="47" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="O93" s="6" t="s">
         <v>24</v>
@@ -7660,42 +7907,42 @@
         <v>107</v>
       </c>
       <c r="Q93" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R93" s="6" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
     </row>
     <row r="94" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A94" s="6" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="B94" s="6">
         <v>10</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="I94" s="6" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="J94" s="6" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="K94" s="46" t="s">
         <v>75</v>
@@ -7703,7 +7950,7 @@
       <c r="L94" s="8"/>
       <c r="M94" s="8"/>
       <c r="N94" s="47" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>24</v>
@@ -7712,56 +7959,75 @@
         <v>107</v>
       </c>
       <c r="Q94" s="6" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R94" s="6" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="N45" r:id="rId1" tooltip="Bukti retest pass change-password" xr:uid="{83495BB2-4F28-4636-8350-D973F94E0902}"/>
-    <hyperlink ref="N46" r:id="rId2" tooltip="Bukti retest pass GET /users" xr:uid="{2A6474F4-7C4B-46EE-BFDD-FFE06AF40E86}"/>
-    <hyperlink ref="N51" r:id="rId3" tooltip="Bukti retest pass GET /users/1" xr:uid="{1D4D0B11-6BC6-4996-9878-75C18A64CB5A}"/>
-    <hyperlink ref="N76" r:id="rId4" tooltip="Bukti verifikasi pemisahan angka &amp; persen Donut Chart" xr:uid="{352E79BE-EA5E-416B-9A46-0975FC5478D9}"/>
-    <hyperlink ref="N77" r:id="rId5" tooltip="Bukti modal detail badge unknown amber" xr:uid="{29EBF0BA-A607-4A63-BA02-BD4E08334471}"/>
-    <hyperlink ref="N72" r:id="rId6" tooltip="Wireframe Desktop 1080p" xr:uid="{C5D30B54-7FD1-4625-80AF-A671A87A34CF}"/>
-    <hyperlink ref="N73" r:id="rId7" tooltip="Wireframe Tablet 768p" xr:uid="{BCF9F7C0-2A4A-40E9-82B6-7F9837E16225}"/>
-    <hyperlink ref="N74" r:id="rId8" tooltip="Wireframe Mobile 375p" xr:uid="{940DC609-433C-41F2-9018-441CF70ED274}"/>
-    <hyperlink ref="N75" r:id="rId9" tooltip="Wireframe RBAC Super Admin" xr:uid="{97835F1A-F840-4B49-B544-65C134EE20E7}"/>
-    <hyperlink ref="N78" r:id="rId10" tooltip="Wireframe Persistensi Settings" xr:uid="{D49569CC-A7E8-4FD1-9EEA-11943C68624C}"/>
-    <hyperlink ref="N79" r:id="rId11" tooltip="2026-10-20_Hari-9_dashboard_desktop-1080p.png" xr:uid="{C44BD706-1024-496D-BC2C-FEC5F2FDDBC4}"/>
-    <hyperlink ref="N80" r:id="rId12" tooltip="2026-10-20_Hari-9_dashboard_devices-table.png" xr:uid="{C4E76EE7-1F92-4D21-BE02-3C227961FFA8}"/>
-    <hyperlink ref="N81" r:id="rId13" tooltip="2026-10-20_Hari-9_dashboard_monitoring-live.png" xr:uid="{008D6612-6DA8-41AF-95FA-34960211B1D3}"/>
-    <hyperlink ref="N82" r:id="rId14" tooltip="2026-10-20_Hari-9_dashboard_location-gis.png" xr:uid="{114DF096-9EB4-45C7-A09A-1AF0A57EECAC}"/>
-    <hyperlink ref="N83" r:id="rId15" tooltip="2026-10-20_Hari-9_dashboard_alerts-incidents.png" xr:uid="{8287D95D-5C56-42D7-AE0D-0B12830ABA1F}"/>
-    <hyperlink ref="N84" r:id="rId16" tooltip="2026-10-20_Hari-9_dashboard_users-management.png" xr:uid="{A1CD8320-354E-4D47-A2C0-889080A5FE2D}"/>
-    <hyperlink ref="N85" r:id="rId17" tooltip="2026-10-20_Hari-9_dashboard_tablet-768p.png" xr:uid="{688E4F75-BC2A-4D87-8928-B390BB230019}"/>
-    <hyperlink ref="N86" r:id="rId18" tooltip="2026-10-20_Hari-9_dashboard_mobile-375p.png" xr:uid="{E56ED74B-D5E4-4FB8-A1EC-6EE6A17542CE}"/>
-    <hyperlink ref="N12" r:id="rId19" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA5214D5-F1E0-4AB5-8F33-130BA9BECE39}"/>
-    <hyperlink ref="N87" r:id="rId20" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA69F703-3295-4E68-83AE-6D1BD44B5B8D}"/>
-    <hyperlink ref="N88" r:id="rId21" tooltip="2026-10-21_Hari-10_final-dashboard_alerts-tickets.png" xr:uid="{4605776D-F959-42A0-8F71-F8599BA27AB1}"/>
-    <hyperlink ref="N89" r:id="rId22" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{D4C20B14-4E67-4FE8-B1D7-74877549AED3}"/>
-    <hyperlink ref="N90" r:id="rId23" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{AE154EBE-7DA7-4240-A572-D2F2DBD07D3E}"/>
-    <hyperlink ref="N91" r:id="rId24" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{FABA0045-223F-4258-9055-43736084C725}"/>
-    <hyperlink ref="N92" r:id="rId25" tooltip="2026-10-21_Hari-10_final-dashboard_desktop-1080p.png" xr:uid="{DF0874B5-F3A5-4940-B56E-5C8C97D816B7}"/>
-    <hyperlink ref="N93" r:id="rId26" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{B17C34F4-F7BE-42EA-851C-9107F4B20CCB}"/>
-    <hyperlink ref="N94" r:id="rId27" tooltip="2026-10-21_Hari-10_final-dashboard_users-rbac.png" xr:uid="{2241DBCB-8785-46FF-94D5-F6C6DED84A05}"/>
-    <hyperlink ref="N54" r:id="rId28" tooltip="2026-10-22_Hari-11_TC-MON-001_icmp-ping.png" xr:uid="{8C32334C-50E2-461D-89AF-8EB45F63C7C7}"/>
-    <hyperlink ref="N55" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-MON-002_http-health.png" xr:uid="{5D47D286-D7AE-4B03-A0A4-866AE4CEBB25}"/>
-    <hyperlink ref="N56" r:id="rId30" tooltip="2026-10-22_Hari-11_TC-MON-003_tcp-port-scan.png" xr:uid="{54A22B2F-0B75-42D5-8371-1C9E401985B0}"/>
-    <hyperlink ref="N57" r:id="rId31" tooltip="2026-10-22_Hari-11_TC-MON-004_latency-logs.png" xr:uid="{3B45532E-6326-4EFF-907E-9865FA5CE054}"/>
-    <hyperlink ref="N59" r:id="rId32" tooltip="2026-10-22_Hari-11_TC-HB-001_iot-heartbeat.png" xr:uid="{756D28A9-DCDF-427F-B5A7-F01AB6696F3F}"/>
-    <hyperlink ref="N40" r:id="rId33" xr:uid="{A3C2BAA6-CBF3-4397-B41D-5A324045423D}"/>
-    <hyperlink ref="N43" r:id="rId34" xr:uid="{07F98721-DFA0-4CCD-906D-1564D3193455}"/>
-    <hyperlink ref="N2" r:id="rId35" xr:uid="{D09C9E3E-C97E-481F-A9D5-438C5725DB68}"/>
-    <hyperlink ref="N58" r:id="rId36" xr:uid="{E0B53A3F-B5C3-43B7-A2D4-E0601746F4FD}"/>
-    <hyperlink ref="N28" r:id="rId37" xr:uid="{2A9B3EBA-EB8F-4B77-9B6F-B5485EC42B5D}"/>
-    <hyperlink ref="N64" r:id="rId38" xr:uid="{55A145A2-869F-426A-A996-3D1E4599B081}"/>
+    <hyperlink ref="N43" r:id="rId1" tooltip="Bukti error 500 column created_at" xr:uid="{F1645194-E524-4B93-93C0-93775656DF38}"/>
+    <hyperlink ref="N45" r:id="rId2" tooltip="Bukti retest pass change-password" xr:uid="{83495BB2-4F28-4636-8350-D973F94E0902}"/>
+    <hyperlink ref="N46" r:id="rId3" tooltip="Bukti retest pass GET /users" xr:uid="{2A6474F4-7C4B-46EE-BFDD-FFE06AF40E86}"/>
+    <hyperlink ref="N51" r:id="rId4" tooltip="Bukti retest pass GET /users/1" xr:uid="{1D4D0B11-6BC6-4996-9878-75C18A64CB5A}"/>
+    <hyperlink ref="N76" r:id="rId5" tooltip="Bukti verifikasi pemisahan angka &amp; persen Donut Chart" xr:uid="{352E79BE-EA5E-416B-9A46-0975FC5478D9}"/>
+    <hyperlink ref="N77" r:id="rId6" tooltip="Bukti modal detail badge unknown amber" xr:uid="{29EBF0BA-A607-4A63-BA02-BD4E08334471}"/>
+    <hyperlink ref="N72" r:id="rId7" tooltip="Wireframe Desktop 1080p" xr:uid="{C5D30B54-7FD1-4625-80AF-A671A87A34CF}"/>
+    <hyperlink ref="N73" r:id="rId8" tooltip="Wireframe Tablet 768p" xr:uid="{BCF9F7C0-2A4A-40E9-82B6-7F9837E16225}"/>
+    <hyperlink ref="N74" r:id="rId9" tooltip="Wireframe Mobile 375p" xr:uid="{940DC609-433C-41F2-9018-441CF70ED274}"/>
+    <hyperlink ref="N75" r:id="rId10" tooltip="Wireframe RBAC Super Admin" xr:uid="{97835F1A-F840-4B49-B544-65C134EE20E7}"/>
+    <hyperlink ref="N78" r:id="rId11" tooltip="Wireframe Persistensi Settings" xr:uid="{D49569CC-A7E8-4FD1-9EEA-11943C68624C}"/>
+    <hyperlink ref="N79" r:id="rId12" tooltip="2026-10-20_Hari-9_dashboard_desktop-1080p.png" xr:uid="{C44BD706-1024-496D-BC2C-FEC5F2FDDBC4}"/>
+    <hyperlink ref="N80" r:id="rId13" tooltip="2026-10-20_Hari-9_dashboard_devices-table.png" xr:uid="{C4E76EE7-1F92-4D21-BE02-3C227961FFA8}"/>
+    <hyperlink ref="N81" r:id="rId14" tooltip="2026-10-20_Hari-9_dashboard_monitoring-live.png" xr:uid="{008D6612-6DA8-41AF-95FA-34960211B1D3}"/>
+    <hyperlink ref="N82" r:id="rId15" tooltip="2026-10-20_Hari-9_dashboard_location-gis.png" xr:uid="{114DF096-9EB4-45C7-A09A-1AF0A57EECAC}"/>
+    <hyperlink ref="N83" r:id="rId16" tooltip="2026-10-20_Hari-9_dashboard_alerts-incidents.png" xr:uid="{8287D95D-5C56-42D7-AE0D-0B12830ABA1F}"/>
+    <hyperlink ref="N84" r:id="rId17" tooltip="2026-10-20_Hari-9_dashboard_users-management.png" xr:uid="{A1CD8320-354E-4D47-A2C0-889080A5FE2D}"/>
+    <hyperlink ref="N85" r:id="rId18" tooltip="2026-10-20_Hari-9_dashboard_tablet-768p.png" xr:uid="{688E4F75-BC2A-4D87-8928-B390BB230019}"/>
+    <hyperlink ref="N86" r:id="rId19" tooltip="2026-10-20_Hari-9_dashboard_mobile-375p.png" xr:uid="{E56ED74B-D5E4-4FB8-A1EC-6EE6A17542CE}"/>
+    <hyperlink ref="N12" r:id="rId20" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA5214D5-F1E0-4AB5-8F33-130BA9BECE39}"/>
+    <hyperlink ref="N87" r:id="rId21" tooltip="2026-10-21_Hari-10_final-dashboard_monitoring-live.png" xr:uid="{AA69F703-3295-4E68-83AE-6D1BD44B5B8D}"/>
+    <hyperlink ref="N88" r:id="rId22" tooltip="2026-10-21_Hari-10_final-dashboard_alerts-tickets.png" xr:uid="{4605776D-F959-42A0-8F71-F8599BA27AB1}"/>
+    <hyperlink ref="N89" r:id="rId23" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{D4C20B14-4E67-4FE8-B1D7-74877549AED3}"/>
+    <hyperlink ref="N90" r:id="rId24" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{AE154EBE-7DA7-4240-A572-D2F2DBD07D3E}"/>
+    <hyperlink ref="N91" r:id="rId25" tooltip="2026-10-21_Hari-10_final-dashboard_devices-management.png" xr:uid="{FABA0045-223F-4258-9055-43736084C725}"/>
+    <hyperlink ref="N92" r:id="rId26" tooltip="2026-10-21_Hari-10_final-dashboard_desktop-1080p.png" xr:uid="{DF0874B5-F3A5-4940-B56E-5C8C97D816B7}"/>
+    <hyperlink ref="N93" r:id="rId27" tooltip="2026-10-21_Hari-10_final-dashboard_reports-export.png" xr:uid="{B17C34F4-F7BE-42EA-851C-9107F4B20CCB}"/>
+    <hyperlink ref="N94" r:id="rId28" tooltip="2026-10-21_Hari-10_final-dashboard_users-rbac.png" xr:uid="{2241DBCB-8785-46FF-94D5-F6C6DED84A05}"/>
+    <hyperlink ref="N54" r:id="rId29" tooltip="2026-10-22_Hari-11_TC-MON-001_icmp-ping.png" xr:uid="{8C32334C-50E2-461D-89AF-8EB45F63C7C7}"/>
+    <hyperlink ref="N55" r:id="rId30" tooltip="2026-10-22_Hari-11_TC-MON-002_http-health.png" xr:uid="{5D47D286-D7AE-4B03-A0A4-866AE4CEBB25}"/>
+    <hyperlink ref="N56" r:id="rId31" tooltip="2026-10-22_Hari-11_TC-MON-003_tcp-port-scan.png" xr:uid="{54A22B2F-0B75-42D5-8371-1C9E401985B0}"/>
+    <hyperlink ref="N57" r:id="rId32" tooltip="2026-10-22_Hari-11_TC-MON-004_latency-logs.png" xr:uid="{3B45532E-6326-4EFF-907E-9865FA5CE054}"/>
+    <hyperlink ref="N58" r:id="rId33" tooltip="2026-10-22_Hari-11_TC-MON-005_monitoring-summary.png" xr:uid="{C3BDC459-DA6D-4F63-83EB-830608126897}"/>
+    <hyperlink ref="N28" r:id="rId34" tooltip="2026-10-23_Hari-12_TC-INC-001_auto-incident-generated.png" xr:uid="{007CCACA-3220-4F7C-912C-66F1A0DC4260}"/>
+    <hyperlink ref="N29" r:id="rId35" tooltip="2026-10-23_Hari-12_TC-REC-001_auto-resolved-recovery.png" xr:uid="{DB45E82C-A556-4308-B54C-1019F073E6BD}"/>
+    <hyperlink ref="N30" r:id="rId36" tooltip="2026-10-23_Hari-12_TC-FAIL-001_offline-detection.png" xr:uid="{028E6BEF-3D80-4EAC-B73A-A23554BC740F}"/>
+    <hyperlink ref="N31" r:id="rId37" tooltip="2026-10-23_Hari-12_TC-NOTIF-001_alert-notification-trigger.png" xr:uid="{3D282DAD-DBA6-48CA-AB3F-2D3422710268}"/>
+    <hyperlink ref="N32" r:id="rId38" tooltip="2026-10-23_Hari-12_TC-HB-002_iot-heartbeat-recovery.png" xr:uid="{D3C4FE45-45EE-4B9C-B10E-CB4590A69183}"/>
+    <hyperlink ref="N33" r:id="rId39" tooltip="2026-10-23_Hari-12_TC-WARN-001_high-latency-warning.png" xr:uid="{5C311F97-1645-4AF3-BE81-26737B5A7616}"/>
+    <hyperlink ref="N13" r:id="rId40" tooltip="2026-10-24_Hari-13_TC-ASSET-001_mikrotik-router-inventory.png" xr:uid="{FDF4D14C-C5D5-4582-AB14-CEA7F79D4EE0}"/>
+    <hyperlink ref="N14" r:id="rId41" tooltip="2026-10-24_Hari-13_TC-ASSET-002_cisco-switch-inventory.png" xr:uid="{B9E2F447-BAC9-4B67-95B5-7CAF928E0B44}"/>
+    <hyperlink ref="N15" r:id="rId42" tooltip="2026-10-24_Hari-13_TC-ASSET-003_unifi-cctv-inventory.png" xr:uid="{F3983513-8E89-4698-819D-D6471553D351}"/>
+    <hyperlink ref="N16" r:id="rId43" tooltip="2026-10-24_Hari-13_TC-ASSET-004_ubuntu-server-inventory.png" xr:uid="{5DBD0251-C75D-467F-AFE4-E6BA0F8483D3}"/>
+    <hyperlink ref="N17" r:id="rId44" tooltip="2026-10-24_Hari-13_TC-ASSET-005_raspberry-pi-gateway.png" xr:uid="{BBB0DDF3-46B9-41AC-A656-81556AC87881}"/>
+    <hyperlink ref="N18" r:id="rId45" tooltip="2026-10-24_Hari-13_TC-ASSET-006_website-service-online.png" xr:uid="{E05D0B9F-D8C4-40EB-9BD3-208BAB08B4D6}"/>
+    <hyperlink ref="N19" r:id="rId46" tooltip="2026-10-24_Hari-13_TC-ASSET-007_esp32-node-detail.png" xr:uid="{9D0542B8-2529-4508-8B1F-4CC57B36FBF0}"/>
+    <hyperlink ref="N20" r:id="rId47" tooltip="2026-10-24_Hari-13_TC-ASSET-008_mqtt-broker-telemetry.png" xr:uid="{C16E7186-745F-49BF-8F50-609D36152464}"/>
+    <hyperlink ref="N21" r:id="rId48" tooltip="2026-10-24_Hari-13_TC-ASSET-009_pc-headoffice-inventory.png" xr:uid="{7E6B24A3-D823-4A83-85AD-6C6BFF68A2EE}"/>
+    <hyperlink ref="N22" r:id="rId49" tooltip="2026-10-24_Hari-13_TC-ASSET-010_filter-category-router.png" xr:uid="{3FD571B0-C8DB-41DE-A520-A60E0198F20D}"/>
+    <hyperlink ref="N23" r:id="rId50" tooltip="2026-10-24_Hari-13_TC-ASSET-011_filter-category-iotnode.png" xr:uid="{AE0B56BA-97F6-470E-8FCC-4EA979E82728}"/>
+    <hyperlink ref="N24" r:id="rId51" tooltip="2026-10-24_Hari-13_TC-ASSET-012_filter-location-headoffice.png" xr:uid="{92DD1907-892B-4518-8C88-B697E5ECF6F7}"/>
+    <hyperlink ref="N25" r:id="rId52" tooltip="2026-10-24_Hari-13_TC-ASSET-013_mikrotik-ip-verification.png" xr:uid="{9D3FD046-52F4-4BC1-83F1-BFDEBD4829B0}"/>
+    <hyperlink ref="N26" r:id="rId53" tooltip="2026-10-24_Hari-13_TC-ASSET-014_esp32-mqtt-telemetry-config.png" xr:uid="{97B88EBF-9951-4531-8502-F11879584B4F}"/>
+    <hyperlink ref="N27" r:id="rId54" tooltip="2026-10-24_Hari-13_TC-ASSET-015_priority-1-critical-assets.png" xr:uid="{51A986EA-7186-4816-BE34-DED43A545689}"/>
+    <hyperlink ref="N59" r:id="rId55" tooltip="2026-10-24_Hari-13_TC-HB-001_iot-heartbeat-telemetry.png" xr:uid="{35DDC9E2-E8AB-4E6C-AB71-473234EF7D38}"/>
+    <hyperlink ref="N60" r:id="rId56" tooltip="2026-10-24_Hari-13_TC-HB-002_unregistered-device-rejection.png" xr:uid="{4E938102-9653-4E6B-9323-88CAE94A927F}"/>
+    <hyperlink ref="N61" r:id="rId57" tooltip="2026-10-24_Hari-13_TC-HB-003_latest-iot-heartbeat-denah.png" xr:uid="{AEB6E9F5-C394-44F4-AEA3-AF7F37891BAC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId39"/>
+  <pageSetup orientation="portrait" r:id="rId58"/>
 </worksheet>
 </file>
 
@@ -7809,7 +8075,7 @@
         <v>427</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -7823,7 +8089,7 @@
         <v>87</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>260</v>
@@ -7835,13 +8101,13 @@
         <v>71</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H2" s="12" t="s">
         <v>90</v>
       </c>
       <c r="I2" s="32" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
@@ -7852,7 +8118,7 @@
         <v>87</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>282</v>
@@ -7864,24 +8130,24 @@
         <v>71</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H3" s="12" t="s">
         <v>96</v>
       </c>
       <c r="I3" s="32" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>93</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>260</v>
@@ -7893,24 +8159,24 @@
         <v>71</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>96</v>
       </c>
       <c r="I4" s="32" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>96</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>282</v>
@@ -7922,187 +8188,187 @@
         <v>71</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>96</v>
       </c>
       <c r="I5" s="32" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>100</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I6" s="32" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I7" s="32" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>420</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I8" s="32" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B9" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>420</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I9" s="32" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I10" s="32" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>101</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>481</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>492</v>
-      </c>
       <c r="F11" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>101</v>
       </c>
       <c r="I11" s="32" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
@@ -8110,19 +8376,19 @@
       <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="59" t="s">
-        <v>586</v>
-      </c>
-      <c r="B13" s="59"/>
-      <c r="C13" s="59"/>
+      <c r="A13" s="57" t="s">
+        <v>588</v>
+      </c>
+      <c r="B13" s="57"/>
+      <c r="C13" s="57"/>
       <c r="M13" s="49"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="59" t="s">
-        <v>587</v>
-      </c>
-      <c r="B14" s="59"/>
-      <c r="C14" s="59"/>
+      <c r="A14" s="57" t="s">
+        <v>589</v>
+      </c>
+      <c r="B14" s="57"/>
+      <c r="C14" s="57"/>
       <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
@@ -8273,7 +8539,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="N1" s="22" t="s">
         <v>62</v>
@@ -8302,7 +8568,7 @@
         <v>67</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>24</v>
@@ -8320,29 +8586,29 @@
         <v>21</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="6" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="L2" s="6">
         <v>404</v>
       </c>
       <c r="M2" s="51" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="N2" s="33" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q2" s="4" t="s">
         <v>71</v>
@@ -8354,7 +8620,7 @@
         <v>90</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="W2" s="2"/>
     </row>
@@ -8363,7 +8629,7 @@
         <v>69</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>24</v>
@@ -8381,29 +8647,29 @@
         <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="6" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="L3" s="6">
         <v>500</v>
       </c>
       <c r="M3" s="51" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="N3" s="33" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q3" s="4" t="s">
         <v>71</v>
@@ -8415,16 +8681,16 @@
         <v>96</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="W3" s="2"/>
     </row>
     <row r="4" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>24</v>
@@ -8442,29 +8708,29 @@
         <v>21</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I4" s="10"/>
       <c r="J4" s="6" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="L4" s="6">
         <v>500</v>
       </c>
       <c r="M4" s="51" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="N4" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>71</v>
@@ -8476,15 +8742,15 @@
         <v>96</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>24</v>
@@ -8502,29 +8768,29 @@
         <v>21</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" s="6" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="L5" s="6">
         <v>500</v>
       </c>
       <c r="M5" s="51" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="N5" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q5" s="4" t="s">
         <v>71</v>
@@ -8536,15 +8802,15 @@
         <v>96</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>24</v>
@@ -8553,7 +8819,7 @@
         <v>100</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>70</v>
@@ -8562,32 +8828,32 @@
         <v>21</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="M6" s="52" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>24</v>
@@ -8596,15 +8862,15 @@
         <v>101</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>24</v>
@@ -8613,7 +8879,7 @@
         <v>101</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>70</v>
@@ -8622,32 +8888,32 @@
         <v>21</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" s="6" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>277</v>
       </c>
       <c r="M7" s="51" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R7" s="4" t="s">
         <v>24</v>
@@ -8656,15 +8922,15 @@
         <v>101</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>24</v>
@@ -8673,7 +8939,7 @@
         <v>101</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>420</v>
@@ -8682,32 +8948,32 @@
         <v>47</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="M8" s="51" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R8" s="4" t="s">
         <v>24</v>
@@ -8716,15 +8982,15 @@
         <v>101</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>24</v>
@@ -8733,7 +8999,7 @@
         <v>101</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>420</v>
@@ -8742,32 +9008,32 @@
         <v>47</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" s="6" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="M9" s="51" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R9" s="4" t="s">
         <v>24</v>
@@ -8776,15 +9042,15 @@
         <v>101</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>24</v>
@@ -8793,41 +9059,41 @@
         <v>101</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="M10" s="51" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R10" s="4" t="s">
         <v>24</v>
@@ -8836,15 +9102,15 @@
         <v>101</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="11" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="42" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C11" s="43" t="s">
         <v>24</v>
@@ -8853,41 +9119,41 @@
         <v>101</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F11" s="43" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G11" s="43" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H11" s="43" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I11" s="38"/>
       <c r="J11" s="39" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="K11" s="39" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="L11" s="39" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="M11" s="51" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="N11" s="43" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="O11" s="43" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="P11" s="43" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q11" s="43" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R11" s="43" t="s">
         <v>24</v>
@@ -8896,15 +9162,15 @@
         <v>101</v>
       </c>
       <c r="T11" s="39" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="12" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="50" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>24</v>
@@ -8913,7 +9179,7 @@
         <v>107</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>70</v>
@@ -8922,34 +9188,34 @@
         <v>21</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="M12" s="48" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="N12" s="53" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="O12" s="55" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R12" s="4" t="s">
         <v>24</v>
@@ -8958,15 +9224,15 @@
         <v>107</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="50" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>24</v>
@@ -8975,7 +9241,7 @@
         <v>107</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>70</v>
@@ -8984,34 +9250,34 @@
         <v>21</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="M13" s="48" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="N13" s="54" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="O13" s="55" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q13" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R13" s="4" t="s">
         <v>24</v>
@@ -9020,15 +9286,15 @@
         <v>107</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="50" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>24</v>
@@ -9046,34 +9312,34 @@
         <v>47</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="M14" s="48" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="N14" s="54" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="O14" s="55" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R14" s="4" t="s">
         <v>24</v>
@@ -9082,15 +9348,15 @@
         <v>107</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="50" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>24</v>
@@ -9102,40 +9368,40 @@
         <v>164</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="M15" s="48" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="N15" s="54" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="O15" s="55" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R15" s="4" t="s">
         <v>24</v>
@@ -9144,15 +9410,15 @@
         <v>107</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
     </row>
     <row r="16" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="50" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>24</v>
@@ -9161,7 +9427,7 @@
         <v>107</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>420</v>
@@ -9170,34 +9436,34 @@
         <v>47</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="M16" s="48" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="N16" s="54" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="O16" s="55" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R16" s="4" t="s">
         <v>24</v>
@@ -9206,15 +9472,15 @@
         <v>107</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="50" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>24</v>
@@ -9232,34 +9498,34 @@
         <v>47</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="M17" s="48" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="N17" s="54" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="O17" s="55" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q17" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R17" s="4" t="s">
         <v>24</v>
@@ -9268,15 +9534,15 @@
         <v>107</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
     </row>
     <row r="18" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="50" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>24</v>
@@ -9285,43 +9551,43 @@
         <v>107</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="M18" s="48" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="N18" s="54" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="O18" s="55" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R18" s="4" t="s">
         <v>24</v>
@@ -9330,15 +9596,15 @@
         <v>107</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="50" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>24</v>
@@ -9350,40 +9616,40 @@
         <v>282</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="M19" s="48" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="N19" s="54" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="O19" s="55" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="R19" s="4" t="s">
         <v>24</v>
@@ -9392,7 +9658,7 @@
         <v>107</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>821</v>
+        <v>823</v>
       </c>
     </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.35">
@@ -9782,10 +10048,10 @@
         <v>5</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -9820,10 +10086,10 @@
         <v>5</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -9992,13 +10258,13 @@
         <v>82</v>
       </c>
       <c r="D14" s="13">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E14" s="13">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="F14" s="13">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G14" s="13">
         <v>0</v>
@@ -11056,7 +11322,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="27" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B14" s="13">
         <f>COUNTIF(MASTER_TC!C:C,A14)</f>
@@ -11081,7 +11347,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B15" s="30">
         <f>SUM(B2:B14)</f>

</xml_diff>

<commit_message>
feat(qa): restore authentic day-6 database and bug retest screenshots, fix execution log row 14
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\docs\qa\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Desktop\docs\qa-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E068549-CA26-4798-A0F9-323449E3512F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C2ACAB-54CB-4D82-B840-322EFBE7E7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="220" windowWidth="14400" windowHeight="7810" firstSheet="2" activeTab="4" xr2:uid="{D20540B9-5A4B-4C0F-A1AA-6997D01BA992}"/>
   </bookViews>
@@ -10264,7 +10264,7 @@
         <v>18</v>
       </c>
       <c r="F14" s="13">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G14" s="13">
         <v>0</v>

</xml_diff>

<commit_message>
feat(qa): mobile responsiveness suite, 3g network throttling, error sanitization and 7 test cases day-16
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17299131-5262-4B13-9450-4F368E802905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75382754-465F-445A-8E27-053E2EACCA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2093" uniqueCount="1067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2184" uniqueCount="1118">
   <si>
     <t>TC ID</t>
   </si>
@@ -3446,6 +3446,159 @@
   </si>
   <si>
     <t>Modul pelaporan SLA dan kecerdasan buatan tervalidasi akurat; fitur ekspor PDF/Excel siap digunakan.</t>
+  </si>
+  <si>
+    <t>TC-H16-001</t>
+  </si>
+  <si>
+    <t>Network Simulation</t>
+  </si>
+  <si>
+    <t>Network Throttling 3G Simulation &amp; Dashboard Executive KPI</t>
+  </si>
+  <si>
+    <t>Performance / Network</t>
+  </si>
+  <si>
+    <t>Frontend port 5500 &amp; Backend port 3000 aktif, DevTools Network throttling diatur ke 3G</t>
+  </si>
+  <si>
+    <t>1. Buka DevTools F12 -&gt; tab Network. 2. Pilih Throttling 3G (Slow/Fast 3G). 3. Muat ulang dashboard eksekutif. 4. Amati waterfall request dan rendering KPI 15 perangkat.</t>
+  </si>
+  <si>
+    <t>Pemuatan skrip dan aset berjalan teratur (graceful loading), 6 kartu KPI dan donut chart ter-render stabil tanpa fatal script error.</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Waterfall request 3G terpantau stabil (~2.03s per call), KPI 15 perangkat dan peta sebaran 3 lokasi tampil lengkap.</t>
+  </si>
+  <si>
+    <t>TC-H16-002</t>
+  </si>
+  <si>
+    <t>Responsive Mobile UI</t>
+  </si>
+  <si>
+    <t>Mobile Viewport Dashboard &amp; Responsive KPI Layout</t>
+  </si>
+  <si>
+    <t>UI / Responsiveness</t>
+  </si>
+  <si>
+    <t>DevTools device toolbar aktif (resolusi smartphone &lt;640px / 434x993)</t>
+  </si>
+  <si>
+    <t>1. Tekan Ctrl+Shift+M untuk beralih ke mobile viewport. 2. Amati susunan header topbar, banner dashboard, dan grid KPI.</t>
+  </si>
+  <si>
+    <t>Header topbar rapi, banner auto-wrap, grid 6 kartu KPI beradaptasi otomatis menjadi 2 kolom proporsional, dan bottom bar aktif di bawah.</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Tampilan dashboard HP proporsional, tidak ada elemen melar keluar batas layar horizontal.</t>
+  </si>
+  <si>
+    <t>TC-H16-003</t>
+  </si>
+  <si>
+    <t>User Authentication &amp; RBAC</t>
+  </si>
+  <si>
+    <t>Mobile User Profile &amp; Account Switcher Dropdown Interaction</t>
+  </si>
+  <si>
+    <t>UI / Functional</t>
+  </si>
+  <si>
+    <t>Sesi login aktif sebagai Reza Tri Wardana (Admin) pada viewport mobile</t>
+  </si>
+  <si>
+    <t>1. Klik ikon avatar profil warna cyan di pojok kanan atas topbar HP. 2. Verifikasi menu dropdown yang muncul.</t>
+  </si>
+  <si>
+    <t>Dropdown menu profil melayang rapi di bawah avatar, menampilkan nama user, role admin, opsi ganti foto, dan tombol Kembali ke Halaman Masuk / Ganti Akun tanpa terpotong tepi layar.</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Menu ganti akun tampil utuh 100%, klikabel, dan terisolasi rapi di layar HP.</t>
+  </si>
+  <si>
+    <t>TC-H16-004</t>
+  </si>
+  <si>
+    <t>Mobile Devices Table Horizontal Swipe &amp; Touch Scroll</t>
+  </si>
+  <si>
+    <t>Navigasi ke halaman Inventarisasi Perangkat pada viewport mobile</t>
+  </si>
+  <si>
+    <t>1. Buka menu Perangkat via bottom nav bar. 2. Gulir ke tabel daftar perangkat. 3. Lakukan gestur swipe / scroll menyamping ke kanan dan kiri.</t>
+  </si>
+  <si>
+    <t>Tabel 15 perangkat dapat digeser horizontal dengan mulus di dalam card container tanpa merusak lebar halaman web.</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Seluruh kolom tabel (No, Kode Aset, Nama, IP, Lokasi, Status) dapat dibaca utuh dengan touch-swipe scroll yang responsif.</t>
+  </si>
+  <si>
+    <t>TC-H16-005</t>
+  </si>
+  <si>
+    <t>Mobile Devices Table Full Inventory Rendering (15 Aset)</t>
+  </si>
+  <si>
+    <t>Tabel perangkat pada layar smartphone termuat penuh</t>
+  </si>
+  <si>
+    <t>1. Gulir ke bagian bawah tabel perangkat. 2. Verifikasi baris ke-15 (SWM-01 Switch Manageable).</t>
+  </si>
+  <si>
+    <t>Seluruh 15 baris aset dari database MariaDB ter-render lengkap dari baris 1 hingga baris 15.</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Baris ke-15 terbukti tampil utuh dengan nomor urut, kode aset, dan IP address yang akurat.</t>
+  </si>
+  <si>
+    <t>TC-H16-006</t>
+  </si>
+  <si>
+    <t>API Security</t>
+  </si>
+  <si>
+    <t>Backend API Error Sanitization 404 &amp; Zero Data Leakage</t>
+  </si>
+  <si>
+    <t>Security / API</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Server backend port 3000 aktif</t>
+  </si>
+  <si>
+    <t>1. Akses endpoint palsu GET /api/endpoint-palsu-testing via browser/HTTP client. 2. Analisis response payload dan status code.</t>
+  </si>
+  <si>
+    <t>Server merespon dengan HTTP 404 dan JSON payload tersanitasi bersih tanpa mengekspos stack trace atau struktur database.</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Response: {"success":false,"error":"Endpoint tidak ditemukan"} dengan HTTP status 404, zero data leakage terverifikasi 100%.</t>
+  </si>
+  <si>
+    <t>TC-H16-007</t>
+  </si>
+  <si>
+    <t>Device Keyword Search CCTV Filter Integrity</t>
+  </si>
+  <si>
+    <t>Halaman perangkat aktif dengan 15 data aset</t>
+  </si>
+  <si>
+    <t>1. Masukkan kata kunci 'cctv' pada kolom pencarian aset. 2. Verifikasi hasil baris tabel yang ditampilkan.</t>
+  </si>
+  <si>
+    <t>Tabel menyaring data secara instan dan menampilkan tepat 2 perangkat (CCTV Head Office dan CCTV Marketing).</t>
+  </si>
+  <si>
+    <t>Sesuai harapan. Tepat 2 unit CCTV tersaring akurat dengan IP 192.168.1.39 dan 192.168.1.8.</t>
   </si>
 </sst>
 </file>
@@ -3455,7 +3608,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3539,6 +3692,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3661,7 +3822,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3808,11 +3969,13 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4128,7 +4291,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R111"/>
+  <dimension ref="A1:R118"/>
   <sheetFormatPr defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" customWidth="1"/>
@@ -7175,7 +7338,7 @@
       <c r="M67" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N67" s="57" t="s">
+      <c r="N67" s="56" t="s">
         <v>1018</v>
       </c>
       <c r="O67" s="5" t="s">
@@ -7231,7 +7394,7 @@
       <c r="M68" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N68" s="57" t="s">
+      <c r="N68" s="56" t="s">
         <v>1028</v>
       </c>
       <c r="O68" s="5" t="s">
@@ -7287,7 +7450,7 @@
       <c r="M69" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N69" s="57" t="s">
+      <c r="N69" s="56" t="s">
         <v>1037</v>
       </c>
       <c r="O69" s="5" t="s">
@@ -7343,7 +7506,7 @@
       <c r="M70" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N70" s="57" t="s">
+      <c r="N70" s="56" t="s">
         <v>1046</v>
       </c>
       <c r="O70" s="5" t="s">
@@ -7399,7 +7562,7 @@
       <c r="M71" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N71" s="57" t="s">
+      <c r="N71" s="56" t="s">
         <v>1055</v>
       </c>
       <c r="O71" s="5" t="s">
@@ -7455,7 +7618,7 @@
       <c r="M72" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N72" s="58" t="s">
+      <c r="N72" s="57" t="s">
         <v>1065</v>
       </c>
       <c r="O72" s="5" t="s">
@@ -9555,6 +9718,363 @@
       </c>
       <c r="R111" t="s">
         <v>753</v>
+      </c>
+    </row>
+    <row r="112" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B112">
+        <v>16</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D112" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E112" t="s">
+        <v>1070</v>
+      </c>
+      <c r="F112" t="s">
+        <v>272</v>
+      </c>
+      <c r="G112" t="s">
+        <v>1071</v>
+      </c>
+      <c r="H112" t="s">
+        <v>1072</v>
+      </c>
+      <c r="I112" t="s">
+        <v>1073</v>
+      </c>
+      <c r="J112" t="s">
+        <v>1074</v>
+      </c>
+      <c r="K112" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L112" t="s">
+        <v>21</v>
+      </c>
+      <c r="M112" t="s">
+        <v>277</v>
+      </c>
+      <c r="N112" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-001_network-throttling-3g-dashboard-kpi.png", "2026-10-27_Hari-16_TC-H16-001_network-throttling-3g-dashboard-kpi.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-001_network-throttling-3g-dashboard-kpi.png</v>
+      </c>
+      <c r="O112" t="s">
+        <v>404</v>
+      </c>
+      <c r="P112" s="59">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B113">
+        <v>16</v>
+      </c>
+      <c r="C113" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D113" t="s">
+        <v>1077</v>
+      </c>
+      <c r="E113" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F113" t="s">
+        <v>272</v>
+      </c>
+      <c r="G113" t="s">
+        <v>1079</v>
+      </c>
+      <c r="H113" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I113" t="s">
+        <v>1081</v>
+      </c>
+      <c r="J113" t="s">
+        <v>1082</v>
+      </c>
+      <c r="K113" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L113" t="s">
+        <v>21</v>
+      </c>
+      <c r="M113" t="s">
+        <v>277</v>
+      </c>
+      <c r="N113" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-002_mobile-viewport-dashboard-kpi-layout.png", "2026-10-27_Hari-16_TC-H16-002_mobile-viewport-dashboard-kpi-layout.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-002_mobile-viewport-dashboard-kpi-layout.png</v>
+      </c>
+      <c r="O113" t="s">
+        <v>404</v>
+      </c>
+      <c r="P113" s="59">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B114">
+        <v>16</v>
+      </c>
+      <c r="C114" t="s">
+        <v>1084</v>
+      </c>
+      <c r="D114" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E114" t="s">
+        <v>1086</v>
+      </c>
+      <c r="F114" t="s">
+        <v>272</v>
+      </c>
+      <c r="G114" t="s">
+        <v>1087</v>
+      </c>
+      <c r="H114" t="s">
+        <v>1088</v>
+      </c>
+      <c r="I114" t="s">
+        <v>1089</v>
+      </c>
+      <c r="J114" t="s">
+        <v>1090</v>
+      </c>
+      <c r="K114" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L114" t="s">
+        <v>21</v>
+      </c>
+      <c r="M114" t="s">
+        <v>277</v>
+      </c>
+      <c r="N114" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-003_mobile-user-profile-account-switcher-dropdown.png", "2026-10-27_Hari-16_TC-H16-003_mobile-user-profile-account-switcher-dropdown.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-003_mobile-user-profile-account-switcher-dropdown.png</v>
+      </c>
+      <c r="O114" t="s">
+        <v>404</v>
+      </c>
+      <c r="P114" s="59">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B115">
+        <v>16</v>
+      </c>
+      <c r="C115" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D115" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E115" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F115" t="s">
+        <v>272</v>
+      </c>
+      <c r="G115" t="s">
+        <v>1093</v>
+      </c>
+      <c r="H115" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I115" t="s">
+        <v>1095</v>
+      </c>
+      <c r="J115" t="s">
+        <v>1096</v>
+      </c>
+      <c r="K115" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L115" t="s">
+        <v>21</v>
+      </c>
+      <c r="M115" t="s">
+        <v>277</v>
+      </c>
+      <c r="N115" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-004_mobile-devices-table-horizontal-swipe-scroll.png", "2026-10-27_Hari-16_TC-H16-004_mobile-devices-table-horizontal-swipe-scroll.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-004_mobile-devices-table-horizontal-swipe-scroll.png</v>
+      </c>
+      <c r="O115" t="s">
+        <v>404</v>
+      </c>
+      <c r="P115" s="59">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B116">
+        <v>16</v>
+      </c>
+      <c r="C116" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D116" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E116" t="s">
+        <v>1086</v>
+      </c>
+      <c r="F116" t="s">
+        <v>272</v>
+      </c>
+      <c r="G116" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H116" t="s">
+        <v>1100</v>
+      </c>
+      <c r="I116" t="s">
+        <v>1101</v>
+      </c>
+      <c r="J116" t="s">
+        <v>1102</v>
+      </c>
+      <c r="K116" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L116" t="s">
+        <v>21</v>
+      </c>
+      <c r="M116" t="s">
+        <v>277</v>
+      </c>
+      <c r="N116" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png", "2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png</v>
+      </c>
+      <c r="O116" t="s">
+        <v>404</v>
+      </c>
+      <c r="P116" s="59">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B117">
+        <v>16</v>
+      </c>
+      <c r="C117" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D117" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E117" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F117" t="s">
+        <v>1107</v>
+      </c>
+      <c r="G117" t="s">
+        <v>1108</v>
+      </c>
+      <c r="H117" t="s">
+        <v>1109</v>
+      </c>
+      <c r="I117" t="s">
+        <v>1110</v>
+      </c>
+      <c r="J117" t="s">
+        <v>1111</v>
+      </c>
+      <c r="K117" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L117" t="s">
+        <v>21</v>
+      </c>
+      <c r="M117" t="s">
+        <v>277</v>
+      </c>
+      <c r="N117" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png", "2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png</v>
+      </c>
+      <c r="O117" t="s">
+        <v>404</v>
+      </c>
+      <c r="P117" s="59">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B118">
+        <v>16</v>
+      </c>
+      <c r="C118" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D118" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E118" t="s">
+        <v>728</v>
+      </c>
+      <c r="F118" t="s">
+        <v>272</v>
+      </c>
+      <c r="G118" t="s">
+        <v>1114</v>
+      </c>
+      <c r="H118" t="s">
+        <v>1115</v>
+      </c>
+      <c r="I118" t="s">
+        <v>1116</v>
+      </c>
+      <c r="J118" t="s">
+        <v>1117</v>
+      </c>
+      <c r="K118" s="60" t="s">
+        <v>27</v>
+      </c>
+      <c r="L118" t="s">
+        <v>21</v>
+      </c>
+      <c r="M118" t="s">
+        <v>277</v>
+      </c>
+      <c r="N118" s="56" t="str">
+        <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png", "2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png")</f>
+        <v>2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png</v>
+      </c>
+      <c r="O118" t="s">
+        <v>404</v>
+      </c>
+      <c r="P118" s="59">
+        <v>46322</v>
       </c>
     </row>
   </sheetData>
@@ -9640,7 +10160,7 @@
     <hyperlink ref="N72" r:id="rId79" xr:uid="{12D4C9A3-6BC5-4A52-9045-6452F292C102}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId80"/>
 </worksheet>
 </file>
 
@@ -9989,19 +10509,19 @@
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="56" t="s">
+      <c r="A13" s="58" t="s">
         <v>789</v>
       </c>
-      <c r="B13" s="56"/>
-      <c r="C13" s="56"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
       <c r="M13" s="28"/>
     </row>
     <row r="14" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="56" t="s">
+      <c r="A14" s="58" t="s">
         <v>790</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
+      <c r="B14" s="58"/>
+      <c r="C14" s="58"/>
       <c r="M14" s="28"/>
     </row>
     <row r="15" spans="1:14" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
docs(qa): synchronize full 16-day handovers, test reports, and authentic screenshots Day 16
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75382754-465F-445A-8E27-053E2EACCA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{079684CA-33DD-4E5C-B5C8-D42181C2EBA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3971,11 +3971,11 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -9751,7 +9751,7 @@
       <c r="J112" t="s">
         <v>1074</v>
       </c>
-      <c r="K112" s="60" t="s">
+      <c r="K112" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L112" t="s">
@@ -9767,7 +9767,7 @@
       <c r="O112" t="s">
         <v>404</v>
       </c>
-      <c r="P112" s="59">
+      <c r="P112" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       <c r="J113" t="s">
         <v>1082</v>
       </c>
-      <c r="K113" s="60" t="s">
+      <c r="K113" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L113" t="s">
@@ -9818,7 +9818,7 @@
       <c r="O113" t="s">
         <v>404</v>
       </c>
-      <c r="P113" s="59">
+      <c r="P113" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -9853,7 +9853,7 @@
       <c r="J114" t="s">
         <v>1090</v>
       </c>
-      <c r="K114" s="60" t="s">
+      <c r="K114" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L114" t="s">
@@ -9869,7 +9869,7 @@
       <c r="O114" t="s">
         <v>404</v>
       </c>
-      <c r="P114" s="59">
+      <c r="P114" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -9904,7 +9904,7 @@
       <c r="J115" t="s">
         <v>1096</v>
       </c>
-      <c r="K115" s="60" t="s">
+      <c r="K115" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L115" t="s">
@@ -9920,7 +9920,7 @@
       <c r="O115" t="s">
         <v>404</v>
       </c>
-      <c r="P115" s="59">
+      <c r="P115" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -9955,7 +9955,7 @@
       <c r="J116" t="s">
         <v>1102</v>
       </c>
-      <c r="K116" s="60" t="s">
+      <c r="K116" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L116" t="s">
@@ -9971,7 +9971,7 @@
       <c r="O116" t="s">
         <v>404</v>
       </c>
-      <c r="P116" s="59">
+      <c r="P116" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -10006,7 +10006,7 @@
       <c r="J117" t="s">
         <v>1111</v>
       </c>
-      <c r="K117" s="60" t="s">
+      <c r="K117" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L117" t="s">
@@ -10022,7 +10022,7 @@
       <c r="O117" t="s">
         <v>404</v>
       </c>
-      <c r="P117" s="59">
+      <c r="P117" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -10057,7 +10057,7 @@
       <c r="J118" t="s">
         <v>1117</v>
       </c>
-      <c r="K118" s="60" t="s">
+      <c r="K118" s="59" t="s">
         <v>27</v>
       </c>
       <c r="L118" t="s">
@@ -10073,7 +10073,7 @@
       <c r="O118" t="s">
         <v>404</v>
       </c>
-      <c r="P118" s="59">
+      <c r="P118" s="58">
         <v>46322</v>
       </c>
     </row>
@@ -10158,9 +10158,16 @@
     <hyperlink ref="N70" r:id="rId77" xr:uid="{8D48B14F-5B96-4013-BF36-44D8E733794C}"/>
     <hyperlink ref="N71" r:id="rId78" xr:uid="{EEDC24C4-D93D-4655-9461-D8AF36FD26DB}"/>
     <hyperlink ref="N72" r:id="rId79" xr:uid="{12D4C9A3-6BC5-4A52-9045-6452F292C102}"/>
+    <hyperlink ref="N112" r:id="rId80" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-001_network-throttling-3g-dashboard-kpi.png" display="2026-10-27_Hari-16_TC-H16-001_network-throttling-3g-dashboard-kpi.png" xr:uid="{070C1A69-6A0B-406D-975E-CD7B2DB2CC63}"/>
+    <hyperlink ref="N113" r:id="rId81" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-002_mobile-viewport-dashboard-kpi-layout.png" display="2026-10-27_Hari-16_TC-H16-002_mobile-viewport-dashboard-kpi-layout.png" xr:uid="{E481732C-C6BE-4A36-B74B-D1503BEF885A}"/>
+    <hyperlink ref="N114" r:id="rId82" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-003_mobile-user-profile-account-switcher-dropdown.png" display="2026-10-27_Hari-16_TC-H16-003_mobile-user-profile-account-switcher-dropdown.png" xr:uid="{28E57332-0A6E-42B9-91EF-DE84FBC6B1BD}"/>
+    <hyperlink ref="N115" r:id="rId83" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-004_mobile-devices-table-horizontal-swipe-scroll.png" display="2026-10-27_Hari-16_TC-H16-004_mobile-devices-table-horizontal-swipe-scroll.png" xr:uid="{88EEBA14-BC1D-470E-AABF-A6B7AF0C8156}"/>
+    <hyperlink ref="N116" r:id="rId84" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png" display="2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png" xr:uid="{6F7FA9CB-B516-427C-9B63-C5E56C4A6FB4}"/>
+    <hyperlink ref="N117" r:id="rId85" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png" display="2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png" xr:uid="{1B98F40B-1904-4F52-A4A5-DD74EC5BEB74}"/>
+    <hyperlink ref="N118" r:id="rId86" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png" display="2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png" xr:uid="{A011486E-4D7D-43F0-8F79-F86D7CB87B28}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId80"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId87"/>
 </worksheet>
 </file>
 
@@ -10509,19 +10516,19 @@
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="58" t="s">
+      <c r="A13" s="60" t="s">
         <v>789</v>
       </c>
-      <c r="B13" s="58"/>
-      <c r="C13" s="58"/>
+      <c r="B13" s="60"/>
+      <c r="C13" s="60"/>
       <c r="M13" s="28"/>
     </row>
     <row r="14" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="58" t="s">
+      <c r="A14" s="60" t="s">
         <v>790</v>
       </c>
-      <c r="B14" s="58"/>
-      <c r="C14" s="58"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
       <c r="M14" s="28"/>
     </row>
     <row r="15" spans="1:14" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
docs(qa): polish 01_Master_Test_Cases.xlsx formatting, borders, row heights, and evidence hyperlinks
</commit_message>
<xml_diff>
--- a/docs/qa-testing/01_Master_Test_Cases.xlsx
+++ b/docs/qa-testing/01_Master_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F5C1CB-99C1-4D83-855E-67283285CF7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DBC4FD-2B6C-43C7-84E2-FBA890E14776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2242" uniqueCount="1155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2246" uniqueCount="1155">
   <si>
     <t>TC ID</t>
   </si>
@@ -3619,9 +3619,6 @@
     <t>Dashboard live t-aims.teknolab.biz.id aktif</t>
   </si>
   <si>
-    <t>1. Buka dashboard live. 2. Periksa kartu System Availability &amp; SLA Summary 30 Days. 3. Verifikasi rendering solid batang progress bar.</t>
-  </si>
-  <si>
     <t>Nilai persentase SLA 30 hari teragregasi presisi dan batang progress bar tampil penuh berwarna hijau/kuning/merah proporsional.</t>
   </si>
   <si>
@@ -3643,18 +3640,12 @@
     <t>Halaman #page-devices aktif pada domain live</t>
   </si>
   <si>
-    <t>1. Akses menu Inventaris Perangkat. 2. Hitung total baris tabel master inventaris. 3. Verifikasi 4 node baru (PC-03, CLOUD-01, RTR-04, CAS-01). 4. Buka dropdown filter kategori.</t>
-  </si>
-  <si>
     <t>Tabel memuat lengkap 19 perangkat aktif dan opsi Cloud Panel (Cloud VPS) tersedia pada filter kategori.</t>
   </si>
   <si>
     <t>Sesuai harapan. Total perangkat 19 unit valid, opsi Cloud Panel aktif ter-highlight.</t>
   </si>
   <si>
-    <t>2026-10-30_Hari-19_TC-H19-002_master-inventory-19-devices-cloudpanel.png; 2026-10-30_Hari-19_TC-H19-002b_dropdown-kategori-cloudpanel.png</t>
-  </si>
-  <si>
     <t>TC-H19-003</t>
   </si>
   <si>
@@ -3670,9 +3661,6 @@
     <t>Modal detail perangkat LAN privat aktif dan DevTools Network terbuka</t>
   </si>
   <si>
-    <t>1. Buka detail CCTV Head Office (192.168.1.5). 2. Klik tombol Uji Ping Sekarang. 3. Amati payload dan header request /api/monitoring/real-ping di tab Network.</t>
-  </si>
-  <si>
     <t>Aset LAN privat tidak false-offline dan request ping menggunakan autentikasi yang sah.</t>
   </si>
   <si>
@@ -3682,9 +3670,6 @@
     <t>BUG-H19-API-001</t>
   </si>
   <si>
-    <t>2026-10-30_Hari-19_TC-H19-003_real-ping-401-unauthorized-inspection.png; 2026-10-30_Hari-19_TC-H19-003b_real-ping-error-toast-offline.png</t>
-  </si>
-  <si>
     <t>TC-H19-004</t>
   </si>
   <si>
@@ -3700,9 +3685,6 @@
     <t>Halaman inventaris perangkat terbuka sebagai Reza Tri Wardana (Admin)</t>
   </si>
   <si>
-    <t>1. Klik tombol Ubah Status Alat pada modal CCTV Head Office. 2. Verifikasi modal Quick Status yang muncul.</t>
-  </si>
-  <si>
     <t>Modal pop-up Ubah Status Perangkat terbuka mulus menampilkan 3 opsi status operasional: ONLINE, PERINGATAN, dan OFFLINE.</t>
   </si>
   <si>
@@ -3710,6 +3692,35 @@
   </si>
   <si>
     <t>2026-10-30_Hari-19_TC-H19-004_quick-status-override-modal.png</t>
+  </si>
+  <si>
+    <t>1. Buka dashboard live.
+2. Periksa kartu System Availability &amp; SLA Summary 30 Days.
+3. Verifikasi rendering solid batang progress bar.</t>
+  </si>
+  <si>
+    <t>1. Akses menu Inventaris Perangkat.
+2. Hitung total baris tabel master inventaris (19 unit).
+3. Verifikasi 4 node baru (PC-03, CLOUD-01, RTR-04, CAS-01).
+4. Buka dropdown filter kategori (opsi Cloud Panel).</t>
+  </si>
+  <si>
+    <t>2026-10-30_Hari-19_TC-H19-002_master-inventory-19-devices-cloudpanel.png</t>
+  </si>
+  <si>
+    <t>1. Buka detail CCTV Head Office (192.168.1.5).
+2. Buka DevTools browser tab Network.
+3. Klik tombol Uji Ping Sekarang.
+4. Amati request payload &amp; header /api/monitoring/real-ping.</t>
+  </si>
+  <si>
+    <t>2026-10-30_Hari-19_TC-H19-003_real-ping-401-unauthorized-inspection.png</t>
+  </si>
+  <si>
+    <t>1. Buka modal detail perangkat CCTV Head Office.
+2. Klik tombol Ubah Status Alat.
+3. Verifikasi pop-up Quick Status Override.
+4. Uji pilihan status (Online, Peringatan, Offline).</t>
   </si>
 </sst>
 </file>
@@ -3897,7 +3908,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -3987,12 +3998,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4240,8 +4266,50 @@
     <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -10307,244 +10375,256 @@
       <c r="R117" s="41"/>
     </row>
     <row r="118" spans="1:18" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A118" s="34" t="s">
+      <c r="A118" s="85" t="s">
         <v>1096</v>
       </c>
-      <c r="B118" s="34">
+      <c r="B118" s="85">
         <v>16</v>
       </c>
-      <c r="C118" s="35" t="s">
+      <c r="C118" s="88" t="s">
         <v>1005</v>
       </c>
-      <c r="D118" s="35" t="s">
+      <c r="D118" s="88" t="s">
         <v>1097</v>
       </c>
-      <c r="E118" s="34" t="s">
+      <c r="E118" s="85" t="s">
         <v>728</v>
       </c>
-      <c r="F118" s="36" t="s">
+      <c r="F118" s="89" t="s">
         <v>272</v>
       </c>
-      <c r="G118" s="35" t="s">
+      <c r="G118" s="88" t="s">
         <v>1098</v>
       </c>
-      <c r="H118" s="35" t="s">
+      <c r="H118" s="88" t="s">
         <v>1099</v>
       </c>
-      <c r="I118" s="35" t="s">
+      <c r="I118" s="88" t="s">
         <v>1100</v>
       </c>
-      <c r="J118" s="35" t="s">
+      <c r="J118" s="88" t="s">
         <v>1101</v>
       </c>
-      <c r="K118" s="38" t="s">
+      <c r="K118" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="L118" s="34" t="s">
+      <c r="L118" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="M118" s="34" t="s">
+      <c r="M118" s="85" t="s">
         <v>277</v>
       </c>
-      <c r="N118" s="54" t="str">
+      <c r="N118" s="91" t="str">
         <f>HYPERLINK("evidence/screenshots/Hari-16/2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png", "2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png")</f>
         <v>2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png</v>
       </c>
-      <c r="O118" s="40" t="s">
-        <v>29</v>
-      </c>
-      <c r="P118" s="52">
+      <c r="O118" s="92" t="s">
+        <v>29</v>
+      </c>
+      <c r="P118" s="93">
         <v>46322</v>
       </c>
       <c r="Q118" s="34"/>
       <c r="R118" s="35"/>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
+    <row r="119" spans="1:18" ht="57" x14ac:dyDescent="0.25">
+      <c r="A119" s="86" t="s">
         <v>1119</v>
       </c>
-      <c r="B119">
+      <c r="B119" s="86">
         <v>19</v>
       </c>
-      <c r="C119" t="s">
+      <c r="C119" s="94" t="s">
         <v>1120</v>
       </c>
-      <c r="D119" t="s">
+      <c r="D119" s="94" t="s">
         <v>1121</v>
       </c>
-      <c r="E119" t="s">
+      <c r="E119" s="86" t="s">
         <v>1122</v>
       </c>
-      <c r="F119" t="s">
+      <c r="F119" s="95" t="s">
         <v>272</v>
       </c>
-      <c r="G119" t="s">
+      <c r="G119" s="94" t="s">
         <v>1123</v>
       </c>
-      <c r="H119" t="s">
+      <c r="H119" s="94" t="s">
+        <v>1149</v>
+      </c>
+      <c r="I119" s="94" t="s">
         <v>1124</v>
       </c>
-      <c r="I119" t="s">
+      <c r="J119" s="94" t="s">
         <v>1125</v>
       </c>
-      <c r="J119" t="s">
+      <c r="K119" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="L119" s="86" t="s">
+        <v>21</v>
+      </c>
+      <c r="M119" s="86" t="s">
+        <v>277</v>
+      </c>
+      <c r="N119" s="97" t="s">
         <v>1126</v>
       </c>
-      <c r="K119" t="s">
+      <c r="O119" s="98" t="s">
+        <v>29</v>
+      </c>
+      <c r="P119" s="99" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="120" spans="1:18" ht="99.75" x14ac:dyDescent="0.25">
+      <c r="A120" s="86" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B120" s="86">
+        <v>19</v>
+      </c>
+      <c r="C120" s="94" t="s">
+        <v>1128</v>
+      </c>
+      <c r="D120" s="94" t="s">
+        <v>1129</v>
+      </c>
+      <c r="E120" s="86" t="s">
+        <v>728</v>
+      </c>
+      <c r="F120" s="95" t="s">
+        <v>1091</v>
+      </c>
+      <c r="G120" s="94" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H120" s="94" t="s">
+        <v>1150</v>
+      </c>
+      <c r="I120" s="94" t="s">
+        <v>1131</v>
+      </c>
+      <c r="J120" s="94" t="s">
+        <v>1132</v>
+      </c>
+      <c r="K120" s="96" t="s">
         <v>27</v>
       </c>
-      <c r="L119" t="s">
+      <c r="L120" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="M119" t="s">
+      <c r="M120" s="86" t="s">
         <v>277</v>
       </c>
-      <c r="N119" t="s">
-        <v>1127</v>
-      </c>
-      <c r="O119" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>1128</v>
-      </c>
-      <c r="B120">
+      <c r="N120" s="97" t="s">
+        <v>1151</v>
+      </c>
+      <c r="O120" s="98" t="s">
+        <v>29</v>
+      </c>
+      <c r="P120" s="99" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="121" spans="1:18" ht="71.25" x14ac:dyDescent="0.25">
+      <c r="A121" s="86" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B121" s="86">
         <v>19</v>
       </c>
-      <c r="C120" t="s">
-        <v>1129</v>
-      </c>
-      <c r="D120" t="s">
-        <v>1130</v>
-      </c>
-      <c r="E120" t="s">
-        <v>728</v>
-      </c>
-      <c r="F120" t="s">
-        <v>1091</v>
-      </c>
-      <c r="G120" t="s">
-        <v>1131</v>
-      </c>
-      <c r="H120" t="s">
-        <v>1132</v>
-      </c>
-      <c r="I120" t="s">
-        <v>1133</v>
-      </c>
-      <c r="J120" t="s">
+      <c r="C121" s="94" t="s">
         <v>1134</v>
       </c>
-      <c r="K120" t="s">
+      <c r="D121" s="94" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E121" s="86" t="s">
+        <v>1136</v>
+      </c>
+      <c r="F121" s="95" t="s">
+        <v>272</v>
+      </c>
+      <c r="G121" s="94" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H121" s="94" t="s">
+        <v>1152</v>
+      </c>
+      <c r="I121" s="94" t="s">
+        <v>1138</v>
+      </c>
+      <c r="J121" s="94" t="s">
+        <v>1139</v>
+      </c>
+      <c r="K121" s="96" t="s">
         <v>27</v>
       </c>
-      <c r="L120" t="s">
+      <c r="L121" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="M120" t="s">
+      <c r="M121" s="86" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N121" s="97" t="s">
+        <v>1153</v>
+      </c>
+      <c r="O121" s="98" t="s">
+        <v>29</v>
+      </c>
+      <c r="P121" s="99" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="122" spans="1:18" ht="57" x14ac:dyDescent="0.25">
+      <c r="A122" s="86" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B122" s="86">
+        <v>19</v>
+      </c>
+      <c r="C122" s="94" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D122" s="94" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E122" s="86" t="s">
+        <v>1144</v>
+      </c>
+      <c r="F122" s="95" t="s">
+        <v>272</v>
+      </c>
+      <c r="G122" s="94" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H122" s="94" t="s">
+        <v>1154</v>
+      </c>
+      <c r="I122" s="94" t="s">
+        <v>1146</v>
+      </c>
+      <c r="J122" s="94" t="s">
+        <v>1147</v>
+      </c>
+      <c r="K122" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="L122" s="86" t="s">
+        <v>21</v>
+      </c>
+      <c r="M122" s="86" t="s">
         <v>277</v>
       </c>
-      <c r="N120" t="s">
-        <v>1135</v>
-      </c>
-      <c r="O120" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>1136</v>
-      </c>
-      <c r="B121">
-        <v>19</v>
-      </c>
-      <c r="C121" t="s">
-        <v>1137</v>
-      </c>
-      <c r="D121" t="s">
-        <v>1138</v>
-      </c>
-      <c r="E121" t="s">
-        <v>1139</v>
-      </c>
-      <c r="F121" t="s">
-        <v>272</v>
-      </c>
-      <c r="G121" t="s">
-        <v>1140</v>
-      </c>
-      <c r="H121" t="s">
-        <v>1141</v>
-      </c>
-      <c r="I121" t="s">
-        <v>1142</v>
-      </c>
-      <c r="J121" t="s">
-        <v>1143</v>
-      </c>
-      <c r="K121" t="s">
-        <v>27</v>
-      </c>
-      <c r="L121" t="s">
-        <v>21</v>
-      </c>
-      <c r="M121" t="s">
-        <v>1144</v>
-      </c>
-      <c r="N121" t="s">
-        <v>1145</v>
-      </c>
-      <c r="O121" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>1146</v>
-      </c>
-      <c r="B122">
-        <v>19</v>
-      </c>
-      <c r="C122" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D122" t="s">
+      <c r="N122" s="97" t="s">
         <v>1148</v>
       </c>
-      <c r="E122" t="s">
-        <v>1149</v>
-      </c>
-      <c r="F122" t="s">
-        <v>272</v>
-      </c>
-      <c r="G122" t="s">
-        <v>1150</v>
-      </c>
-      <c r="H122" t="s">
-        <v>1151</v>
-      </c>
-      <c r="I122" t="s">
-        <v>1152</v>
-      </c>
-      <c r="J122" t="s">
-        <v>1153</v>
-      </c>
-      <c r="K122" t="s">
-        <v>27</v>
-      </c>
-      <c r="L122" t="s">
-        <v>21</v>
-      </c>
-      <c r="M122" t="s">
-        <v>277</v>
-      </c>
-      <c r="N122" t="s">
-        <v>1154</v>
-      </c>
-      <c r="O122" t="s">
-        <v>29</v>
+      <c r="O122" s="98" t="s">
+        <v>29</v>
+      </c>
+      <c r="P122" s="99" t="s">
+        <v>961</v>
       </c>
     </row>
   </sheetData>
@@ -10635,9 +10715,13 @@
     <hyperlink ref="N116" r:id="rId84" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png" display="2026-10-27_Hari-16_TC-H16-005_mobile-devices-table-full-inventory-rendering.png" xr:uid="{6F7FA9CB-B516-427C-9B63-C5E56C4A6FB4}"/>
     <hyperlink ref="N117" r:id="rId85" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png" display="2026-10-27_Hari-16_TC-H16-006_backend-api-error-sanitization-404-zero-leakage.png" xr:uid="{1B98F40B-1904-4F52-A4A5-DD74EC5BEB74}"/>
     <hyperlink ref="N118" r:id="rId86" tooltip="Klik untuk membuka bukti screenshot 2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png" display="2026-10-27_Hari-16_TC-H16-007_device-keyword-search-cctv-filter-integrity.png" xr:uid="{A011486E-4D7D-43F0-8F79-F86D7CB87B28}"/>
+    <hyperlink ref="N119" r:id="rId87" xr:uid="{39BC971E-0395-4920-8E78-9C11583DB081}"/>
+    <hyperlink ref="N120" r:id="rId88" xr:uid="{1B429784-A44C-4768-B53C-6844A7707310}"/>
+    <hyperlink ref="N121" r:id="rId89" xr:uid="{82C20ED7-AFB2-4800-B9CE-C9F2900C7FEB}"/>
+    <hyperlink ref="N122" r:id="rId90" xr:uid="{9732E7AF-605F-418B-88EF-48820057E7DB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId87"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId91"/>
 </worksheet>
 </file>
 
@@ -10986,19 +11070,19 @@
       <c r="N12" s="14"/>
     </row>
     <row r="13" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="85" t="s">
+      <c r="A13" s="87" t="s">
         <v>789</v>
       </c>
-      <c r="B13" s="85"/>
-      <c r="C13" s="85"/>
+      <c r="B13" s="87"/>
+      <c r="C13" s="87"/>
       <c r="M13" s="14"/>
     </row>
     <row r="14" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="85" t="s">
+      <c r="A14" s="87" t="s">
         <v>790</v>
       </c>
-      <c r="B14" s="85"/>
-      <c r="C14" s="85"/>
+      <c r="B14" s="87"/>
+      <c r="C14" s="87"/>
       <c r="M14" s="14"/>
     </row>
     <row r="15" spans="1:14" ht="15" x14ac:dyDescent="0.25">

</xml_diff>